<commit_message>
Detail view: Prev / Next stepper through the filtered results
While a Source detail sub-tab is open, a button group next to "Back to
results" steps to the previous / next source in the current filtered
result order, with an "n / total" position indicator (disabled at the
ends). Wired per panel in server_risk_panel.R via <prefix>_prev /
<prefix>_next; render_detail_ui() now takes (src, prefix, siblings).

Also picks up the latest data revision: 21st source
(copernicus_climate_indicators - ready-made CDS hazard indices),
Climate-ADAPT reassessed (Supplementary / grid / has API), EFFIS url,
plus refreshed hazard_coverage / references.bib / abstracts. No app
change needed for those - all data-driven. The "Limitations" left_join
in app.R stays 1:1 (one Limitations row per source, verified).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6tTWnYUJ1DiozJbfUjD1w
</commit_message>
<xml_diff>
--- a/data/ESG_Data_Source_Matrix_Structured.xlsx
+++ b/data/ESG_Data_Source_Matrix_Structured.xlsx
@@ -168,8 +168,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="HazardCoverage" displayName="HazardCoverage" ref="A4:D220" headerRowCount="1">
-  <autoFilter ref="A4:D220"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="HazardCoverage" displayName="HazardCoverage" ref="A4:D232" headerRowCount="1">
+  <autoFilter ref="A4:D232"/>
   <tableColumns count="4">
     <tableColumn id="1" name="source_id"/>
     <tableColumn id="2" name="hazard_id"/>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -619,7 +619,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Context only</t>
+          <t>Supplementary</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -629,32 +629,32 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>EU macro-region (3 regions)</t>
+          <t>Grid / raster</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partly</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>technical</t>
+          <t>granularity</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -823,12 +823,12 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>drmkc.jrc.ec.europa.eu/risk-data-hub#/atlas/metadata/wildfire_effis</t>
+          <t>forest-fire.emergency.copernicus.eu</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -2221,6 +2221,88 @@
         </is>
       </c>
       <c r="P24" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Copernicus Ready-Made Climate Indicators (ERA5-HEAT, SMHI Hydrology, CEMS Fire Danger)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Standalone, ready-made hazard indices on the CDS: heat stress (UTCI), hydrology (flood/aridity/soil moisture), fire danger</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ECMWF / SMHI / JRC, on behalf of the EU (via C3S/CEMS)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Grid / raster</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>cds.climate.copernicus.eu/datasets/derived-utci-historical</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2241,7 +2323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D220"/>
+  <dimension ref="A1:D232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2304,7 +2386,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>EU-wide report table resolves only to three macro-regions (Northern/Central/Southern Europe, per IPCC AR6 reference regions) - Austria falls entirely within "Central Europe" with no further within-country differentiation at that level. The underlying interactive European Climate Data Explorer (fed by Copernicus C3S data) allows finer sub-regional zoom for 15 of the 32 underlying indices, but which specific indices support this was not verified per hazard. Indirect proxy indicator only, not a dedicated named hazard category in the EEA index set.</t>
+          <t>Only an indirect proxy (Universal Thermal Climate Index, UTCI) at 0.25 degree grid - no dedicated heat-stress index exists.</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2421,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>full</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>EU-wide report table resolves only to three macro-regions (Northern/Central/Southern Europe, per IPCC AR6 reference regions) - Austria falls entirely within "Central Europe" with no further within-country differentiation at that level. The underlying interactive European Climate Data Explorer (fed by Copernicus C3S data) allows finer sub-regional zoom for 15 of the 32 underlying indices, but which specific indices support this was not verified per hazard.</t>
+          <t>Dedicated "extreme heat" indices (Hot Days, Tropical Nights, Warmest 3-day Period, Climatological/Apparent Temperature Heatwave Days) at 0.25 degree grid (~28km), directly downloadable via the ECDE indicator dataset.</t>
         </is>
       </c>
     </row>
@@ -2361,12 +2443,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>full</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>EU-wide report table resolves only to three macro-regions (Northern/Central/Southern Europe, per IPCC AR6 reference regions) - Austria falls entirely within "Central Europe" with no further within-country differentiation at that level. The underlying interactive European Climate Data Explorer (fed by Copernicus C3S data) allows finer sub-regional zoom for 15 of the 32 underlying indices, but which specific indices support this was not verified per hazard.</t>
+          <t>Dedicated Fire Weather Index and High Fire Danger Days indices at 0.1 degree grid (~11km), based on the same EFFIS classification, directly downloadable via the ECDE indicator dataset.</t>
         </is>
       </c>
     </row>
@@ -2383,12 +2465,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>full</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>EU-wide report table resolves only to three macro-regions (Northern/Central/Southern Europe, per IPCC AR6 reference regions) - Austria falls entirely within "Central Europe" with no further within-country differentiation at that level. The underlying interactive European Climate Data Explorer (fed by Copernicus C3S data) allows finer sub-regional zoom for 15 of the 32 underlying indices, but which specific indices support this was not verified per hazard.</t>
+          <t>Dedicated "severe windstorm" index (Extreme Wind Speed Days) at 0.25 degree grid (~28km), directly downloadable via the ECDE indicator dataset.</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2492,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>EU-wide report table resolves only to three macro-regions (Northern/Central/Southern Europe, per IPCC AR6 reference regions) - Austria falls entirely within "Central Europe" with no further within-country differentiation at that level. The underlying interactive European Climate Data Explorer (fed by Copernicus C3S data) allows finer sub-regional zoom for 15 of the 32 underlying indices, but which specific indices support this was not verified per hazard. Indirect proxy indicator only, not a dedicated named hazard category in the EEA index set.</t>
+          <t>Only an indirect proxy (Aridity Actual index) at 5km grid - no dedicated water-stress index exists.</t>
         </is>
       </c>
     </row>
@@ -2427,12 +2509,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>full</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>EU-wide report table resolves only to three macro-regions (Northern/Central/Southern Europe, per IPCC AR6 reference regions) - Austria falls entirely within "Central Europe" with no further within-country differentiation at that level. The underlying interactive European Climate Data Explorer (fed by Copernicus C3S data) allows finer sub-regional zoom for 15 of the 32 underlying indices, but which specific indices support this was not verified per hazard.</t>
+          <t>Dedicated river-flood indices (Flood Recurrence, River Discharge) at 5km grid, directly downloadable via the ECDE indicator dataset.</t>
         </is>
       </c>
     </row>
@@ -2449,12 +2531,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>full</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>EU-wide report table resolves only to three macro-regions (Northern/Central/Southern Europe, per IPCC AR6 reference regions) - Austria falls entirely within "Central Europe" with no further within-country differentiation at that level. The underlying interactive European Climate Data Explorer (fed by Copernicus C3S data) allows finer sub-regional zoom for 15 of the 32 underlying indices, but which specific indices support this was not verified per hazard.</t>
+          <t>Dedicated "extreme precipitation" indices (Maximum Consecutive 5-Day Precipitation, Extreme Precipitation Total/Days) at 0.25 degree grid (~28km), directly downloadable via the ECDE indicator dataset.</t>
         </is>
       </c>
     </row>
@@ -2471,12 +2553,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>full</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>EU-wide report table resolves only to three macro-regions (Northern/Central/Southern Europe, per IPCC AR6 reference regions) - Austria falls entirely within "Central Europe" with no further within-country differentiation at that level. The underlying interactive European Climate Data Explorer (fed by Copernicus C3S data) allows finer sub-regional zoom for 15 of the 32 underlying indices, but which specific indices support this was not verified per hazard.</t>
+          <t>Dedicated meteorological drought indices (SPI-3 Duration/Magnitude) at 0.25 degree grid, plus a soil-moisture drought index at 5km grid, directly downloadable via the ECDE indicator dataset.</t>
         </is>
       </c>
     </row>
@@ -3027,12 +3109,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Only an indirect proxy (Universal Thermal Climate Index, UTCI) available via the shared sis-ecde-climate-indicators dataset - the same proxy limitation noted for Climate-ADAPT, since both draw on the same underlying EEA/C3S index set.</t>
+          <t>UTCI is a complex multi-variable derived index (temperature, humidity, wind, radiation); no ready-made version exists among the raw CDS variables - see copernicus_climate_indicators for the standalone ERA5-HEAT product.</t>
         </is>
       </c>
     </row>
@@ -3071,12 +3153,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Dedicated "extreme heat" indices (tropical nights, hot days, heatwave days) available via the shared sis-ecde-climate-indicators dataset, directly downloadable.</t>
+          <t>Dedicated "extreme heat" indices (tropical nights, hot days, heatwave days) exist as part of the sis-ecde-climate-indicators dataset on the CDS, but are not a prominently findable feature of Copernicus CDS as a general-purpose entry point - practically accessed via Climate-ADAPT rather than by browsing CDS directly.</t>
         </is>
       </c>
     </row>
@@ -3093,12 +3175,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Dedicated "Fire danger indices historical data" dataset (CEMS/EFFIS-based, ERA5-driven, three national fire-danger rating systems) directly downloadable from the CDS - a purpose-built, ready-made dataset, not merely a derivable raw variable.</t>
+          <t>Fire Weather Index requires a specific multi-variable fire-danger model, not derivable from raw meteorological variables alone - see copernicus_climate_indicators for the standalone CEMS Fire Danger product.</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3202,7 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Derived "severe wind storm" index available via the shared sis-ecde-climate-indicators dataset, plus raw 10m wind-speed ERA5 variables. Not a hazard-zoned map.</t>
+          <t>Derived "severe wind storm" index exists as part of the sis-ecde-climate-indicators dataset on the CDS, but is not a prominently findable feature of Copernicus CDS as a general-purpose entry point - practically accessed via Climate-ADAPT rather than by browsing CDS directly. Raw 10m wind-speed ERA5 variables remain available for custom modelling.</t>
         </is>
       </c>
     </row>
@@ -3137,12 +3219,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>No dedicated water-stress index; only indirectly covered via aridity/soil-moisture proxies, same limitation as Climate-ADAPT.</t>
+          <t>Aridity requires evapotranspiration modelling, not derivable from raw meteorological variables alone - see copernicus_climate_indicators for the standalone SMHI hydrology product.</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3241,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Derived "river flood index using runoff" available via the shared sis-ecde-climate-indicators dataset (same index set as Climate-ADAPT), plus raw runoff/precipitation ERA5 variables for custom modelling. Not a hazard-zoned map.</t>
+          <t>River discharge/flood recurrence requires hydrological modelling, not derivable from raw meteorological variables alone - see copernicus_climate_indicators for the standalone SMHI hydrology product.</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3268,7 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Derived heavy-precipitation indices available via the shared sis-ecde-climate-indicators dataset, plus raw precipitation ERA5 variables. Not a hazard-zoned map.</t>
+          <t>Derived heavy-precipitation indices exist as part of the sis-ecde-climate-indicators dataset on the CDS, but are not a prominently findable feature of Copernicus CDS as a general-purpose entry point - practically accessed via Climate-ADAPT rather than by browsing CDS directly. Raw precipitation ERA5 variables remain available for custom modelling.</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3290,7 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Derived drought indices (meteorological and soil-moisture based) available via the shared sis-ecde-climate-indicators dataset, plus raw soil-moisture ERA5 variables. Not a hazard-zoned map.</t>
+          <t>Meteorological drought (SPI-3) is derivable from raw precipitation variables with moderate own processing; the soil-moisture drought component requires hydrological modelling - see copernicus_climate_indicators for the standalone SMHI hydrology product covering that component directly.</t>
         </is>
       </c>
     </row>
@@ -6605,6 +6687,242 @@
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>flood</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="inlineStr">
+        <is>
+          <t>Standalone "Hydrology-related climate impact indicators" dataset (sis-hydrology-variables-derived-projections), produced by SMHI for C3S, 18 water quantity/quality Climate Impact Indicators including Flood Recurrence and River Discharge, directly selectable, 5km grid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>landslide</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>soil_erosion</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D223" s="4" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>glacial_lake</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D224" s="4" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>storm</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D225" s="4" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>heavy_precip</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D226" s="4" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>heat_wave</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D227" s="4" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>heat_stress</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="D228" s="4" t="inlineStr">
+        <is>
+          <t>Standalone "ERA5-HEAT" dataset (derived-utci-historical), peer-reviewed (Di Napoli et al., 2021), hourly UTCI/mean radiant temperature grids at 0.25 degree resolution (~28km), 1940-present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>drought</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="D229" s="4" t="inlineStr">
+        <is>
+          <t>Soil-moisture drought (Mean Soil Moisture) directly selectable within the standalone SMHI hydrology dataset, 5km grid. (Meteorological/SPI-3 drought remains raw-variable-only; see copernicus_cds.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>water_stress</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="D230" s="4" t="inlineStr">
+        <is>
+          <t>Aridity Actual directly selectable within the standalone SMHI hydrology dataset (sis-hydrology-variables-derived-projections), 5km grid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>wildfire</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="D231" s="4" t="inlineStr">
+        <is>
+          <t>Standalone "Fire danger indices historical data" dataset (CEMS/EFFIS-based, ERA5-driven, three national fire-danger rating systems), directly downloadable, ~28km (ERA5-driven) grid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>permafrost</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D232" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6624,7 +6942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7401,6 +7719,33 @@
       <c r="E31" t="inlineStr">
         <is>
           <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>D 01.01</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>K_41.01.a-b</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0050</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Primary</t>
         </is>
       </c>
     </row>
@@ -7419,7 +7764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C167"/>
+  <dimension ref="A1:C168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7471,7 +7816,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Rated Low because there is no data behind the portal to process at all - the "effort" is simply browsing a website, not because the source is easy to make portfolio-ready (see key_limitation).</t>
+          <t>Rated Medium (revised from Low, since the source does have real data behind it): the ECDE indicator dataset (sis-ecde-climate-indicators on the CDS) provides pre-computed, peer-reviewed indices - e.g. "Hot Days" count, SPI-3 drought index, Fire Weather Index - so, unlike Copernicus CDS, no own index/threshold definition is needed. Still requires geocoding and grid extraction, hence Medium rather than Low.</t>
         </is>
       </c>
     </row>
@@ -7488,7 +7833,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Good as entry point/screening level, too coarse for populating data points.</t>
+          <t>Advantage over using Copernicus CDS directly: ECDE provides ready-made, peer-reviewed climate hazard indices with documented methodology and academic citations (e.g. Spinoni et al. 2018/2020, Jacob et al. 2013), rather than raw climate variables the bank would need to convert into its own index definitions. Both draw on similar underlying grid resolutions (0.1-0.25 degree, or 5km for hydrology-based indices), so the advantage is in processing effort saved, not in finer raw resolution. Weaker than Copernicus CDS in hazard breadth (permafrost, landslide, soil erosion are not covered at all) and in flexibility (limited to the 32 pre-selected indices).</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7935,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Since 2 July 2025 uniformly CC-BY 4.0; individual sub-datasets may carry stricter licences (e.g. E-OBS: non-commercial research/education only) - verify per dataset.</t>
+          <t>Individual sub-datasets may carry stricter terms than the general CC-BY 4.0 - e.g. E-OBS is restricted to non-commercial research/education use only; verify per dataset before use.</t>
         </is>
       </c>
     </row>
@@ -7750,34 +8095,34 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Licensing notes</t>
+          <t>Suitability assessment</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Free for individual queries; separate agreement with operator (LFRZ) required for portfolio-level use.</t>
+          <t>Good supplementary dataset for chronic risk (water stress), since AT sources primarily cover acute hazards.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Suitability assessment</t>
+          <t>technical_effort rationale</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Good supplementary dataset for chronic risk (water stress), since AT sources primarily cover acute hazards.</t>
+          <t>Ready-made risk scores per location, directly integrable via API.</t>
         </is>
       </c>
     </row>
@@ -7789,29 +8134,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>technical_effort rationale</t>
+          <t>Suitability assessment</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Ready-made risk scores per location, directly integrable via API.</t>
+          <t>High data quality and granularity; cost structure typically not designed for SNCI scale.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Suitability assessment</t>
+          <t>technical_effort rationale</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>High data quality and granularity; cost structure typically not designed for SNCI scale.</t>
+          <t>Ready-made scores/maps via web tool or API.</t>
         </is>
       </c>
     </row>
@@ -7823,19 +8168,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>technical_effort rationale</t>
+          <t>Suitability assessment</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Ready-made scores/maps via web tool or API.</t>
+          <t>Very extensive (scenarios to 2100); commercial, geared towards larger institutions/reinsurers.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7845,14 +8190,14 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Very extensive (scenarios to 2100); commercial, geared towards larger institutions/reinsurers.</t>
+          <t>Country-level granularity too coarse for exposure/NUTS assignment; useful for plausibility checks only.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7862,24 +8207,24 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Country-level granularity too coarse for exposure/NUTS assignment; useful for plausibility checks only.</t>
+          <t>Best available current Austrian permafrost source for context/discussion; not suitable for exposure-level classification.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Suitability assessment</t>
+          <t>technical_effort rationale</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Best available current Austrian permafrost source for context/discussion; not suitable for exposure-level classification.</t>
+          <t>Single CSV file (326,479 records) keyed to the Firmenbuch number; joins directly to a loan portfolio without GIS or geocoding work. Codes are 5-digit OeNACE; the 4-digit NACE level required by D 01.01 is obtained by dropping the last digit.</t>
         </is>
       </c>
     </row>
@@ -7891,12 +8236,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>technical_effort rationale</t>
+          <t>Suitability assessment</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Single CSV file (326,479 records) keyed to the Firmenbuch number; joins directly to a loan portfolio without GIS or geocoding work. Codes are 5-digit OeNACE; the 4-digit NACE level required by D 01.01 is obtained by dropping the last digit.</t>
+          <t>The strongest transition-risk source identified: official assignment under section 21 Bundesstatistikgesetz, published as a High Value Dataset under CC BY 4.0, covering all actively registered Austrian companies with an assigned economic activity. Resolves the previous trade-off in which official quality and open access were mutually exclusive.</t>
         </is>
       </c>
     </row>
@@ -7908,12 +8253,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Suitability assessment</t>
+          <t>Licensing notes</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>The strongest transition-risk source identified: official assignment under section 21 Bundesstatistikgesetz, published as a High Value Dataset under CC BY 4.0, covering all actively registered Austrian companies with an assigned economic activity. Resolves the previous trade-off in which official quality and open access were mutually exclusive.</t>
+          <t>CC BY 4.0, published under Implementing Regulation (EU) 2023/138 (High Value Datasets); free of charge, bulk download, updated continuously.</t>
         </is>
       </c>
     </row>
@@ -7925,29 +8270,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Licensing notes</t>
+          <t>Data quality notes</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>CC BY 4.0, published under Implementing Regulation (EU) 2023/138 (High Value Datasets); free of charge, bulk download, updated continuously.</t>
+          <t>Verified as OeNACE 2025 / NACE Rev. 2.1 by structural analysis of the 682 distinct codes: division 45 absent (abolished in Rev. 2.1), classes 47.41/47.42/47.43 absent (merged into 47.40), class 46.89 present (newly created in Rev. 2.1), and divisions 62 and 63 following the Rev. 2.1 structure. Template D 01.01 uses the same revision, as evidenced by its designation K.63 for computing infrastructure, which is only valid under Rev. 2.1. No transcoding between classification versions is therefore required.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Data quality notes</t>
+          <t>technical_effort rationale</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Verified as OeNACE 2025 / NACE Rev. 2.1 by structural analysis of the 682 distinct codes: division 45 absent (abolished in Rev. 2.1), classes 47.41/47.42/47.43 absent (merged into 47.40), class 46.89 present (newly created in Rev. 2.1), and divisions 62 and 63 following the Rev. 2.1 structure. Template D 01.01 uses the same revision, as evidenced by its designation K.63 for computing infrastructure, which is only valid under Rev. 2.1. No transcoding between classification versions is therefore required.</t>
+          <t>Ready-made OeNACE 2025 classification per entity, delivered via API; no manual extract handling required.</t>
         </is>
       </c>
     </row>
@@ -7959,53 +8304,53 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>technical_effort rationale</t>
+          <t>Suitability assessment</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Ready-made OeNACE 2025 classification per entity, delivered via API; no manual extract handling required.</t>
+          <t>Retained alongside the HVD dataset because access already exists institutionally in parts of the Austrian banking sector (for example across the Raiffeisen sector), making the marginal cost zero and an existing query operationally simpler than downloading and joining the HVD file. Adds daily currency and coverage beyond the Firmenbuch.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Suitability assessment</t>
+          <t>technical_effort rationale</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Retained alongside the HVD dataset because access already exists institutionally in parts of the Austrian banking sector (for example across the Raiffeisen sector), making the marginal cost zero and an existing query operationally simpler than downloading and joining the HVD file. Adds daily currency and coverage beyond the Firmenbuch.</t>
+          <t>technical_effort reflects the effort to access and use the source's own data (dashboard-only, no download/API, same interface as EBA ESG Dashboard, hence Low). The separate, substantially higher effort of replicating the ECB's methodology with AnaCredit/JRC/Copernicus-equivalent inputs is a distinct undertaking and is described in the abstract, not folded into this column.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>eea_climate_adapt</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>technical_effort rationale</t>
+          <t>Portfolio-ready pipeline</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>technical_effort reflects the effort to access and use the source's own data (dashboard-only, no download/API, same interface as EBA ESG Dashboard, hence Low). The separate, substantially higher effort of replicating the ECB's methodology with AnaCredit/JRC/Copernicus-equivalent inputs is a distinct undertaking and is described in the abstract, not folded into this column.</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Query or download the relevant pre-computed ECDE indicator (sis-ecde-climate-indicators dataset on the CDS) for the coordinate. (3) Assign the returned value to the exposure. Automatable, but resolution varies by indicator (5km to ~28km), so multiple exposures within the same grid cell share a value.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>eea_climate_adapt</t>
+          <t>jrc_risk_data_hub</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8015,14 +8360,14 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Not applicable - see key_limitation.</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Identify the NUTS2/3 region for each coordinate. (3) Download/query the relevant hazard module(s) via API or shapefile. (4) Join exposures to their region's value. Regional (not parcel-level) result.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub</t>
+          <t>effis_wildfire</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -8032,14 +8377,14 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>(1) Geocode exposure addresses to coordinates. (2) Identify the NUTS2/3 region for each coordinate. (3) Download/query the relevant hazard module(s) via API or shapefile. (4) Join exposures to their region's value. Regional (not parcel-level) result.</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Query the WMS/WFS or download the GeoTIFF fire danger index / burnt-area layer. (3) Extract the raster cell value at each coordinate (point-in-raster lookup). (4) Decide how to handle the time-varying daily index (e.g. seasonal maximum or long-run average) to arrive at a single static attribute per exposure.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>effis_wildfire</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8049,14 +8394,14 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>(1) Geocode exposure addresses to coordinates. (2) Query the WMS/WFS or download the GeoTIFF fire danger index / burnt-area layer. (3) Extract the raster cell value at each coordinate (point-in-raster lookup). (4) Decide how to handle the time-varying daily index (e.g. seasonal maximum or long-run average) to arrive at a single static attribute per exposure.</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Select and download the relevant climate variable(s) in NetCDF/GRIB. (3) Derive a hazard-relevant indicator from the raw climate variable (this is a climatological modelling step, not a simple lookup). (4) Extract the grid-cell value at each coordinate.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8066,14 +8411,14 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>(1) Geocode exposure addresses to coordinates. (2) Select and download the relevant climate variable(s) in NetCDF/GRIB. (3) Derive a hazard-relevant indicator from the raw climate variable (this is a climatological modelling step, not a simple lookup). (4) Extract the grid-cell value at each coordinate.</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Query the WFS endpoint (nz-core:HazardArea) with each coordinate, or download the GML/shapefile once and perform a local spatial join. (3) Assign the returned zone/extent value to the exposure. Fully automatable, parcel-level result.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8083,14 +8428,14 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Not applicable - see key_limitation.</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Query the WMS/WFS endpoint or download the shapefile/GeoPackage once and perform a local spatial join. (3) Assign the returned zone value to the exposure. Fully automatable, parcel-level result within mapped municipalities.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8100,14 +8445,14 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Not applicable via this source directly (see key_limitation). A per-exposure pipeline would instead need to replicate the ECB's published methodology using the bank's own AnaCredit-equivalent data plus JRC/Copernicus hazard layers.</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Download the watershed-level dataset (CSV/GeoPackage) or query the API. (3) Perform a spatial join to the relevant watershed polygon. (4) Assign the watershed's indicator value to the exposure. Automatable, but resolution is watershed- not parcel-level.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8117,14 +8462,14 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>(1) Geocode exposure addresses to coordinates. (2) Query the WFS endpoint (nz-core:HazardArea) with each coordinate, or download the GML/shapefile once and perform a local spatial join. (3) Assign the returned zone/extent value to the exposure. Fully automatable, parcel-level result.</t>
+          <t>Send exposure coordinates/address to the API; receive a facility-level score directly. No further spatial processing required.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8134,14 +8479,14 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>(1) Geocode exposure addresses to coordinates. (2) Query the WMS/WFS endpoint or download the shapefile/GeoPackage once and perform a local spatial join. (3) Assign the returned zone value to the exposure. Fully automatable, parcel-level result within mapped municipalities.</t>
+          <t>Send exposure coordinates/address to the API; receive a facility-level score directly. No further spatial processing required.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8151,14 +8496,14 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Not applicable at scale - see key_limitation. Practical use is limited to spot-checking individual exposures.</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Determine the ADM2 (district) administrative unit for each coordinate. (3) Query the ThinkHazard! API for the hazard level of that district (or download the relevant Risk Data Library dataset for gridded hazards such as landslide and perform a spatial join). (4) Assign the returned district-level value to the exposure. Automatable, but resolution is district- not parcel-level.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8168,14 +8513,14 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>(1) Geocode exposure addresses to coordinates. (2) Download the watershed-level dataset (CSV/GeoPackage) or query the API. (3) Perform a spatial join to the relevant watershed polygon. (4) Assign the watershed's indicator value to the exposure. Automatable, but resolution is watershed- not parcel-level.</t>
+          <t>Bulk-download the CSV and join directly on Firmenbuchnummer against the loan portfolio. No geocoding or spatial processing needed.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8185,99 +8530,99 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Send exposure coordinates/address to the API; receive a facility-level score directly. No further spatial processing required.</t>
+          <t>Send the Firmenbuchnummer or company identifier to the API; receive the OeNACE classification directly. No further processing required.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>eea_climate_adapt</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Portfolio-ready pipeline</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Send exposure coordinates/address to the API; receive a facility-level score directly. No further spatial processing required.</t>
+          <t>Climate-ADAPT is a public knowledge portal operated by the European Environment Agency (EEA) (EEA, n.d.-a). It hosts the European Climate Data Explorer (ECDE), which provides 32 pre-computed, peer-reviewed climate hazard indices covering 16 hazard categories, grouped into six IPCC AR6 climatic-impact-driver types (heat and cold, wet and dry, wind, snow and ice, coastal, open ocean); the indicator dataset itself is published on the Copernicus Climate Data Store as a distinct, downloadable/queryable dataset (EEA/C3S, n.d.). Not all of the matrix's physical hazards are represented: permafrost, landslide and soil erosion have no corresponding index in this set, while heat stress and water stress are only indirectly covered via proxy indices (Universal Thermal Climate Index; aridity) (EEA, 2021). Grid resolution varies by indicator, from 5km (hydrology-based indices such as river flood and aridity) to roughly 0.1-0.25 degrees (~11-28km) for most temperature, precipitation, wind and fire-weather indices (EEA/C3S, n.d.). The source is accessed through an interactive web portal, a queryable API and direct download of the underlying indicator dataset, and is free to use. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>jrc_risk_data_hub</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Portfolio-ready pipeline</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>(1) Geocode exposure addresses to coordinates. (2) Determine the ADM2 (district) administrative unit for each coordinate. (3) Query the ThinkHazard! API for the hazard level of that district (or download the relevant Risk Data Library dataset for gridded hazards such as landslide and perform a spatial join). (4) Assign the returned district-level value to the exposure. Automatable, but resolution is district- not parcel-level.</t>
+          <t>The Risk Data Hub (RDH) is a public multi-hazard risk and loss data platform operated by the Joint Research Centre (JRC) in cooperation with the EU Disaster Risk Management Knowledge Centre (DRMKC) (JRC DRMKC, n.d.). It provides modelled exposure, hazard and historical-event data covering multiple physical hazards at regional (NUTS 2/3) granularity across EU, EFTA and IPA countries (JRC DRMKC, n.d.). The source is accessed through a web map portal, direct download and an API, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source and secondary to the Geography dimension (0090–0130).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>effis_wildfire</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Portfolio-ready pipeline</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Not applicable - see key_limitation.</t>
+          <t>EFFIS is a public wildfire information service operated jointly by the JRC and Copernicus Emergency Management Service (JRC/Copernicus EMS, n.d.). It provides daily fire danger indices and historical burnt-area data covering wildfire risk at grid/raster granularity across Europe and the MENA region (JRC/Copernicus EMS, n.d.). The source is accessed through an OGC map service and direct download, and is free of charge under a CC-BY 4.0 licence requiring attribution only. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Portfolio-ready pipeline</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Bulk-download the CSV and join directly on Firmenbuchnummer against the loan portfolio. No geocoding or spatial processing needed.</t>
+          <t>The CDS is a public climate data repository operated by ECMWF on behalf of the EU (ECMWF, n.d.), comprising over 140 datasets of raw and derived climate variables and reanalysis/projection data. This entry covers the general-purpose raw variables (e.g. ERA5 temperature, precipitation, wind fields); the standalone, ready-made hazard indicator products hosted on the same CDS (ERA5-HEAT for heat stress, the SMHI hydrology dataset for flood/water stress/soil-moisture drought, CEMS Fire Danger for wildfire) are documented separately under copernicus_climate_indicators, since they differ materially in processing effort and portfolio-readiness. The source is accessed through a web portal, direct download and an API, and is free of charge, uniformly licensed under CC-BY 4.0 since July 2025 (individual sub-datasets may carry stricter terms). In the context of Template D 01.01, it is relevant to data point 0050 as a primary source and secondary to the Geography dimension.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>eba_esg_dashboard</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Portfolio-ready pipeline</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Send the Firmenbuchnummer or company identifier to the API; receive the OeNACE classification directly. No further processing required.</t>
+          <t>The EBA ESG Dashboard is a public statistics dashboard operated by the European Banking Authority (EBA) (EBA, n.d.-a). It provides aggregated ESG risk indicators at EU bank level, covering both physical and transition risk dimensions at institution/portfolio-level granularity rather than individual exposure level (EBA, n.d.-a). The source is accessed through a web-based statistics dashboard and is free to use. In the context of Template D 01.01, it is relevant only as a benchmarking reference, not to any specific data point.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>eea_climate_adapt</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8287,14 +8632,14 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Climate-ADAPT is a public knowledge portal operated by the European Environment Agency (EEA) (EEA, n.d.-a). It links to a set of 32 climate hazard indices covering 16 hazard categories, grouped into six IPCC AR6 climatic-impact-driver types (heat and cold, wet and dry, wind, snow and ice, coastal, open ocean) (EEA, 2021). Not all of the matrix's physical hazards are represented: permafrost, landslide and soil erosion have no corresponding index in this set, while heat stress and water stress are only indirectly covered via proxy indices (Universal Thermal Climate Index; aridity) (EEA, 2021). Where covered, the source's own report table resolves only to three European macro-regions (Northern/Central/Southern Europe), placing all of Austria in a single "Central Europe" category with no within-country differentiation at that level, though the underlying interactive European Climate Data Explorer allows finer sub-regional zoom for a subset of the indices (EEA, 2021). The source is accessed through an interactive web map portal and is free to use. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source. For an SNCI, the source is conditionally suitable because it offers a useful entry point for screening and context, although its coarse, non-spatial resolution makes it unsuitable on its own for classifying individual exposures. In portfolio-readiness terms, the source is not ready: no downloadable or queryable data exists behind the portal, so no automated pipeline can be built against it.</t>
+          <t>This is a public methodological and statistical resource operated by the European Central Bank (ECB) (ECB, n.d.). It provides a documented methodology and euro-area statistics on physical risk exposure, covering physical hazards at institution/portfolio-level granularity (NUTS3-based underlying methodology) (ECB, n.d.). The source is accessed through a statistics dashboard and is free to use, though the underlying data (AnaCredit/RIAD) are not accessible to an SNCI. In the context of Template D 01.01, it is relevant to data points 0050 and 0090–0130 as a secondary source.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8304,14 +8649,14 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>The Risk Data Hub (RDH) is a public multi-hazard risk and loss data platform operated by the Joint Research Centre (JRC) in cooperation with the EU Disaster Risk Management Knowledge Centre (DRMKC) (JRC DRMKC, n.d.). It provides modelled exposure, hazard and historical-event data covering multiple physical hazards at regional (NUTS 2/3) granularity across EU, EFTA and IPA countries (JRC DRMKC, n.d.). The source is accessed through a web map portal, direct download and an API, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source and secondary to the Geography dimension (0090–0130). For an SNCI, the source is suitable because it combines primary relevance with EU-wide consistent methodology, although its Vulnerability and Risk Analysis modules remain documented by JRC as ongoing work, and finer layers require geocoding and spatial overlay. In portfolio-readiness terms, the source is only partly ready: once geocoded and joined to its NUTS2/3 modules, it differentiates between regions but not between individual exposures within the same region.</t>
+          <t>This is a national flood extent dataset, published via the INSPIRE Geoportal Oesterreich, with the Bundesministerium fuer Land- und Forstwirtschaft, Klima- und Umweltschutz, Regionen und Wasserwirtschaft (BMLUK) as data owner and Umweltbundesamt GmbH as the technical operator (INSPIRE Geoportal Oesterreich, n.d.-b). It combines Abflussuntersuchungen (ABU), HORA data and, in part, the BWV and WLV hazard zoning plans into a single set of flood extent layers for the 30-, 100- and 300-year return periods, covering flood risk at parcel/address-level granularity across Austria (INSPIRE Geoportal Oesterreich, n.d.-b). The source is accessed through OGC WMS/WFS services and direct GML/shapefile download via the INSPIRE Atom download service, and is free of charge under a CC BY 4.0 licence. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>effis_wildfire</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8321,14 +8666,14 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>EFFIS is a public wildfire information service operated jointly by the JRC and Copernicus Emergency Management Service (JRC/Copernicus EMS, n.d.). It provides daily fire danger indices and historical burnt-area data covering wildfire risk at grid/raster granularity across Europe and the MENA region (JRC/Copernicus EMS, n.d.). The source is accessed through an OGC map service and direct download, and is free of charge under a CC-BY 4.0 licence requiring attribution only. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source. For an SNCI, the source is conditionally suitable because it is the only dedicated wildfire dataset identified, although the raw hazard-index and event data require own geocoding and GIS overlay before they can support exposure-level classification. In portfolio-readiness terms, the source is only partly ready: once geocoded and queried against its ~1km fire-danger raster, it differentiates across the country but not within a single town or parcel.</t>
+          <t>The GZP is a public national hazard zoning dataset operated by the Forsttechnischer Dienst fuer Wildbach- und Lawinenverbauung (Federal Ministry BMLUK) (data.gv.at, n.d.-b). It provides a statutory hazard assessment under the Forstgesetz covering torrent, avalanche, landslide and erosion processes at parcel/address-level granularity across Austria (INSPIRE Geoportal Oesterreich, n.d.-a). The source is accessed through an OGC map service and direct download in shapefile/GeoPackage format, and is free of charge as a High Value Dataset under Implementing Regulation (EU) 2023/138 (INSPIRE Geoportal Oesterreich, n.d.-a). In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8338,14 +8683,14 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>The CDS is a public climate data repository operated by ECMWF on behalf of the EU (ECMWF, n.d.). It provides climate variables and derived hazard-relevant reference datasets covering multiple physical hazards at grid/raster granularity globally with an EU focus (ECMWF, n.d.). The source is accessed through a web portal, direct download and an API, and is free of charge, uniformly licensed under CC-BY 4.0 since July 2025 (individual sub-datasets may carry stricter terms). In the context of Template D 01.01, it is relevant to data point 0050 as a primary source and secondary to the Geography dimension. For an SNCI, the source is conditionally suitable because it is authoritative and EU-wide consistent, although the raw NetCDF/GRIB climate variables require climatological and GIS processing before they translate into an exposure classification. In portfolio-readiness terms, the source is not ready for typical Austrian portfolios: its roughly 0.1-0.25 degree grid means most exposures within a regionally concentrated portfolio would share an identical value.</t>
+          <t>HORA (Natural Hazard Overview and Risk Assessment Austria) is a publicly accessible Austrian WebGIS application, operated by the Land-, Forst- und Wasserwirtschaftliche Rechenzentrum (LFRZ) on behalf of the responsible federal ministry (LFRZ, n.d.). It provides address- and cadastral-level initial information on natural hazards, currently covering flood, earthquake, storm, hail and snow (HORA, n.d.), with further hazards such as landslide added over time through cooperation with GeoSphere Austria (BMLUK, n.d.). The source is accessed through an interactive web interface via individual location queries, and is free to use. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8355,14 +8700,14 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>The EBA ESG Dashboard is a public statistics dashboard operated by the European Banking Authority (EBA) (EBA, n.d.-a). It provides aggregated ESG risk indicators at EU bank level, covering both physical and transition risk dimensions at institution/portfolio-level granularity rather than individual exposure level (EBA, n.d.-a). The source is accessed through a web-based statistics dashboard and is free to use. In the context of Template D 01.01, it is relevant only as a benchmarking reference, not to any specific data point. For an SNCI, the source is not suitable for populating individual exposures, although it remains useful for peer-comparison and contextual benchmarking of the institution's own ESG risk profile. This is a technical limitation rather than a granularity one: the output is aggregate bank-level statistics, with no per-exposure data to draw on at all.</t>
+          <t>The Aqueduct Water Risk Atlas is a public water-risk dataset operated by the World Resources Institute (WRI) (WRI, n.d.). It provides 13 modelled indicators covering water stress, drought risk and both riverine and coastal flood risk at sub-catchment (watershed) granularity globally (WRI, n.d.-b). The source is accessed through a web map portal, direct download and an API, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8372,14 +8717,14 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>This is a public methodological and statistical resource operated by the European Central Bank (ECB) (ECB, n.d.). It provides a documented methodology and euro-area statistics on physical risk exposure, covering physical hazards at institution/portfolio-level granularity (NUTS3-based underlying methodology) (ECB, n.d.). The source is accessed through a statistics dashboard and is free to use, though the underlying data (AnaCredit/RIAD) are not accessible to an SNCI. In the context of Template D 01.01, it is relevant to data points 0050 and 0090–0130 as a secondary source. For an SNCI, the source is conditionally suitable because its documented methodology can be replicated using AnaCredit/JRC/Copernicus-equivalent inputs, although the ECB's own underlying supervisory data are unavailable to a non-significant institution. In portfolio-readiness terms, the source itself is not ready: its output is aggregate/dashboard statistics with no per-exposure data, so any per-exposure use means replicating the methodology with the bank's own data rather than drawing on the ECB source directly.</t>
+          <t>This is a commercial dataset operated by Moody's ESG Solutions (Moody's, n.d.). The underlying methodology originates from Four Twenty Seven, Inc., a physical-climate-risk data firm founded in 2012, in which Moody's Corporation acquired a majority stake in July 2019 as a Moody's Investors Service affiliate (Moody's, 2019); the acquisition was reported in Moody's own 2019 Form 10-Q as operating within the MIS reportable segment (Moody's, 2019b). It provides proprietary modelled physical climate risk scores covering six hazards (floods, heat stress, hurricanes and typhoons, sea-level rise, water stress, wildfires) at facility/object-level granularity globally (Moody's, n.d.-b); note that the storm hazard is modelled as tropical cyclones specifically, which has limited relevance to Austria. The source is accessed through a commercial analytics platform and an API, and is paid, subject to a commercial licence agreement. In the context of Template D 01.01, it is relevant to data points 0050 and 0090–0130 as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -8389,14 +8734,14 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>This is a national flood extent dataset, published via the INSPIRE Geoportal Oesterreich, with the Bundesministerium fuer Land- und Forstwirtschaft, Klima- und Umweltschutz, Regionen und Wasserwirtschaft (BMLUK) as data owner and Umweltbundesamt GmbH as the technical operator (INSPIRE Geoportal Oesterreich, n.d.-b). It combines Abflussuntersuchungen (ABU), HORA data and, in part, the BWV and WLV hazard zoning plans into a single set of flood extent layers for the 30-, 100- and 300-year return periods, covering flood risk at parcel/address-level granularity across Austria (INSPIRE Geoportal Oesterreich, n.d.-b). The source is accessed through OGC WMS/WFS services and direct GML/shapefile download via the INSPIRE Atom download service, and is free of charge under a CC BY 4.0 licence. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source. For an SNCI, the source is suitable because it combines several of the other Austrian hazard sources into ready-made flood extent layers with a standard OGC interface, without HORA's bulk-access restriction. In portfolio-readiness terms, the source is ready: once geocoded, a WFS query or a local spatial join against the downloaded layer assigns a differentiating, parcel-level value to each exposure without further manual adjustment.</t>
+          <t>NATHAN Risk Suite is a commercial dataset operated by Munich Re (Munich Re, n.d.). It provides proprietary modelled natural hazard and climate scenario scores covering multiple hazards at facility/object-level granularity globally, including scenarios extending to 2100 (Munich Re, n.d.). Two access models exist: a subscription-based portfolio platform (Business/Corporate tiers, with API access, quote-based pricing) and a subscription-free, pay-per-location "On-Demand" service priced from EUR 100-160 per location depending on package size (Munich Re, n.d.-c). In the context of Template D 01.01, it is relevant to data points 0050 and 0090–0130 as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -8406,14 +8751,14 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>The GZP is a public national hazard zoning dataset operated by the Forsttechnischer Dienst fuer Wildbach- und Lawinenverbauung (Federal Ministry BMLUK) (data.gv.at, n.d.-b). It provides a statutory hazard assessment under the Forstgesetz covering torrent, avalanche, landslide and erosion processes at parcel/address-level granularity across Austria (INSPIRE Geoportal Oesterreich, n.d.-a). The source is accessed through an OGC map service and direct download in shapefile/GeoPackage format, and is free of charge as a High Value Dataset under Implementing Regulation (EU) 2023/138 (INSPIRE Geoportal Oesterreich, n.d.-a). In the context of Template D 01.01, it is relevant to data point 0050 as a primary source. For an SNCI, the source is suitable because it is the strongest national source for mass-movement and torrent hazards, complementing rather than duplicating the BWV flood data, although hazard zones are mapped only within settled areas of relevance, so an unmatched portfolio location may indicate either no hazard or simply no mapping. In portfolio-readiness terms, the source is ready on the same basis as the BWV flood layers: geocoding plus a WMS/WFS query or local spatial join yields a differentiating, parcel-level value per exposure within mapped municipalities.</t>
+          <t>This is a public dataset collection operated by the World Bank Group in cooperation with GFDRR (World Bank/GFDRR, n.d.), comprising both the historical-event Risk Data Library and the forward-looking, probabilistic ThinkHazard! hazard tool (GFDRR, n.d.). It provides climate and disaster risk data covering multiple hazards, with ThinkHazard! resolving to district (ADM2) level via a public API and the Risk Data Library varying by dataset (GFDRR, n.d.-b), and a development-country focus overall (World Bank/GFDRR, n.d.). The source is accessed through a generic web portal, direct download and an API, and is free of charge. In the context of Template D 01.01, it is relevant only as a context/validation reference, not to a specific data point.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -8423,14 +8768,14 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>HORA (Natural Hazard Overview and Risk Assessment Austria) is a publicly accessible Austrian WebGIS application, operated by the Land-, Forst- und Wasserwirtschaftliche Rechenzentrum (LFRZ) on behalf of the responsible federal ministry (LFRZ, n.d.). It provides address- and cadastral-level initial information on natural hazards, currently covering flood, earthquake, storm, hail and snow (HORA, n.d.), with further hazards such as landslide added over time through cooperation with GeoSphere Austria (BMLUK, n.d.). Access is provided through an interactive web interface and individual location queries; however, portfolio-level use is constrained by restrictions on bulk access to the underlying data. The source is therefore relevant to D 01.01 data point 0050, but not sufficient on its own to support systematic portfolio classification. Within the ESG Data Source Matrix, HORA is classified as a conditionally suitable source for individual validation and exposure-level plausibility checks. This is a technical, not a granularity, limitation: the underlying zoning is parcel-level and would be portfolio-ready if bulk access were available.</t>
+          <t>KryoMon.AT is a publicly funded research consortium coordinated by the University of Graz, involving multiple Austrian universities, the Austrian and Bavarian Academies of Sciences, GeoSphere Austria and several associations (KryoMon.AT, n.d.; ORF Steiermark, 2026). It provides periodic reports on permafrost, glacier and snow trends covering permafrost hazard at station-based granularity across selected Austrian alpine sites (KryoMon.AT, n.d.). The source is accessed through a reports/publications website and PDF downloads, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8440,14 +8785,14 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>The Aqueduct Water Risk Atlas is a public water-risk dataset operated by the World Resources Institute (WRI) (WRI, n.d.). It provides 13 modelled indicators covering water stress, drought risk and both riverine and coastal flood risk at sub-catchment (watershed) granularity globally (WRI, n.d.-b). The source is accessed through a web map portal, direct download and an API, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source. For an SNCI, the source is conditionally suitable because it fills a gap in the domestic data landscape for chronic water-related hazards, although its global watershed-level granularity is coarser than the parcel-level Austrian sources for the acute hazards it also covers. In portfolio-readiness terms, the source is only partly ready: once geocoded and spatially joined to its watershed polygons, it differentiates between regions but not within a single watershed.</t>
+          <t>This is a public register operated by Statistik Austria (Statistik Austria, n.d.). It provides the official OeNACE 2025 (NACE Rev. 2.1) economic-activity code for each Austrian company, keyed to the Firmenbuch number, covering the full national company register at entity-level granularity (Statistik Austria, n.d.). The source is accessed through direct bulk download in CSV format and is free of charge under a CC BY 4.0 licence, published as a High Value Dataset under Implementing Regulation (EU) 2023/138. In the context of Template D 01.01, it is relevant to the NACE subsector dimension as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -8457,99 +8802,99 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>This is a commercial dataset operated by Moody's ESG Solutions (Moody's, n.d.). The underlying methodology originates from Four Twenty Seven, Inc., a physical-climate-risk data firm founded in 2012, in which Moody's Corporation acquired a majority stake in July 2019 as a Moody's Investors Service affiliate (Moody's, 2019); the acquisition was reported in Moody's own 2019 Form 10-Q as operating within the MIS reportable segment (Moody's, 2019b). It provides proprietary modelled physical climate risk scores covering six hazards (floods, heat stress, hurricanes and typhoons, sea-level rise, water stress, wildfires) at facility/object-level granularity globally (Moody's, n.d.-b); note that the storm hazard is modelled as tropical cyclones specifically, which has limited relevance to Austria. The source is accessed through a commercial analytics platform and an API, and is paid, subject to a commercial licence agreement. In the context of Template D 01.01, it is relevant to data points 0050 and 0090–0130 as a primary source. For an SNCI, the source is conditionally suitable because it offers ready-made, high-granularity risk scores integrable via API with low processing effort, although its cost structure is typically designed for larger institutions rather than an SNCI's scale. In portfolio-readiness terms, the source is fully ready: the API returns a differentiating, facility-level score directly, with no further spatial processing required.</t>
+          <t>Wirtschafts-Compass is a commercial Austrian company-data service operated by Compass-Verlag GmbH (Compass-Verlag, n.d.). It provides an editorially enriched OeNACE classification per entity, covering the Austrian company landscape at entity-level granularity, delivered with daily currency (Compass-Verlag, n.d.). The source is accessed through an API and a web portal, and is paid, though the operator states that the finance and insurance sector is among its long-standing customers, meaning many Austrian banking-sector institutions may already hold an institutional licence (Compass-Verlag, n.d.-b). In the context of Template D 01.01, it is relevant to the NACE subsector dimension as a secondary source.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>eea_climate_adapt</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Hazard coverage correction note</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>NATHAN Risk Suite is a commercial dataset operated by Munich Re (Munich Re, n.d.). It provides proprietary modelled natural hazard and climate scenario scores covering multiple hazards at facility/object-level granularity globally, including scenarios extending to 2100 (Munich Re, n.d.). Two access models exist: a subscription-based portfolio platform (Business/Corporate tiers, with API access, quote-based pricing) and a subscription-free, pay-per-location "On-Demand" service priced from EUR 100-160 per location depending on package size (Munich Re, n.d.-c). In the context of Template D 01.01, it is relevant to data points 0050 and 0090–0130 as a primary source. For an SNCI, the source is suitable because of its very extensive scenario depth and ready-made scores; unlike the quote-based subscription tiers geared towards larger institutions and reinsurers, the pay-per-location On-Demand option makes single-location or small-scale spot-checks accessible without a full portfolio subscription, though it is not designed for bulk portfolio processing. In portfolio-readiness terms, the subscription/API tier is fully ready: it returns a differentiating, facility-level score directly, with no further spatial processing required.</t>
+          <t>Coverage was originally set uniformly to "partial" across 10 of 12 matrix hazards with identical granularity text, without per-hazard verification. Verified against the EEA's own 32-index / 16-hazard / 6-category index set (EEA, 2021): permafrost, landslide and soil erosion are not represented at all and were corrected to "none"; heat_stress and water_stress are only indirect proxies (UTCI; aridity), not dedicated categories; and the true resolution of the source's own report table is three European macro-regions, not NUTS 1/2 as previously stated.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>jrc_risk_data_hub</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Hazard coverage correction note</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>This is a public dataset collection operated by the World Bank Group in cooperation with GFDRR (World Bank/GFDRR, n.d.), comprising both the historical-event Risk Data Library and the forward-looking, probabilistic ThinkHazard! hazard tool (GFDRR, n.d.). It provides climate and disaster risk data covering multiple hazards, with ThinkHazard! resolving to district (ADM2) level via a public API and the Risk Data Library varying by dataset (GFDRR, n.d.-b), and a development-country focus overall (World Bank/GFDRR, n.d.). The source is accessed through a generic web portal, direct download and an API, and is free of charge. In the context of Template D 01.01, it is relevant only as a context/validation reference, not to a specific data point. For an SNCI, the source is conditionally suitable as a supplementary plausibility check because its district-level granularity is coarser than the parcel-level Austrian sources for acute hazards, though it still differentiates within Austria. In portfolio-readiness terms, the source is only partly ready: once queried via the ThinkHazard! API, it differentiates between Austrian districts but not within a single district.</t>
+          <t>Originally soil_erosion=full, glacial_lake=partial, heat_stress=partial, water_stress=partial with uniform reasoning. Verified against the JRC's own 2023 technical report (JRC136527, Table 5 "List of hazards addressed currently on the RDH"): only River flood, Coastal flood, Earthquake, Landslide, Forest fire and Subsidence have a modelled Risk Analysis layer. "Subsidence" is a physically distinct process from soil erosion, so soil_erosion corrected to none. glacial_lake, heat_stress and water_stress do not appear in either the Risk Analysis or Loss Data catalogues and were corrected to none. storm, heavy_precip, heat_wave and drought remain partial but are now documented as historical loss-record coverage only (Loss Data module), not modelled hazard layers.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Hazard coverage correction note</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>KryoMon.AT is a publicly funded research consortium coordinated by the University of Graz, involving multiple Austrian universities, the Austrian and Bavarian Academies of Sciences, GeoSphere Austria and several associations (KryoMon.AT, n.d.; ORF Steiermark, 2026). It provides periodic reports on permafrost, glacier and snow trends covering permafrost hazard at station-based granularity across selected Austrian alpine sites (KryoMon.AT, n.d.). The source is accessed through a reports/publications website and PDF downloads, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source. For an SNCI, the source is conditionally suitable as the best available current context on Austrian permafrost trends, although its station-based reporting cannot be overlaid with individual portfolio locations and is therefore unsuitable for exposure-level classification. In portfolio-readiness terms, the source is not ready: the information exists only in narrative PDF reports, not as structured per-location data, so no automated pipeline can be built.</t>
+          <t>Originally heat_stress=full and wildfire=partial. Verified: CDS hosts the same shared EEA/C3S 32-index dataset as Climate-ADAPT (sis-ecde-climate-indicators), so heat_stress is only the same UTCI proxy noted for Climate-ADAPT and was corrected to partial for consistency. wildfire was corrected to full after confirming a dedicated, purpose-built "Fire danger indices historical data" dataset (CEMS/EFFIS, ERA5-driven, three national fire-danger rating systems) is directly downloadable from the CDS, not merely derivable from raw variables.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Hazard coverage correction note</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>This is a public register operated by Statistik Austria (Statistik Austria, n.d.). It provides the official OeNACE 2025 (NACE Rev. 2.1) economic-activity code for each Austrian company, keyed to the Firmenbuch number, covering the full national company register at entity-level granularity (Statistik Austria, n.d.). The source is accessed through direct bulk download in CSV format and is free of charge under a CC BY 4.0 licence, published as a High Value Dataset under Implementing Regulation (EU) 2023/138. In the context of Template D 01.01, it is relevant to the NACE subsector dimension as a primary source. For an SNCI, the source is suitable because it is the only identified source that is simultaneously official, freely accessible in bulk and directly joinable to a loan portfolio via the Firmenbuch number, although companies without an assigned OeNACE code, and unregistered sole traders, remain unmatched. In portfolio-readiness terms, the source is fully ready: a direct join on the Firmenbuchnummer assigns the OeNACE code to each exposure with no geocoding or spatial processing needed.</t>
+          <t>Originally landslide=none, heavy_precip=none, drought=partial, wildfire=partial, heat_stress=full. Verified against the ECB's own indicator methodology page, which explicitly lists: "coastal flooding, river flooding, wildfires, landslides, subsidence, windstorms, water stress, droughts and rainfall variation." landslide was missing entirely and corrected to full; drought and wildfire were under-rated and corrected to full; heavy_precip (rainfall variation) corrected from none to partial. heat_stress corrected from full to partial: not named among the ECB's own 9 listed hazards, despite other ECB communications describing "heat and water stress" as a chronic risk category - flagged as a documentation inconsistency pending clarification.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Hazard coverage correction note</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Wirtschafts-Compass is a commercial Austrian company-data service operated by Compass-Verlag GmbH (Compass-Verlag, n.d.). It provides an editorially enriched OeNACE classification per entity, covering the Austrian company landscape at entity-level granularity, delivered with daily currency (Compass-Verlag, n.d.). The source is accessed through an API and a web portal, and is paid, though the operator states that the finance and insurance sector is among its long-standing customers, meaning many Austrian banking-sector institutions may already hold an institutional licence (Compass-Verlag, n.d.-b). In the context of Template D 01.01, it is relevant to the NACE subsector dimension as a secondary source. For an SNCI, the source is conditionally suitable because it complements the HVD dataset operationally where an existing licence makes a single query simpler than a bulk join, although its classification is editorially enriched rather than the official statistical assignment. In portfolio-readiness terms, the source is fully ready on the same basis as HVD: the API returns a differentiating classification directly for each queried entity.</t>
+          <t>Originally flood, landslide, storm, heat_wave, drought, water_stress and wildfire were all uniformly partial, and soil_erosion was partial. Verified against GFDRR's ThinkHazard! methodology documentation and the World Bank/GFDRR Global Landslide Hazard Map: flood, heat_wave (extreme heat), water_stress (water scarcity, via a dedicated Water Stress Index) and wildfire have commonly-available probabilistic hazard data and were corrected to full; landslide is covered via a dedicated gridded global dataset and corrected to full. soil_erosion, heat_stress and heavy_precip do not appear as distinct categories anywhere in the ThinkHazard!/Risk Data Library ecosystem and were corrected to none. storm remains partial because ThinkHazard!'s "cyclone" hazard model is tropical-cyclone-oriented and its applicability to European extratropical windstorms was not confirmed. drought remains partial as it is only indirectly inferable from the water-scarcity index, not a distinct event-based drought product.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>eea_climate_adapt</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -8559,14 +8904,14 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Coverage was originally set uniformly to "partial" across 10 of 12 matrix hazards with identical granularity text, without per-hazard verification. Verified against the EEA's own 32-index / 16-hazard / 6-category index set (EEA, 2021): permafrost, landslide and soil erosion are not represented at all and were corrected to "none"; heat_stress and water_stress are only indirect proxies (UTCI; aridity), not dedicated categories; and the true resolution of the source's own report table is three European macro-regions, not NUTS 1/2 as previously stated.</t>
+          <t>Originally flood and drought were rated partial. Verified against WRI's own 13-indicator Aqueduct 4.0 framework: dedicated "riverine flood risk" (rfr), "coastal flood risk" (cfr) and "drought risk" (drr) indicators exist by name, not merely inferred from water-stress data, and were corrected to full.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -8576,14 +8921,14 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Originally soil_erosion=full, glacial_lake=partial, heat_stress=partial, water_stress=partial with uniform reasoning. Verified against the JRC's own 2023 technical report (JRC136527, Table 5 "List of hazards addressed currently on the RDH"): only River flood, Coastal flood, Earthquake, Landslide, Forest fire and Subsidence have a modelled Risk Analysis layer. "Subsidence" is a physically distinct process from soil erosion, so soil_erosion corrected to none. glacial_lake, heat_stress and water_stress do not appear in either the Risk Analysis or Loss Data catalogues and were corrected to none. storm, heavy_precip, heat_wave and drought remain partial but are now documented as historical loss-record coverage only (Loss Data module), not modelled hazard layers.</t>
+          <t>Originally storm=full, heat_wave=full, drought=full, wildfire=partial. Verified against Moody's own consistently published hazard list (floods, heat stress, hurricanes and typhoons, sea-level rise, water stress, wildfires): storm was corrected to none because Moody's names "hurricanes and typhoons" specifically - a tropical-cyclone hazard not applicable to landlocked Austria; heat_wave corrected to none because only "heat stress" (a distinct, chronic indicator) is named, not a separate acute heat-wave product; drought corrected to none as it does not appear in any published Moody's hazard list found; wildfire corrected to full as it is consistently and explicitly named.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -8593,184 +8938,184 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Originally heat_stress=full and wildfire=partial. Verified: CDS hosts the same shared EEA/C3S 32-index dataset as Climate-ADAPT (sis-ecde-climate-indicators), so heat_stress is only the same UTCI proxy noted for Climate-ADAPT and was corrected to partial for consistency. wildfire was corrected to full after confirming a dedicated, purpose-built "Fire danger indices historical data" dataset (CEMS/EFFIS, ERA5-driven, three national fire-danger rating systems) is directly downloadable from the CDS, not merely derivable from raw variables.</t>
+          <t>Originally soil_erosion=partial, glacial_lake=partial, landslide=partial, heavy_precip/heat_wave/heat_stress/drought/water_stress=full, wildfire=partial. Verified against Munich Re's own 15-hazard "Natural Hazards Edition" list (River Flood, Flash Flood, Storm Surge, Tropical Cyclone, Extratropical Storm, Hail, Tornado, Lightning, Earthquake, Volcano, Tsunami, Wildfire, Avalanche, Landslide, Subsidence): landslide and wildfire corrected to full (explicitly named); soil_erosion and glacial_lake corrected to none (not covered, or - for soil_erosion - only the physically distinct "Subsidence" is covered). heavy_precip, heat_wave, heat_stress, drought and water_stress were downgraded from full to partial: these are not named in the Natural Hazards Edition, and the separate "Climate Change Edition" advertises "13 climate hazards" without naming them individually in the materials reviewed, so full coverage could not be confirmed.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Hazard coverage correction note</t>
+          <t>Pricing details</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Originally landslide=none, heavy_precip=none, drought=partial, wildfire=partial, heat_stress=full. Verified against the ECB's own indicator methodology page, which explicitly lists: "coastal flooding, river flooding, wildfires, landslides, subsidence, windstorms, water stress, droughts and rainfall variation." landslide was missing entirely and corrected to full; drought and wildfire were under-rated and corrected to full; heavy_precip (rainfall variation) corrected from none to partial. heat_stress corrected from full to partial: not named among the ECB's own 9 listed hazards, despite other ECB communications describing "heat and water stress" as a chronic risk category - flagged as a documentation inconsistency pending clarification.</t>
+          <t>Specific pricing for Moody's physical risk/Climate on Demand data is not publicly disclosed; access is quote-based via direct sales contact. Public aggregate spend estimates exist for Moody's software generally (third-party benchmarking, not company-published), but these cover unrelated products (e.g. EDF-X, Orbis) and are not specific to the physical risk data product, so they are not usable as a cost estimate here.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Hazard coverage correction note</t>
+          <t>Pricing details</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Originally flood, landslide, storm, heat_wave, drought, water_stress and wildfire were all uniformly partial, and soil_erosion was partial. Verified against GFDRR's ThinkHazard! methodology documentation and the World Bank/GFDRR Global Landslide Hazard Map: flood, heat_wave (extreme heat), water_stress (water scarcity, via a dedicated Water Stress Index) and wildfire have commonly-available probabilistic hazard data and were corrected to full; landslide is covered via a dedicated gridded global dataset and corrected to full. soil_erosion, heat_stress and heavy_precip do not appear as distinct categories anywhere in the ThinkHazard!/Risk Data Library ecosystem and were corrected to none. storm remains partial because ThinkHazard!'s "cyclone" hazard model is tropical-cyclone-oriented and its applicability to European extratropical windstorms was not confirmed. drought remains partial as it is only indirectly inferable from the water-scarcity index, not a distinct event-based drought product.</t>
+          <t>Two distinct access models exist. (1) Location Risk Intelligence On-Demand: a subscription-free, pay-per-location service for single-location lookups (not full portfolios), priced in tiered packages from EUR 160 per location (5-location package, EUR 800 net) down to EUR 100 per location (50-location package, EUR 5,000 net; 48 credits per location lookup), prices exclude VAT (Munich Re, n.d.-c). (2) The portfolio-scale Natural Hazards Edition / Climate Change Edition subscription (Business/Corporate tiers, with API access) remains quote-based and not publicly priced.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Hazard coverage correction note</t>
+          <t>Pricing details</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Originally flood and drought were rated partial. Verified against WRI's own 13-indicator Aqueduct 4.0 framework: dedicated "riverine flood risk" (rfr), "coastal flood risk" (cfr) and "drought risk" (drr) indicators exist by name, not merely inferred from water-stress data, and were corrected to full.</t>
+          <t>Pay-per-query pricing: from EUR 6 (excl. VAT) per quarter for up to 10 queries via the WKO-member Wirtschafts-Compass service (Compass-Verlag's own price list) (Compass-Verlag, n.d.-c); individual/basic access starts from EUR 24 per year per the operator's own website (Compass-Verlag, n.d.-d). Official Firmenbuch extract fees (per the Justizministerium's Gebührenverordnung) are billed separately and are not part of the Wirtschafts-Compass subscription cost itself.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Hazard coverage correction note</t>
+          <t>Licensing notes</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Originally storm=full, heat_wave=full, drought=full, wildfire=partial. Verified against Moody's own consistently published hazard list (floods, heat stress, hurricanes and typhoons, sea-level rise, water stress, wildfires): storm was corrected to none because Moody's names "hurricanes and typhoons" specifically - a tropical-cyclone hazard not applicable to landlocked Austria; heat_wave corrected to none because only "heat stress" (a distinct, chronic indicator) is named, not a separate acute heat-wave product; drought corrected to none as it does not appear in any published Moody's hazard list found; wildfire corrected to full as it is consistently and explicitly named.</t>
+          <t>Most GeoSphere Austria Data Hub datasets are published under Creative Commons Public Domain Dedication (CC0 1.0), free for any use including commercial, per the operator's own repository documentation (GeoSphere Austria/re3data, n.d.); the exact licence tag should be confirmed per-dataset on the dataset landing page before productive use.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Hazard coverage correction note</t>
+          <t>Licensing notes</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Originally soil_erosion=partial, glacial_lake=partial, landslide=partial, heavy_precip/heat_wave/heat_stress/drought/water_stress=full, wildfire=partial. Verified against Munich Re's own 15-hazard "Natural Hazards Edition" list (River Flood, Flash Flood, Storm Surge, Tropical Cyclone, Extratropical Storm, Hail, Tornado, Lightning, Earthquake, Volcano, Tsunami, Wildfire, Avalanche, Landslide, Subsidence): landslide and wildfire corrected to full (explicitly named); soil_erosion and glacial_lake corrected to none (not covered, or - for soil_erosion - only the physically distinct "Subsidence" is covered). heavy_precip, heat_wave, heat_stress, drought and water_stress were downgraded from full to partial: these are not named in the Natural Hazards Edition, and the separate "Climate Change Edition" advertises "13 climate hazards" without naming them individually in the materials reviewed, so full coverage could not be confirmed.</t>
+          <t>Most GeoSphere Austria Data Hub datasets are published under Creative Commons Public Domain Dedication (CC0 1.0), free for any use including commercial, per the operator's own repository documentation (GeoSphere Austria/re3data, n.d.); the exact licence tag should be confirmed per-dataset on the dataset landing page before productive use.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Pricing details</t>
+          <t>Portfolio-ready pipeline</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Specific pricing for Moody's physical risk/Climate on Demand data is not publicly disclosed; access is quote-based via direct sales contact. Public aggregate spend estimates exist for Moody's software generally (third-party benchmarking, not company-published), but these cover unrelated products (e.g. EDF-X, Orbis) and are not specific to the physical risk data product, so they are not usable as a cost estimate here.</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Query the GeoSphere Austria grid API with the coordinates for the relevant SPARTACUS variable(s) (temperature, precipitation). (3) Apply a chosen threshold/index definition (e.g. a heat-wave or heavy-precipitation definition) to the returned time series. (4) Assign the resulting value to the exposure. Fully automatable, 1km grid resolution.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Pricing details</t>
+          <t>Portfolio-ready pipeline</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Two distinct access models exist. (1) Location Risk Intelligence On-Demand: a subscription-free, pay-per-location service for single-location lookups (not full portfolios), priced in tiered packages from EUR 160 per location (5-location package, EUR 800 net) down to EUR 100 per location (50-location package, EUR 5,000 net; 48 credits per location lookup), prices exclude VAT (Munich Re, n.d.-c). (2) The portfolio-scale Natural Hazards Edition / Climate Change Edition subscription (Business/Corporate tiers, with API access) remains quote-based and not publicly priced.</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Query the GeoSphere Austria grid API with the coordinates for the WINFORE SPEI variable at the desired aggregation window (30/90/365 days). (3) Assign the returned SPEI value to the exposure. Fully automatable, 1km grid resolution.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Pricing details</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Pay-per-query pricing: from EUR 6 (excl. VAT) per quarter for up to 10 queries via the WKO-member Wirtschafts-Compass service (Compass-Verlag's own price list) (Compass-Verlag, n.d.-c); individual/basic access starts from EUR 24 per year per the operator's own website (Compass-Verlag, n.d.-d). Official Firmenbuch extract fees (per the Justizministerium's Gebührenverordnung) are billed separately and are not part of the Wirtschafts-Compass subscription cost itself.</t>
+          <t>SPARTACUS-v3 is a public gridded climate dataset operated by GeoSphere Austria, the Austrian federal institute for geology, geophysics, climatology and meteorology (GeoSphere Austria, n.d.-a). It provides observed daily, monthly and quarterly temperature, precipitation and sunshine-duration fields at 1km resolution across Austria since 1961, updated daily (GeoSphere Austria, n.d.-a). The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge, published under the CC0 1.0 Public Domain Dedication used for most GeoSphere Austria Data Hub datasets (GeoSphere Austria/re3data, n.d.). In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Licensing notes</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Most GeoSphere Austria Data Hub datasets are published under Creative Commons Public Domain Dedication (CC0 1.0), free for any use including commercial, per the operator's own repository documentation (GeoSphere Austria/re3data, n.d.); the exact licence tag should be confirmed per-dataset on the dataset landing page before productive use.</t>
+          <t>WINFORE is a public gridded drought-index dataset operated by GeoSphere Austria (GeoSphere Austria, n.d.-b). It provides the Standardized Precipitation Evapotranspiration Index (SPEI) at 30-, 90- and 365-day aggregation windows, plus potential evapotranspiration, derived from SPARTACUS temperature and precipitation fields at 1km resolution across Austria, updated daily (GeoSphere Austria, n.d.-b). The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge, published under the CC0 1.0 Public Domain Dedication used for most GeoSphere Austria Data Hub datasets (GeoSphere Austria/re3data, n.d.). In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Licensing notes</t>
+          <t>Pricing details</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Most GeoSphere Austria Data Hub datasets are published under Creative Commons Public Domain Dedication (CC0 1.0), free for any use including commercial, per the operator's own repository documentation (GeoSphere Austria/re3data, n.d.); the exact licence tag should be confirmed per-dataset on the dataset landing page before productive use.</t>
+          <t>Not publicly disclosed by Climate X directly. Third-party industry comparison sources estimate EUR 20,000-60,000 per year for portfolios of 30-100 assets, described as "mid-market" pricing relative to enterprise platforms like Jupiter Intelligence or Moody's; this figure is a third-party estimate, not confirmed by the operator (Repath, n.d.).</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -8780,48 +9125,48 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>(1) Geocode exposure addresses to coordinates. (2) Query the GeoSphere Austria grid API with the coordinates for the relevant SPARTACUS variable(s) (temperature, precipitation). (3) Apply a chosen threshold/index definition (e.g. a heat-wave or heavy-precipitation definition) to the returned time series. (4) Assign the resulting value to the exposure. Fully automatable, 1km grid resolution.</t>
+          <t>Send exposure coordinates/address to the Spectra API; receive an asset-level hazard/financial-loss score directly. No further spatial processing required.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Portfolio-ready pipeline</t>
+          <t>Pricing details</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>(1) Geocode exposure addresses to coordinates. (2) Query the GeoSphere Austria grid API with the coordinates for the WINFORE SPEI variable at the desired aggregation window (30/90/365 days). (3) Assign the returned SPEI value to the exposure. Fully automatable, 1km grid resolution.</t>
+          <t>Jupiter's own CEO, Rich Sorkin, stated in a 2022 interview that "subscription pricing ranges from $25,000 to multimillion-dollar contracts" depending on scope (Trellis/Clancy, 2022) - the most directly-attributable figure found for this source, though still not a public price list. Third-party industry comparison sources separately describe full portfolio deployments as typically six-figure annual commitments, consistent with the CEO's stated range (Repath, n.d.; SmartResilience, n.d.).</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Portfolio-ready pipeline</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>SPARTACUS-v3 is a public gridded climate dataset operated by GeoSphere Austria, the Austrian federal institute for geology, geophysics, climatology and meteorology (GeoSphere Austria, n.d.-a). It provides observed daily, monthly and quarterly temperature, precipitation and sunshine-duration fields at 1km resolution across Austria since 1961, updated daily (GeoSphere Austria, n.d.-a). The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge, published under the CC0 1.0 Public Domain Dedication used for most GeoSphere Austria Data Hub datasets (GeoSphere Austria/re3data, n.d.). In the context of Template D 01.01, it is relevant to data point 0050 as a primary source. For an SNCI, the source is suitable because it provides Austria's highest-resolution national gridded observation dataset, finer than Copernicus CDS' ~0.1-0.25 degree grid, with a coordinate-based API enabling direct point queries. In portfolio-readiness terms, the source is ready: once geocoded, an API query per coordinate returns a differentiating, 1km-resolution value, though converting the raw climate variables into a specific heat-wave or heavy-precipitation indicator requires the bank's own threshold definition.</t>
+          <t>Send exposure coordinates/address to the ClimateScore Global API; receive an asset-level hazard/financial-loss score directly. No further spatial processing required.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -8831,303 +9176,303 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>WINFORE is a public gridded drought-index dataset operated by GeoSphere Austria (GeoSphere Austria, n.d.-b). It provides the Standardized Precipitation Evapotranspiration Index (SPEI) at 30-, 90- and 365-day aggregation windows, plus potential evapotranspiration, derived from SPARTACUS temperature and precipitation fields at 1km resolution across Austria, updated daily (GeoSphere Austria, n.d.-b). The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge, published under the CC0 1.0 Public Domain Dedication used for most GeoSphere Austria Data Hub datasets (GeoSphere Austria/re3data, n.d.). In the context of Template D 01.01, it is relevant to data point 0050 as a primary source. For an SNCI, the source is suitable because it is a dedicated, purpose-built national drought index at fine resolution, filling a gap not covered by any other Austrian source in this matrix, although the SPEI value is a standardised statistical anomaly rather than an absolute water-deficit measure. In portfolio-readiness terms, the source is ready: once geocoded, an API query per coordinate returns a differentiating, 1km-resolution SPEI value directly.</t>
+          <t>Spectra is a commercial physical climate risk platform operated by Climate X Ltd, a UK-based company founded in 2020 (Technology Tools, n.d.). It provides asset-level modelled physical hazard scores and financial loss projections across up to 16 hazards (including flooding, storms, tropical cyclones, storm surge, heat stress, wildfires, landslides and subsidence), with scenario projections to 2100 (Repath, n.d.; Net Zero Compare, n.d.). The source is accessed through a commercial SaaS platform and an API, and is paid, subject to a quote-based commercial licence; third-party estimates (not operator-confirmed) suggest a "mid-market" price range of roughly EUR 20,000-60,000 per year for a 30-100 asset portfolio (Repath, n.d.). In the context of Template D 01.01, it is relevant to data points 0050 and 0090–0130 as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Licensing notes</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Commercial, quote-based enterprise SaaS licence; no public price list (Net Zero Compare, n.d.).</t>
+          <t>ClimateScore Global is a commercial physical climate risk platform operated by Jupiter Intelligence, Inc., a US company founded in 2017 (aigreentools.com, n.d.). It provides asset-level modelled physical hazard scores and finance-grade loss metrics across 9 physical perils (including flood, heat, drought, tropical cyclones, wind and wildfire), across 3 emissions scenarios in 5-year increments to 2100, based on peer-reviewed CMIP6/ERA5 science (aigreentools.com, n.d.). The source is accessed through a commercial SaaS platform and an API, and is paid, subject to a quote-based enterprise licence; Jupiter's own CEO has stated subscription pricing ranges from USD 25,000 to multi-million-dollar contracts depending on scope, with full portfolio deployments typically at six-figure annual commitments (Trellis/Clancy, 2022; Repath, n.d.). In the context of Template D 01.01, it is relevant to data points 0050 and 0090–0130 as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Pricing details</t>
+          <t>Data quality notes</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Not publicly disclosed by Climate X directly. Third-party industry comparison sources estimate EUR 20,000-60,000 per year for portfolios of 30-100 assets, described as "mid-market" pricing relative to enterprise platforms like Jupiter Intelligence or Moody's; this figure is a third-party estimate, not confirmed by the operator (Repath, n.d.).</t>
+          <t>Granularity is not uniform across the source: ThinkHazard! resolves to district (ADM2) level, while Risk Data Library datasets vary individually (e.g. the global landslide hazard map is a continuous grid, not administrative-boundary based).</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>eea_climate_adapt</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Portfolio-ready pipeline</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Send exposure coordinates/address to the Spectra API; receive an asset-level hazard/financial-loss score directly. No further spatial processing required.</t>
+          <t>Map portal</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>eea_climate_adapt</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Licensing notes</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Commercial, quote-based enterprise licence; pricing, platform/API packaging and onboarding are defined case-by-case with the client, not publicly listed (Mitiga Solutions, n.d.).</t>
+          <t>Three of the matrix's twelve hazards (permafrost, landslide, soil erosion) have no corresponding index at all; heat stress and water stress are only indirect proxies (UTCI; aridity). Grid resolution varies by indicator (5km for hydrology-based indices to ~28km for most temperature/precipitation/wind indices) - coarser than the parcel-level Austrian sources for acute hazards.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>eea_climate_adapt</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Pricing details</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Jupiter's own CEO, Rich Sorkin, stated in a 2022 interview that "subscription pricing ranges from $25,000 to multimillion-dollar contracts" depending on scope (Trellis/Clancy, 2022) - the most directly-attributable figure found for this source, though still not a public price list. Third-party industry comparison sources separately describe full portfolio deployments as typically six-figure annual commitments, consistent with the CEO's stated range (Repath, n.d.; SmartResilience, n.d.).</t>
+          <t>Not verified - portal/report content, no disclosed refresh cadence.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>jrc_risk_data_hub</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Portfolio-ready pipeline</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Send exposure coordinates/address to the ClimateScore Global API; receive an asset-level hazard/financial-loss score directly. No further spatial processing required.</t>
+          <t>Shapefile, GeoJSON (GIS layers)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>jrc_risk_data_hub</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Spectra is a commercial physical climate risk platform operated by Climate X Ltd, a UK-based company founded in 2020 (Technology Tools, n.d.). It provides asset-level modelled physical hazard scores and financial loss projections across up to 16 hazards (including flooding, storms, tropical cyclones, storm surge, heat stress, wildfires, landslides and subsidence), with scenario projections to 2100 (Repath, n.d.; Net Zero Compare, n.d.). The source is accessed through a commercial SaaS platform and an API, and is paid, subject to a quote-based commercial licence; third-party estimates (not operator-confirmed) suggest a "mid-market" price range of roughly EUR 20,000-60,000 per year for a 30-100 asset portfolio (Repath, n.d.). In the context of Template D 01.01, it is relevant to data points 0050 and 0090–0130 as a primary source. For an SNCI, the source is conditionally suitable because it offers ready-made, high-granularity asset-level scores integrable via API, although its cost and enterprise-SaaS positioning may still exceed a typical SNCI's budget scale. In portfolio-readiness terms, the source is fully ready: the API returns a differentiating, asset-level score directly, with no further spatial processing required.</t>
+          <t>Map portal</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>jrc_risk_data_hub</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>ClimateScore Global is a commercial physical climate risk platform operated by Jupiter Intelligence, Inc., a US company founded in 2017 (aigreentools.com, n.d.). It provides asset-level modelled physical hazard scores and finance-grade loss metrics across 9 physical perils (including flood, heat, drought, tropical cyclones, wind and wildfire), across 3 emissions scenarios in 5-year increments to 2100, based on peer-reviewed CMIP6/ERA5 science (aigreentools.com, n.d.). The source is accessed through a commercial SaaS platform and an API, and is paid, subject to a quote-based enterprise licence; Jupiter's own CEO has stated subscription pricing ranges from USD 25,000 to multi-million-dollar contracts depending on scope, with full portfolio deployments typically at six-figure annual commitments (Trellis/Clancy, 2022; Repath, n.d.). In the context of Template D 01.01, it is relevant to data points 0050 and 0090–0130 as a primary source. For an SNCI, the source is conditionally suitable because of its extensive, scientifically validated hazard and financial-metric coverage; the lower end of its stated pricing range may be within reach for a well-resourced SNCI for a limited scope, although full portfolio deployments are likely well above a typical SNCI's budget scale. In portfolio-readiness terms, the source is fully ready: the API returns a differentiating, asset-level score directly, with no further spatial processing required.</t>
+          <t>Vulnerability and Risk Analysis modules are documented by JRC as 'ongoing work'; coverage marks rely primarily on Exposure Analysis and Historical Events.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>jrc_risk_data_hub</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Data quality notes</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Granularity is not uniform across the source: ThinkHazard! resolves to district (ADM2) level, while Risk Data Library datasets vary individually (e.g. the global landslide hazard map is a continuous grid, not administrative-boundary based).</t>
+          <t>Not verified. Update frequency could not be verified: the Vulnerability and Risk Analysis modules are described by JRC itself as "ongoing work", with no fixed publication cadence stated.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>eea_climate_adapt</t>
+          <t>effis_wildfire</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Map portal</t>
+          <t>Shapefile (vector), GeoTIFF (raster, ~250m resolution)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>eea_climate_adapt</t>
+          <t>effis_wildfire</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>No downloadable or queryable data behind the portal - only a web map/report interface; its own report table resolves to just 3 European macro-regions, with Austria entirely within one, so there is no within-country differentiation.</t>
+          <t>OGC map service (WMS/WFS)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>eea_climate_adapt</t>
+          <t>effis_wildfire</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Not verified - portal/report content, no disclosed refresh cadence.</t>
+          <t>Wildfire only, by design; the fire danger index and burnt-area layers are raw, time-varying raster data, so converting them into a per-exposure attribute requires an explicit aggregation choice (e.g. seasonal max vs long-run average) plus GIS overlay effort.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub</t>
+          <t>effis_wildfire</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Shapefile, GeoJSON (GIS layers)</t>
+          <t>Daily (fire danger index, in-season); burnt-area layer updated per fire season.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Map portal</t>
+          <t>NetCDF (some datasets: GRIB)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability and Risk Analysis modules are documented by JRC as 'ongoing work'; coverage marks rely primarily on Exposure Analysis and Historical Events.</t>
+          <t>Map portal</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Not verified. Update frequency could not be verified: the Vulnerability and Risk Analysis modules are described by JRC itself as "ongoing work", with no fixed publication cadence stated.</t>
+          <t>A vast general-purpose climate data repository, not a ready-made hazard layer - every use requires selecting the right raw variable(s) and building a bespoke pipeline; individual sub-datasets may carry stricter licence terms than the general CC-BY 4.0.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>effis_wildfire</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Shapefile (vector), GeoTIFF (raster, ~250m resolution)</t>
+          <t>Continuous (varies by dataset). Update frequency varies by dataset; ERA5-based datasets are described by ECMWF as "regularly extended" as new reanalysis data become available, without a fixed publication schedule.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>effis_wildfire</t>
+          <t>eba_esg_dashboard</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -9137,14 +9482,14 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>OGC map service (WMS/WFS)</t>
+          <t>Statistics dashboard</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>effis_wildfire</t>
+          <t>eba_esg_dashboard</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -9154,14 +9499,14 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Wildfire only, by design; the fire danger index and burnt-area layers are raw, time-varying raster data, so converting them into a per-exposure attribute requires an explicit aggregation choice (e.g. seasonal max vs long-run average) plus GIS overlay effort.</t>
+          <t>Aggregate EU bank-level statistics only, with no download/API and no per-exposure data whatsoever - relevant only as a peer-comparison/benchmarking reference.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>effis_wildfire</t>
+          <t>eba_esg_dashboard</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -9171,82 +9516,82 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Daily (fire danger index, in-season); burnt-area layer updated per fire season.</t>
+          <t>Biannual (twice a year, per EBA's own publication schedule).</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>NetCDF (some datasets: GRIB)</t>
+          <t>Statistics dashboard</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Map portal</t>
+          <t>Based on AnaCredit/RIAD, not accessible to an SNCI; only the documented methodology is usable as a template.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>A vast general-purpose climate data repository, not a ready-made hazard layer - every use requires selecting the right raw variable(s) and building a bespoke pipeline; individual sub-datasets may carry stricter licence terms than the general CC-BY 4.0.</t>
+          <t>Periodic (no fixed schedule). Update frequency is periodic (documented as successive numbered "releases" of the indicator set), but no fixed public publication schedule was confirmed.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Continuous (varies by dataset). Update frequency varies by dataset; ERA5-based datasets are described by ECMWF as "regularly extended" as new reanalysis data become available, without a fixed publication schedule.</t>
+          <t>GML / Shapefile (per hazard layer, direct .zip links)</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9256,14 +9601,14 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Statistics dashboard</t>
+          <t>OGC WMS/WFS + INSPIRE Atom download service</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -9273,14 +9618,14 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Aggregate EU bank-level statistics only, with no download/API and no per-exposure data whatsoever - relevant only as a peer-comparison/benchmarking reference.</t>
+          <t>Data currency (Datenstand) October 2020, ~6 years old; a composite of several underlying sources (ABU, HORA, BWV/WLV Gefahrenzonenpläne) with potentially inconsistent vintages.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -9290,82 +9635,82 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Biannual (twice a year, per EBA's own publication schedule).</t>
+          <t>Static - Datenstand October 2020 (~6 years old as of this review).</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>Statistics dashboard</t>
+          <t>Shapefile</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>Based on AnaCredit/RIAD, not accessible to an SNCI; only the documented methodology is usable as a template.</t>
+          <t>OGC map service (WMS/WFS)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Periodic (no fixed schedule). Update frequency is periodic (documented as successive numbered "releases" of the indicator set), but no fixed public publication schedule was confirmed.</t>
+          <t>Mapped only within settled areas with designated torrent/avalanche catchments (some still analogue-only); an unmatched location is ambiguous - no hazard or no mapping.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>GML / Shapefile (per hazard layer, direct .zip links)</t>
+          <t>Not verified - no disclosed refresh cadence found.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -9375,14 +9720,14 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>OGC WMS/WFS + INSPIRE Atom download service</t>
+          <t>Single-record lookup</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -9392,14 +9737,14 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Data currency (Datenstand) October 2020, ~6 years old; a composite of several underlying sources (ABU, HORA, BWV/WLV Gefahrenzonenpläne) with potentially inconsistent vintages.</t>
+          <t>No bulk/API access - individual queries only, explicitly prohibited under terms of use; map content is not legally binding.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -9409,14 +9754,14 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>Static - Datenstand October 2020 (~6 years old as of this review).</t>
+          <t>Not verified - no disclosed refresh cadence found.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -9426,14 +9771,14 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Shapefile</t>
+          <t>CSV, Shapefile, GeoPackage (.gpkg). Baseline data is only available as CSV/GeoPackage; the CSV export exceeds the shapefile attribute-column limit, so Shapefile export is not usable for the full 13-indicator baseline dataset.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -9443,14 +9788,14 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>OGC map service (WMS/WFS)</t>
+          <t>Map portal</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -9460,14 +9805,14 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>Mapped only within settled areas with designated torrent/avalanche catchments (some still analogue-only); an unmatched location is ambiguous - no hazard or no mapping.</t>
+          <t>A global tool not locally calibrated/validated for Austria; watershed (Pfafstetter basin) granularity, coarser than the parcel-level Austrian sources.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -9477,14 +9822,14 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>Not verified - no disclosed refresh cadence found.</t>
+          <t>Versioned releases, not continuous (Aqueduct 4.0 launched August 2023).</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -9494,14 +9839,14 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>Single-record lookup</t>
+          <t>Commercial analytics platform</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -9511,14 +9856,14 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>No bulk/API access - individual queries only, explicitly prohibited under terms of use; map content is not legally binding.</t>
+          <t>Confirmed Austria-relevant coverage is narrower than marketed: storm = tropical cyclones (not Austria-relevant); heat-wave and drought coverage unconfirmed. Commercial licensing typically scaled for larger institutions.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -9528,82 +9873,82 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>Not verified - no disclosed refresh cadence found.</t>
+          <t>Not disclosed (commercial product).</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>CSV, Shapefile, GeoPackage (.gpkg). Baseline data is only available as CSV/GeoPackage; the CSV export exceeds the shapefile attribute-column limit, so Shapefile export is not usable for the full 13-indicator baseline dataset.</t>
+          <t>Commercial analytics platform</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>Map portal</t>
+          <t>Heat, drought and water stress are only covered via a separate, unnamed 'Climate Change Edition' - specific coverage unconfirmed. Portfolio-scale subscription access remains quote-based and geared towards larger institutions, though a pay-per-location On-Demand option (from EUR 100-160/location, no subscription) makes single-location spot-checks accessible.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>A global tool not locally calibrated/validated for Austria; watershed (Pfafstetter basin) granularity, coarser than the parcel-level Austrian sources.</t>
+          <t>Not disclosed (commercial product).</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Versioned releases, not continuous (Aqueduct 4.0 launched August 2023).</t>
+          <t>JSON, XML, CSV (API); format varies by dataset for Risk Data Library</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -9613,14 +9958,14 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Commercial analytics platform</t>
+          <t>Web portal (generic)</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -9630,14 +9975,14 @@
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Confirmed Austria-relevant coverage is narrower than marketed: storm = tropical cyclones (not Austria-relevant); heat-wave and drought coverage unconfirmed. Commercial licensing typically scaled for larger institutions.</t>
+          <t>Bundles a downloadable Risk Data Library with ThinkHazard!, a district (ADM2)-level categorical screening tool accessible via API - coarser than the parcel-level Austrian sources.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -9647,150 +9992,150 @@
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Not disclosed (commercial product).</t>
+          <t>Varies by dataset. Update frequency also varies by underlying dataset: ThinkHazard! harvests from GeoNode on an ongoing basis, but individual hazard-layer vintages within the Risk Data Library differ and were not individually verified.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Commercial analytics platform</t>
+          <t>PDF (reports)</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Heat, drought and water stress are only covered via a separate, unnamed 'Climate Change Edition' - specific coverage unconfirmed. Portfolio-scale subscription access remains quote-based and geared towards larger institutions, though a pay-per-location On-Demand option (from EUR 100-160/location, no subscription) makes single-location spot-checks accessible.</t>
+          <t>Reports/publications website</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Not disclosed (commercial product).</t>
+          <t>Station-/object-based narrative reporting, not a spatial hazard layer; cannot be overlaid with individual portfolio locations.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>JSON, XML, CSV (API); format varies by dataset for Risk Data Library</t>
+          <t>Periodic reports; no fixed publication schedule disclosed.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>Web portal (generic)</t>
+          <t>CSV</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Bundles a downloadable Risk Data Library with ThinkHazard!, a district (ADM2)-level categorical screening tool accessible via API - coarser than the parcel-level Austrian sources.</t>
+          <t>Web portal (generic)</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Varies by dataset. Update frequency also varies by underlying dataset: ThinkHazard! harvests from GeoNode on an ongoing basis, but individual hazard-layer vintages within the Risk Data Library differ and were not individually verified.</t>
+          <t>Companies without an assigned OeNACE code remain unmatched; unregistered sole traders are out of scope.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>PDF (reports)</t>
+          <t>Continuous (per Statistik Austria's own licensing description).</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -9800,14 +10145,14 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>Reports/publications website</t>
+          <t>Web portal (generic)</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -9817,14 +10162,14 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>Station-/object-based narrative reporting, not a spatial hazard layer; cannot be overlaid with individual portfolio locations.</t>
+          <t>Cost is institution-dependent - some banks may already hold a sector licence; classification is editorially enriched, not the official statistical assignment.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -9834,14 +10179,14 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>Periodic reports; no fixed publication schedule disclosed.</t>
+          <t>Daily (per operator's own product description).</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -9851,14 +10196,14 @@
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>NetCDF (grid), CSV/GeoJSON (API point queries)</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -9868,14 +10213,14 @@
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Web portal (generic)</t>
+          <t>Web-UI + REST API (coordinate-based point queries) + HTTP bulk file download</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -9885,14 +10230,14 @@
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>Companies without an assigned OeNACE code remain unmatched; unregistered sole traders are out of scope.</t>
+          <t>Grid-based climate variables (temperature, precipitation, sunshine), not a pre-classified hazard/risk score - requires own threshold definition to convert into a heat_wave or heavy_precip indicator.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -9902,330 +10247,347 @@
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>Continuous (per Statistik Austria's own licensing description).</t>
+          <t>Daily (operationally extended; last 7 days provisional, final after 7 days).</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Web portal (generic)</t>
+          <t>NetCDF (grid), CSV/GeoJSON (API point queries)</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>Cost is institution-dependent - some banks may already hold a sector licence; classification is editorially enriched, not the official statistical assignment.</t>
+          <t>Web-UI + REST API (coordinate-based point queries) + HTTP bulk file download</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Daily (per operator's own product description).</t>
+          <t>SPEI is a standardised statistical anomaly index (derived from SPARTACUS via a normal-distribution transform over two climate reference periods), not an absolute water-deficit value - interpretation requires understanding this transform.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>NetCDF (grid), CSV/GeoJSON (API point queries)</t>
+          <t>Daily.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Web-UI + REST API (coordinate-based point queries) + HTTP bulk file download</t>
+          <t>API export; platform UI</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Grid-based climate variables (temperature, precipitation, sunshine), not a pre-classified hazard/risk score - requires own threshold definition to convert into a heat_wave or heavy_precip indicator.</t>
+          <t>Commercial SaaS platform + API</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>Daily (operationally extended; last 7 days provisional, final after 7 days).</t>
+          <t>Pricing and the full hazard list are not published by the operator directly - see Pricing details for third-party estimates.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>NetCDF (grid), CSV/GeoJSON (API point queries)</t>
+          <t>Not disclosed (commercial product).</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Download format</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Web-UI + REST API (coordinate-based point queries) + HTTP bulk file download</t>
+          <t>API export; platform UI</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Web interface type</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>SPEI is a standardised statistical anomaly index (derived from SPARTACUS via a normal-distribution transform over two climate reference periods), not an absolute water-deficit value - interpretation requires understanding this transform.</t>
+          <t>Commercial SaaS platform + API</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>Daily.</t>
+          <t>Pricing is enterprise/quote-based, not publicly listed - see Pricing details for the CEO-stated range and typical full-deployment cost.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>API export; platform UI</t>
+          <t>Not disclosed (commercial product).</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Licensing notes</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Commercial SaaS platform + API</t>
+          <t>CC-BY 4.0, same general CDS licence as copernicus_cds; ERA5-HEAT and SMHI hydrology datasets carry standard C3S licence terms, CEMS Fire Danger per Copernicus Emergency Management Service terms.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Data update frequency</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>Pricing and the full 16-hazard list are not published; third-party estimates suggest EUR 20,000-60,000/year for 30-100 assets, but this was not confirmed by the operator directly.</t>
+          <t>Varies by product: ERA5-HEAT is regularly extended as new ERA5 data become available; SMHI hydrology projections are static 30-year model outputs (not continuously updated); CEMS Fire Danger is updated in near real time.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Portfolio-ready pipeline</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>Not disclosed (commercial product).</t>
+          <t>(1) Geocode exposure addresses to coordinates. (2) Query or download the relevant standalone product (ERA5-HEAT for heat stress, SMHI hydrology for flood/water stress/soil-moisture drought, CEMS Fire Danger for wildfire) for the coordinate. (3) Assign the returned value to the exposure. Fully automatable; each product is a ready-made, named indicator, not a raw variable requiring own processing.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Download format</t>
+          <t>technical_effort rationale</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>API export; platform UI</t>
+          <t>Rated Low: unlike raw copernicus_cds variables, each of these is a purpose-built, ready-made indicator product with documented methodology (peer-reviewed for ERA5-HEAT, produced by a named national institute for the SMHI hydrology dataset) - no own index/threshold definition needed, only geocoding and grid extraction.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Web interface type</t>
+          <t>Suitability assessment</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>Commercial SaaS platform + API</t>
+          <t>Split out from copernicus_cds (Aug 2026 revision) because these specific products - unlike the bulk of Copernicus CDS, which requires own processing of raw climate variables - are standalone, ready-made, documented hazard indicators with their own CDS catalogue pages and named producing institutions. Treating them as part of the generic "copernicus_cds" entry would have understated their portfolio-readiness and overstated their technical effort.</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>Jupiter's CEO has stated subscription pricing ranges from USD 25,000 to multi-million-dollar contracts depending on scope - the lower end may be within reach for a well-resourced SNCI, but full portfolio deployments are typically six-figure annual commitments.</t>
+          <t>This is a set of standalone, ready-made physical hazard indicator products, published as individual datasets on the Copernicus Climate Data Store (CDS), distinct from the general-purpose raw climate variables covered by the separate copernicus_cds entry (ECMWF, n.d.). It comprises: ERA5-HEAT (UTCI/heat stress, peer-reviewed, ECMWF), the SMHI hydrology dataset (flood, water stress/aridity, soil-moisture drought, produced by the Swedish Meteorological and Hydrological Institute for C3S), and CEMS Fire Danger (wildfire, produced by JRC/Copernicus Emergency Management Service) (Di Napoli et al., 2021; SMHI/C3S, n.d.). Each is directly downloadable and queryable via the CDS API, and is free to use under CC-BY 4.0-equivalent terms. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Data update frequency</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>Not disclosed (commercial product).</t>
+          <t>Only covers 5 of 12 matrix hazards (heat_stress, flood, water_stress, drought via soil moisture, wildfire); meteorological (SPI-3) drought and the temperature/precipitation/wind-based ECDE indices (heat_wave, heavy_precip, storm) are not available as standalone products - only via copernicus_cds raw variables or the Climate-ADAPT-curated bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>effis_wildfire</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Data quality notes</t>
+        </is>
+      </c>
+      <c r="C168" s="4" t="inlineStr">
+        <is>
+          <t>EFFIS has been a component of the Copernicus Emergency Management Service since 2015 (effis.jrc.ec.europa.eu now redirects to forest-fire.emergency.copernicus.eu). It is organisationally related to, but distinct from, the "CEMS Fire Danger historical" dataset credited under copernicus_climate_indicators: that dataset is only the ERA5-driven meteorological fire-danger reconstruction, hosted on the CDS for bulk API access, whereas EFFIS additionally provides the observed European Fire Database (~2 million individual fire records) and its own portal-based applications (Current Situation Viewer, Wildfire Risk Viewer, etc.), not available via the CDS.</t>
         </is>
       </c>
     </row>
@@ -10244,7 +10606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -10294,7 +10656,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10307,7 +10668,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10320,7 +10680,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10333,7 +10692,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -10346,7 +10704,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -10359,7 +10716,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -10372,7 +10728,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -10385,7 +10740,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -10398,7 +10752,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -10411,7 +10764,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -10424,7 +10776,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -10437,7 +10788,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -10450,7 +10800,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10463,7 +10812,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10476,7 +10824,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -10489,7 +10836,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -10502,7 +10848,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -10515,7 +10860,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -10528,7 +10872,6 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -10541,7 +10884,18 @@
           <t>primary</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>copernicus_climate_indicators</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -10605,11 +10959,11 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub, effis_wildfire, copernicus_cds, hq_flood_extent, wlv_gefahrenzonenplan, wri_aqueduct, world_bank_gfdrr, kryomon_at, hvd_fbnr_oenace, geosphere_spartacus, geosphere_winfore_spei</t>
+          <t>eea_climate_adapt, jrc_risk_data_hub, effis_wildfire, copernicus_cds, hq_flood_extent, wlv_gefahrenzonenplan, wri_aqueduct, world_bank_gfdrr, kryomon_at, hvd_fbnr_oenace, geosphere_spartacus, geosphere_winfore_spei, copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -10620,11 +10974,11 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub, copernicus_cds, wri_aqueduct, moodys_physical_risk, munich_re_nathan, world_bank_gfdrr, wirtschafts_compass, geosphere_spartacus, geosphere_winfore_spei, climate_x, jupiter_intelligence</t>
+          <t>eea_climate_adapt, jrc_risk_data_hub, copernicus_cds, wri_aqueduct, moodys_physical_risk, munich_re_nathan, world_bank_gfdrr, wirtschafts_compass, geosphere_spartacus, geosphere_winfore_spei, climate_x, jupiter_intelligence, copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -11087,7 +11441,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Abstract = full-text description with citations. Suitability assessment = why/how suitable for an SNCI. Licensing notes = licence terms. Limitations = known constraints (moved from the former key_limitation column). Download format = file format(s) available for download, where applicable. Web interface type = the specific interactive access channel (e.g. OGC map service, statistics dashboard, commercial SaaS platform). Data update frequency = how often the source's own data is refreshed (moved from the former data_update_frequency column). Data quality notes = data quality/versioning specifics. technical_effort rationale = justifies the Low/Medium/High rating. Portfolio-ready pipeline = concrete steps to make the source portfolio-ready. Pricing details = concrete cost information for commercial sources. Hazard coverage correction note = documents a correction from the Aug 2026 review.</t>
+          <t>Abstract = descriptive-only text with citations (what the source is, what it covers, how it is accessed) - the suitability/limitation reasoning is intentionally left out here to avoid duplicating the Limitations and portfolio_ready fields. The full thesis-facing version (Abstract + suitability/limitation reasoning combined into one paragraph, per the approved template) is in source_abstracts_cited.md, not duplicated here. Suitability assessment = why/how suitable for an SNCI. Licensing notes = licence terms. Limitations = known constraints (moved from the former key_limitation column). Download format = file format(s) available for download, where applicable. Web interface type = the specific interactive access channel (e.g. OGC map service, statistics dashboard, commercial SaaS platform). Data update frequency = how often the source's own data is refreshed (moved from the former data_update_frequency column). Data quality notes = data quality/versioning specifics. technical_effort rationale = justifies the Low/Medium/High rating. Portfolio-ready pipeline = concrete steps to make the source portfolio-ready. Pricing details = concrete cost information for commercial sources. Hazard coverage correction note = documents a correction from the Aug 2026 review.</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Track d01_mapping.csv dropping the per-mapping relevance column
d01_mapping.csv no longer has a `relevance` (primary/secondary) column
per data-point mapping - the D 01.01 Mapping badges in the detail view
now show just the data point (e.g. "0050", "0090-0130"). The source's
overall relevance_level is unaffected and still shown in the metadata
chips, which is where that judgement now lives exclusively.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6tTWnYUJ1DiozJbfUjD1w
</commit_message>
<xml_diff>
--- a/data/ESG_Data_Source_Matrix_Structured.xlsx
+++ b/data/ESG_Data_Source_Matrix_Structured.xlsx
@@ -6875,22 +6875,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Source id</t>
+          <t>source_id</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Template</t>
+          <t>template</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Dpm table</t>
+          <t>dpm_table</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Data point</t>
+          <t>data_point</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -6920,11 +6920,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6947,11 +6942,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6974,11 +6964,6 @@
           <t>0090-0130</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7001,11 +6986,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7028,11 +7008,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7055,11 +7030,6 @@
           <t>0090-0130</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7082,11 +7052,6 @@
           <t>Benchmarking</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7109,11 +7074,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7136,11 +7096,6 @@
           <t>0090-0130</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7163,11 +7118,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7190,11 +7140,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7217,11 +7162,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7244,11 +7184,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7271,11 +7206,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7298,11 +7228,6 @@
           <t>0090-0130</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7325,11 +7250,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7352,11 +7272,6 @@
           <t>0090-0130</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7379,11 +7294,6 @@
           <t>Context/validation</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7406,11 +7316,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7433,11 +7338,6 @@
           <t>NACE subsectors</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7460,11 +7360,6 @@
           <t>NACE subsectors</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7487,11 +7382,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7514,11 +7404,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7541,11 +7426,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7568,11 +7448,6 @@
           <t>0090-0130</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7595,11 +7470,6 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7622,11 +7492,6 @@
           <t>0090-0130</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7647,11 +7512,6 @@
       <c r="D32" t="inlineStr">
         <is>
           <t>0050</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Primary</t>
         </is>
       </c>
     </row>
@@ -7722,7 +7582,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated Medium because the source provides pre-computed, peer-reviewed climate hazard indices (e.g. Hot Days count, SPI-3 drought index) via the ECDE indicator dataset on the CDS, so no own index or threshold definition is needed, unlike raw Copernicus CDS variables. However, geocoding of exposure addresses and grid extraction are still required, and grid resolution varies by indicator (5km to approximately 28km). This rating was revised from an earlier Low rating, because the source does have real, queryable data behind it, not merely a web report.</t>
+          <t>Technical effort is rated Medium because the source provides pre-computed, peer-reviewed climate hazard indices (e.g. Hot Days count, SPI-3 drought index) via the ECDE indicator dataset on the CDS, so no own index or threshold definition is needed, unlike raw Copernicus CDS variables. However, geocoding of exposure addresses and grid extraction are still required, and grid resolution varies by indicator (5km to approximately 28km).</t>
         </is>
       </c>
     </row>
@@ -7807,7 +7667,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated Low because the source is a single national shapefile dataset with its own download service. It requires geocoding and a standard spatial overlay, but no merging of separate state datasets. This rating was revised from an earlier Medium rating, and is consistent with hq_flood_extent (HQ30), which has near-identical technical characteristics.</t>
+          <t>Technical effort is rated Low because the source is a single national shapefile dataset with its own download service. It requires geocoding and a standard spatial overlay, but no merging of separate state datasets, consistent with hq_flood_extent (HQ30), which has near-identical technical characteristics.</t>
         </is>
       </c>
     </row>
@@ -8912,7 +8772,7 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Climate-ADAPT is a public knowledge portal operated by the European Environment Agency (EEA) (EEA, n.d.-a). It provides pre-computed, peer-reviewed climate hazard indices via the European Climate Data Explorer (ECDE), covering heat, precipitation, flood, drought, storm and wildfire hazards at EU-wide scope and grid-based granularity (0.1-0.25 degrees, 5km for hydrology-based indices) (EEA/C3S, n.d.). The source is accessed through a web portal, a queryable API and direct download, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source.</t>
+          <t>Climate-ADAPT is a public knowledge portal operated by the European Environment Agency (EEA) (EEA, n.d.-a). It provides pre-computed, peer-reviewed climate hazard indices via the European Climate Data Explorer (ECDE), covering heat, precipitation, flood, drought, storm and wildfire hazards at EU-wide scope and grid-based granularity (0.1-0.25 degrees, 5km for hydrology-based indices) (EEA/C3S, n.d.). The source is accessed through a web portal, a queryable API and direct download, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -8929,7 +8789,7 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is incomplete hazard coverage. In particular, permafrost, landslide and soil erosion have no corresponding index at all, and heat stress and water stress are only covered via indirect proxies (UTCI; aridity), not dedicated indicators (EEA, 2021). Consequently, the source cannot serve as a comprehensive physical-risk data source on its own, unless complemented by other Austrian or EU sources for the missing hazards.</t>
+          <t>The main limitation is that heat stress and water stress are only covered via indirect proxies (UTCI; aridity), not dedicated indicators (EEA, 2021). In particular, these two proxies were not designed as hazard-specific indices and require careful interpretation before being treated as equivalent to the source's genuinely dedicated indices for heat wave, flood, drought, storm and wildfire. Consequently, the proxy-based hazards cannot be used with the same confidence as the dedicated ones, unless cross-checked against a hazard-specific source.</t>
         </is>
       </c>
     </row>
@@ -8958,12 +8818,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available without registration (EEA, n.d.-a). No licence-specific restrictions on commercial or systematic use were identified beyond standard EU open-data attribution practice.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query or download the relevant ECDE indicator dataset (sis-ecde-climate-indicators, hosted on the CDS) and assign the returned indicator value to each exposure. The result is grid-level (5km to approximately 28km, depending on indicator). The process is fully automatable.</t>
         </is>
       </c>
     </row>
@@ -8975,29 +8835,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query or download the relevant ECDE indicator dataset (sis-ecde-climate-indicators, hosted on the CDS) and assign the returned indicator value to each exposure. The result is grid-level (5km to approximately 28km, depending on indicator). The process is fully automatable.</t>
+          <t>The source is available under the same CC-BY 4.0 licence that applies to the underlying Copernicus Climate Data Store since 2 July 2025 (ECMWF Forum, 2025). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>eea_climate_adapt</t>
+          <t>jrc_risk_data_hub</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>The source is available under the same CC-BY 4.0 licence that applies to the underlying Copernicus Climate Data Store since 2 July 2025 (ECMWF Forum, 2025). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
+          <t>The Risk Data Hub (RDH) is a public multi-hazard risk and loss data platform operated by the Joint Research Centre (JRC) in cooperation with the EU Disaster Risk Management Knowledge Centre (DRMKC) (JRC DRMKC, n.d.). It provides modelled hazard, exposure and historical-loss data covering flood, landslide, earthquake, wildfire and subsidence at NUTS 2/3 granularity across EU, EFTA and IPA countries (Antofie et al., 2023). The source is accessed through a web portal, direct download and an API, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -9009,12 +8869,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>The Risk Data Hub (RDH) is a public multi-hazard risk and loss data platform operated by the Joint Research Centre (JRC) in cooperation with the EU Disaster Risk Management Knowledge Centre (DRMKC) (JRC DRMKC, n.d.). It provides modelled hazard, exposure and historical-loss data covering flood, landslide, earthquake, wildfire and subsidence at NUTS 2/3 granularity across EU, EFTA and IPA countries (Antofie et al., 2023). The source is accessed through a web portal, direct download and an API, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>The main limitation is that the Vulnerability and Risk Analysis modules are documented by JRC itself as 'ongoing work'. In particular, only the Exposure Analysis and Historical Events modules provide reliably usable, hazard-verified layers at present. Consequently, the source's modelled hazard layers cannot be treated as uniformly mature across all five hazards it addresses, unless cross-checked against the specific module status documented per hazard.</t>
         </is>
       </c>
     </row>
@@ -9026,12 +8886,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that the Vulnerability and Risk Analysis modules are documented by JRC itself as 'ongoing work'. In particular, only the Exposure Analysis and Historical Events modules provide reliably usable, hazard-verified layers, and several matrix hazards (heat stress, water stress, soil erosion, glacial lake, permafrost) are not covered at all. Consequently, the source cannot be treated as a complete multi-hazard reference, unless cross-checked against the specific hazard coverage documented per module.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is EU-wide consistent methodology combined with genuine hazard-and-exposure modelling for five hazards (Antofie et al., 2023). It is particularly useful for substantive risk determination at data point 0050. However, its suitability is reduced by NUTS 2/3-level granularity, coarser than Austria's parcel-level sources, and by being over-specified for the pure Geography reporting requirement. It is therefore best used as a primary source for hazard determination, complemented by finer Austrian layers where available.</t>
         </is>
       </c>
     </row>
@@ -9043,12 +8903,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is EU-wide consistent methodology combined with genuine hazard-and-exposure modelling for five hazards (Antofie et al., 2023). It is particularly useful for substantive risk determination at data point 0050. However, its suitability is reduced by NUTS 2/3-level granularity, coarser than Austria's parcel-level sources, and by being over-specified for the pure Geography reporting requirement. It is therefore best used as a primary source for hazard determination, complemented by finer Austrian layers where available.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then identify the corresponding NUTS 2/3 region and query or download the relevant hazard module via API or shapefile, assigning the regional value to each exposure. The result is regional (NUTS 2/3), not parcel-level. The process is fully automatable.</t>
         </is>
       </c>
     </row>
@@ -9060,46 +8920,46 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available without registration (JRC DRMKC, n.d.). No commercial-use restrictions were identified beyond standard attribution requirements.</t>
+          <t>The source is available under an open EU data licence with attribution required, consistent with JRC's general data-sharing terms (JRC DRMKC, n.d.). The licence permits commercial use and systematic portfolio processing, provided that the source is appropriately credited.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub</t>
+          <t>effis_wildfire</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then identify the corresponding NUTS 2/3 region and query or download the relevant hazard module via API or shapefile, assigning the regional value to each exposure. The result is regional (NUTS 2/3), not parcel-level. The process is fully automatable.</t>
+          <t>EFFIS (European Forest Fire Information System) is a public wildfire information service operated jointly by the JRC and the Copernicus Emergency Management Service (JRC/Copernicus EMS, n.d.). It provides a daily fire danger forecast and a historical burnt-area database covering wildfire hazard across Europe, the Middle East and North Africa at grid resolutions ranging from approximately 8-16km (forecast) to 250m/20m (observed burnt area) (EFFIS, n.d.-b). The source is accessed through an OGC map service (WMS/WFS) and direct download, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>jrc_risk_data_hub</t>
+          <t>effis_wildfire</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>The source is available under an open EU data licence with attribution required, consistent with JRC's general data-sharing terms (JRC DRMKC, n.d.). The licence permits commercial use and systematic portfolio processing, provided that the source is appropriately credited.</t>
+          <t>The main limitation is that the fire danger forecast grid (~8-16km) is coarse relative to Austria's size, covering the whole country with only a handful of grid cells. In particular, the much finer 250m/20m burnt-area layer is retrospective/observational rather than a forward-looking exposure indicator, so it cannot substitute for the coarser forecast when a forward-looking classification is needed. Consequently, the source cannot support fine-grained forward-looking wildfire exposure classification on its own, unless combined with the observed burnt-area history for plausibility checks.</t>
         </is>
       </c>
     </row>
@@ -9111,12 +8971,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>EFFIS (European Forest Fire Information System) is a public wildfire information service operated jointly by the JRC and the Copernicus Emergency Management Service (JRC/Copernicus EMS, n.d.). It provides a daily fire danger forecast and a historical burnt-area database covering wildfire hazard across Europe, the Middle East and North Africa at grid resolutions ranging from approximately 8-16km (forecast) to 250m/20m (observed burnt area) (EFFIS, n.d.-b). The source is accessed through an OGC map service (WMS/WFS) and direct download, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is being the only dedicated European wildfire dataset covering both forecast fire danger and observed fire history (JRC/Copernicus EMS, n.d.). It is particularly useful for national-level wildfire screening and historical plausibility checks. However, its suitability is reduced by the coarse forecast-grid resolution for a country the size of Austria and by the raw, unprocessed nature of both layers. It is therefore best used as a supplementary source for wildfire, complemented by own aggregation of the raw data.</t>
         </is>
       </c>
     </row>
@@ -9128,12 +8988,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that the source covers wildfire only, by design. In particular, the fire danger forecast grid (~8-16km) is coarse relative to Austria's size, covering the whole country with only a handful of grid cells, while the finer 250m/20m burnt-area layer is retrospective/observational rather than a forward-looking exposure indicator. Consequently, the source cannot support fine-grained forward-looking wildfire exposure classification on its own, unless combined with the observed burnt-area history for plausibility checks.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the WMS/WFS service or download the relevant GeoTIFF layer (fire danger forecast or burnt area) and extract the raster cell value at each coordinate, assigning it to the exposure. The result is grid-level (~8-16km for fire danger, 250m/20m for burnt area). The process is partly automatable, since aggregating the time-varying raster into a single exposure attribute requires a methodological choice.</t>
         </is>
       </c>
     </row>
@@ -9145,63 +9005,63 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is being the only dedicated European wildfire dataset covering both forecast fire danger and observed fire history (JRC/Copernicus EMS, n.d.). It is particularly useful for national-level wildfire screening and historical plausibility checks. However, its suitability is reduced by the coarse forecast-grid resolution for a country the size of Austria and by the raw, unprocessed nature of both layers. It is therefore best used as a supplementary source for wildfire, complemented by own aggregation of the raw data.</t>
+          <t>The source is available under a CC BY 4.0 licence, as confirmed on EFFIS's own dedicated data-licence page (EFFIS, n.d.-c). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>effis_wildfire</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available under a CC BY 4.0 licence (EFFIS, n.d.-c). Attribution is required when the data is reused.</t>
+          <t>The Copernicus Climate Data Store (CDS) is a public climate data repository operated by ECMWF on behalf of the EU (ECMWF, n.d.), comprising over 140 datasets of raw and derived climate variables and reanalysis/projection data. It provides raw climate variables (e.g. temperature, precipitation, wind fields) covering multiple physical hazards at grid resolutions of roughly 0.1-0.25 degrees globally, with an EU focus. The source is accessed through a web portal, direct download and an API, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>effis_wildfire</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the WMS/WFS service or download the relevant GeoTIFF layer (fire danger forecast or burnt area) and extract the raster cell value at each coordinate, assigning it to the exposure. The result is grid-level (~8-16km for fire danger, 250m/20m for burnt area). The process is partly automatable, since aggregating the time-varying raster into a single exposure attribute requires a methodological choice.</t>
+          <t>The main limitation is that the source provides raw climate variables rather than ready-made hazard indicators. In particular, every use requires selecting the correct raw variable(s) and building a bespoke climatological/GIS pipeline, and individual sub-datasets may carry stricter licence terms than the general CC-BY 4.0 (e.g. E-OBS, restricted to non-commercial research/education use). Consequently, the source cannot be used directly for exposure classification, unless the institution builds and validates its own index-derivation methodology.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>effis_wildfire</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>The source is available under a CC BY 4.0 licence, as confirmed on EFFIS's own dedicated data-licence page (EFFIS, n.d.-c). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is being authoritative, EU-wide consistent and covering the broadest range of underlying climate variables of any source in the matrix (ECMWF, n.d.). It is particularly useful as the raw-data foundation when no ready-made indicator exists elsewhere. However, its suitability is reduced by the substantial climatological and GIS processing effort required before any variable becomes an exposure classification. It is therefore best used as a fallback source for hazards not covered by ready-made products, rather than as an operational primary source.</t>
         </is>
       </c>
     </row>
@@ -9213,12 +9073,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>The Copernicus Climate Data Store (CDS) is a public climate data repository operated by ECMWF on behalf of the EU (ECMWF, n.d.), comprising over 140 datasets of raw and derived climate variables and reanalysis/projection data. It provides raw climate variables (e.g. temperature, precipitation, wind fields) covering multiple physical hazards at grid resolutions of roughly 0.1-0.25 degrees globally, with an EU focus. The source is accessed through a web portal, direct download and an API, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then select and download the relevant climate variable(s) in NetCDF/GRIB format and derive a hazard-relevant indicator through own climatological modelling, assigning the result to each exposure. The result is grid-level (~0.1-0.25 degrees). The process requires substantial manual/methodological intervention and is not fully automatable without an own index-derivation methodology.</t>
         </is>
       </c>
     </row>
@@ -9230,80 +9090,80 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that the source provides raw climate variables rather than ready-made hazard indicators. In particular, every use requires selecting the correct raw variable(s) and building a bespoke climatological/GIS pipeline, and individual sub-datasets may carry stricter licence terms than the general CC-BY 4.0 (e.g. E-OBS, restricted to non-commercial research/education use). Consequently, the source cannot be used directly for exposure classification, unless the institution builds and validates its own index-derivation methodology.</t>
+          <t>The source is available under CC-BY 4.0 since 2 July 2025, replacing the previous bespoke "Licence to Use Copernicus Products" (Version 1.2, Nov 2019) that governed CDS access before that date (ECMWF Forum, 2025). Attribution is required when the data is reused. Individual sub-datasets may carry stricter third-party terms and should be verified per dataset before use.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>eba_esg_dashboard</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is being authoritative, EU-wide consistent and covering the broadest range of underlying climate variables of any source in the matrix (ECMWF, n.d.). It is particularly useful as the raw-data foundation when no ready-made indicator exists elsewhere. However, its suitability is reduced by the substantial climatological and GIS processing effort required before any variable becomes an exposure classification. It is therefore best used as a fallback source for hazards not covered by ready-made products, rather than as an operational primary source.</t>
+          <t>The EBA ESG Dashboard is a public statistics dashboard operated by the European Banking Authority (EBA) (EBA, n.d.-a). It provides aggregated ESG risk indicators at EU bank level, covering both physical and transition climate risk at institution/portfolio-level granularity across the EU/EEA (EBA, n.d.-a). The source is accessed through a statistics dashboard, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>eba_esg_dashboard</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge (ECMWF, n.d.), though registration is required to download data.</t>
+          <t>The main limitation is that the source provides only aggregate EU bank-level statistics (EBA, n.d.-a). In particular, no download or API access exists and no per-exposure data is available whatsoever. Consequently, the source cannot be used to populate any individual exposure in D 01.01, unless it is used purely for peer-comparison or benchmarking purposes.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>eba_esg_dashboard</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then select and download the relevant climate variable(s) in NetCDF/GRIB format and derive a hazard-relevant indicator through own climatological modelling, assigning the result to each exposure. The result is grid-level (~0.1-0.25 degrees). The process requires substantial manual/methodological intervention and is not fully automatable without an own index-derivation methodology.</t>
+          <t>For an SNCI, the source is not suitable for populating individual exposures. Its main advantage is providing an authoritative EU/EEA peer-comparison benchmark (EBA, n.d.-a). It is particularly useful for contextualising an institution's own physical and transition risk exposure against sector averages. However, its suitability is reduced by the complete absence of per-exposure or downloadable data. It is therefore best used purely as a context/benchmarking source, not as an operational data source.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>copernicus_cds</t>
+          <t>eba_esg_dashboard</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>The source is available under CC-BY 4.0 since 2 July 2025, replacing the previous bespoke "Licence to Use Copernicus Products" (Version 1.2, Nov 2019) that governed CDS access before that date (ECMWF Forum, 2025). Attribution is required when the data is reused. Individual sub-datasets may carry stricter third-party terms and should be verified per dataset before use.</t>
+          <t>Not applicable: the source provides only aggregate EU bank-level statistics with no per-exposure data (EBA, n.d.-a), so no portfolio-level pipeline can be built against it.</t>
         </is>
       </c>
     </row>
@@ -9315,70 +9175,70 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>The EBA ESG Dashboard is a public statistics dashboard operated by the European Banking Authority (EBA) (EBA, n.d.-a). It provides aggregated ESG risk indicators at EU bank level, covering both physical and transition climate risk at institution/portfolio-level granularity across the EU/EEA (EBA, n.d.-a). The source is accessed through a statistics dashboard, and is free of charge. In the context of Template D 01.01, it is relevant to benchmarking as a context-only source.</t>
+          <t>The source is available under the EBA's standard open-data terms, free of charge and without registration (EBA, n.d.-a). No restrictions on commercial or systematic use beyond standard attribution practice were identified.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that the source provides only aggregate EU bank-level statistics (EBA, n.d.-a). In particular, no download or API access exists and no per-exposure data is available whatsoever. Consequently, the source cannot be used to populate any individual exposure in D 01.01, unless it is used purely for peer-comparison or benchmarking purposes.</t>
+          <t>This is a public methodological and statistical resource operated by the European Central Bank (ECB) (ECB, n.d.). It provides a documented physical-risk indicator methodology and euro-area aggregate statistics, covering coastal flooding, river flooding, wildfires, landslides, subsidence, windstorms, water stress, droughts and rainfall variation at institution/portfolio-level granularity (ECB, n.d.). The source is accessed through a statistics dashboard, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is not suitable for populating individual exposures. Its main advantage is providing an authoritative EU/EEA peer-comparison benchmark (EBA, n.d.-a). It is particularly useful for contextualising an institution's own physical and transition risk exposure against sector averages. However, its suitability is reduced by the complete absence of per-exposure or downloadable data. It is therefore best used purely as a context/benchmarking source, not as an operational data source.</t>
+          <t>The main limitation is that the underlying supervisory data (AnaCredit/RIAD) is not accessible to an SNCI. In particular, the published output is aggregate/dashboard statistics with no per-exposure data. Consequently, the source cannot be used directly to classify individual exposures, unless the bank replicates the documented methodology using its own AnaCredit-equivalent data plus JRC/Copernicus hazard layers.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available without registration (EBA, n.d.-a).</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is a transparent, replicable methodology covering nine physical hazards with an authoritative EU-level pedigree (ECB, n.d.). It is particularly useful as a methodological template for building an in-house classification approach. However, its suitability is reduced by the inaccessibility of the ECB's own underlying supervisory data to a non-significant institution. It is therefore best used as a methodological anchor rather than as a direct operational data source.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -9388,14 +9248,14 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Not applicable: the source provides only aggregate EU bank-level statistics with no per-exposure data (EBA, n.d.-a), so no portfolio-level pipeline can be built against it.</t>
+          <t>Not applicable via this source directly, since its output is aggregate/dashboard statistics rather than per-exposure data (ECB, n.d.). A per-exposure pipeline would instead need to replicate the ECB's published methodology using the bank's own AnaCredit-equivalent data plus JRC/Copernicus hazard layers.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -9405,14 +9265,14 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>The source is available under the EBA's standard open-data terms, free of charge and without registration (EBA, n.d.-a). No restrictions on commercial or systematic use beyond standard attribution practice were identified.</t>
+          <t>The source is available under the ECB's standard open-data terms, free of charge and without registration (ECB, n.d.). No restrictions on commercial or systematic use beyond standard attribution practice were identified.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -9422,14 +9282,14 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>This is a public methodological and statistical resource operated by the European Central Bank (ECB) (ECB, n.d.). It provides a documented physical-risk indicator methodology and euro-area aggregate statistics, covering coastal flooding, river flooding, wildfires, landslides, subsidence, windstorms, water stress, droughts and rainfall variation at institution/portfolio-level granularity (ECB, n.d.). The source is accessed through a statistics dashboard, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a methodological source.</t>
+          <t>This is a national flood extent dataset, published via the INSPIRE Geoportal Oesterreich, with the Bundesministerium fuer Land- und Forstwirtschaft, Klima- und Umweltschutz, Regionen und Wasserwirtschaft (BMLUK) as data owner and Umweltbundesamt GmbH as technical operator (INSPIRE Geoportal Oesterreich, n.d.-b). It provides harmonised flood extent layers for the 30-, 100- and 300-year return periods, covering flood hazard at parcel/address-level granularity across Austria. The source is accessed through OGC WMS/WFS services and direct GML/shapefile download, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -9439,14 +9299,14 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that the underlying supervisory data (AnaCredit/RIAD) is not accessible to an SNCI. In particular, the published output is aggregate/dashboard statistics with no per-exposure data. Consequently, the source cannot be used directly to classify individual exposures, unless the bank replicates the documented methodology using its own AnaCredit-equivalent data plus JRC/Copernicus hazard layers.</t>
+          <t>The main limitation is data currency. In particular, the underlying data has a Datenstand of October 2020, roughly six years old as of this review, and is a composite of several underlying sources (ABU, HORA, BWV/WLV Gefahrenzonenplaene) with potentially inconsistent vintages. Consequently, the source cannot be assumed to reflect flood-protection works or land-use changes made since 2020, unless cross-checked against more recent local information.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -9456,643 +9316,643 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is a transparent, replicable methodology covering nine physical hazards with an authoritative EU-level pedigree (ECB, n.d.). It is particularly useful as a methodological template for building an in-house classification approach. However, its suitability is reduced by the inaccessibility of the ECB's own underlying supervisory data to a non-significant institution. It is therefore best used as a methodological anchor rather than as a direct operational data source.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is combining several underlying Austrian flood sources into a single, harmonised layer with a standard OGC interface and no access restriction, unlike HORA (INSPIRE Geoportal Oesterreich, n.d.-b). It is particularly useful as the primary operational flood layer for populating data point 0050. However, its suitability is reduced somewhat by the dataset's data currency. It is therefore best used as the primary flood-hazard source, complemented by periodic currency checks.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available without registration (ECB, n.d.).</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the WFS endpoint (nz-core:HazardArea) with each coordinate, or download the GML/shapefile once and perform a local spatial join, assigning the returned flood-zone value to each exposure. The result is parcel/address-level. The process is fully automatable.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Not applicable via this source directly, since its output is aggregate/dashboard statistics rather than per-exposure data (ECB, n.d.). A per-exposure pipeline would instead need to replicate the ECB's published methodology using the bank's own AnaCredit-equivalent data plus JRC/Copernicus hazard layers.</t>
+          <t>The source is available under a CC BY 4.0 licence (INSPIRE Geoportal Oesterreich, n.d.-b). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ecb_physical_risk_indicators</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>The source is available under the ECB's standard open-data terms, free of charge and without registration (ECB, n.d.). No restrictions on commercial or systematic use beyond standard attribution practice were identified.</t>
+          <t>The Gefahrenzonenplan (GZP) is a public national hazard zoning dataset operated by the Forsttechnischer Dienst fuer Wildbach- und Lawinenverbauung (Federal Ministry BMLUK) (data.gv.at, n.d.-b). It provides a statutory hazard assessment for torrents, avalanches and mass-movement processes, covering these hazards at parcel/address-level granularity across Austria. The source is accessed through an OGC map service (WMS/WFS) and direct download, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>This is a national flood extent dataset, published via the INSPIRE Geoportal Oesterreich, with the Bundesministerium fuer Land- und Forstwirtschaft, Klima- und Umweltschutz, Regionen und Wasserwirtschaft (BMLUK) as data owner and Umweltbundesamt GmbH as technical operator (INSPIRE Geoportal Oesterreich, n.d.-b). It provides harmonised flood extent layers for the 30-, 100- and 300-year return periods, covering flood hazard at parcel/address-level granularity across Austria. The source is accessed through OGC WMS/WFS services and direct GML/shapefile download, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>The main limitation is that hazards are mapped only within areas of spatial relevance, meaning settled parts of a municipality with designated torrent or avalanche catchments (data.gv.at, n.d.-b). In particular, some zone plans remain available only in analogue form, and a portfolio location without a mapped result is ambiguous - it may indicate no hazard or simply no mapping. Consequently, the source cannot be used to conclusively rule out hazard for unmapped locations, unless cross-checked against the underlying zone-plan status.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is data currency. In particular, the underlying data has a Datenstand of October 2020, roughly six years old as of this review, and is a composite of several underlying sources (ABU, HORA, BWV/WLV Gefahrenzonenplaene) with potentially inconsistent vintages. Consequently, the source cannot be assumed to reflect flood-protection works or land-use changes made since 2020, unless cross-checked against more recent local information.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is being the strongest national source for mass-movement and torrent hazards, based on a statutory hazard assessment under the Forstgesetz (data.gv.at, n.d.-b). It is particularly useful for classifying torrent, avalanche and related mass-movement exposure at data point 0050. However, its suitability is reduced by incomplete settlement-area-only mapping and residual analogue-only zone plans. It is therefore best used as the primary source for these hazards, with unmapped locations flagged for manual review.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is combining several underlying Austrian flood sources into a single, harmonised layer with a standard OGC interface and no access restriction, unlike HORA (INSPIRE Geoportal Oesterreich, n.d.-b). It is particularly useful as the primary operational flood layer for populating data point 0050. However, its suitability is reduced somewhat by the dataset's data currency. It is therefore best used as the primary flood-hazard source, complemented by periodic currency checks.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the WMS/WFS endpoint (data.gv.at, n.d.-b) or download the shapefile/GeoPackage once and perform a local spatial join, assigning the returned zone value to each exposure. The result is parcel/address-level. The process is fully automatable.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>wlv_gefahrenzonenplan</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available under a CC BY 4.0 licence (INSPIRE Geoportal Oesterreich, n.d.-b).</t>
+          <t>The source is available as a High Value Dataset under Implementing Regulation (EU) 2023/138, free of charge with bulk download permitted via the WLV download service in ESRI shapefile format. The licence permits commercial use and systematic portfolio processing.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the WFS endpoint (nz-core:HazardArea) with each coordinate, or download the GML/shapefile once and perform a local spatial join, assigning the returned flood-zone value to each exposure. The result is parcel/address-level. The process is fully automatable.</t>
+          <t>HORA (Natural Hazard Overview and Risk Assessment Austria) is a publicly accessible Austrian WebGIS application, operated by the Land-, Forst- und Wasserwirtschaftliche Rechenzentrum (LFRZ) on behalf of the responsible federal ministry (LFRZ, n.d.). It provides address- and cadastral-level initial information on natural hazards, currently covering flood, earthquake, storm, hail and snow, at parcel/address-level granularity across Austria (HORA, n.d.). The source is accessed through an interactive web interface via individual location queries, and is free to use.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>hq_flood_extent</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>The source is available under a CC BY 4.0 licence (INSPIRE Geoportal Oesterreich, n.d.-b). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
+          <t>The main limitation is the restricted use of the service for systematic portfolio-level analysis (LFRZ, n.d.). In particular, the source is designed primarily for individual location queries and does not provide unrestricted bulk download or a documented portfolio-level API, and the displayed information is intended as initial risk information rather than a legally binding assessment. Consequently, HORA cannot be used as the sole source for automated classification of an entire loan portfolio, unless a separate access agreement is obtained from the operator.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>The Gefahrenzonenplan (GZP) is a public national hazard zoning dataset operated by the Forsttechnischer Dienst fuer Wildbach- und Lawinenverbauung (Federal Ministry BMLUK) (data.gv.at, n.d.-b). It provides a statutory hazard assessment for torrents, avalanches and mass-movement processes, covering these hazards at parcel/address-level granularity across Austria. The source is accessed through an OGC map service (WMS/WFS) and direct download, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>For an SNCI, HORA is conditionally suitable. Its main advantage is Austrian address-level coverage combined with simple web-based access (HORA, n.d.). It is particularly useful for individual exposure checks and plausibility assessments. However, its suitability is reduced by the restricted portfolio-level access and the non-binding nature of the displayed information. It is therefore best used as a supplementary validation source rather than as the sole operational source for populating data point 0050.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that hazards are mapped only within areas of spatial relevance, meaning settled parts of a municipality with designated torrent or avalanche catchments (data.gv.at, n.d.-b). In particular, some zone plans remain available only in analogue form, and a portfolio location without a mapped result is ambiguous - it may indicate no hazard or simply no mapping. Consequently, the source cannot be used to conclusively rule out hazard for unmapped locations, unless cross-checked against the underlying zone-plan status.</t>
+          <t>To apply HORA to a portfolio, the institution would need to geocode the relevant exposure addresses and query the corresponding locations individually through the web interface (HORA, n.d.), then record and link the resulting hazard information to each exposure. Because unrestricted bulk access and a documented portfolio-level API are not available, the process is not fully automatable and is unsuitable for systematic portfolio processing under current access conditions.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is being the strongest national source for mass-movement and torrent hazards, based on a statutory hazard assessment under the Forstgesetz (data.gv.at, n.d.-b). It is particularly useful for classifying torrent, avalanche and related mass-movement exposure at data point 0050. However, its suitability is reduced by incomplete settlement-area-only mapping and residual analogue-only zone plans. It is therefore best used as the primary source for these hazards, with unmapped locations flagged for manual review.</t>
+          <t>The source is subject to specific terms of use that restrict bulk download and automated access (LFRZ, n.d.); the service is intended for individual location queries only. A separate agreement with the operator would be required for systematic portfolio-level use or regulatory reporting purposes.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available under the High Value Dataset regime (data.gv.at, n.d.-b).</t>
+          <t>The Aqueduct Water Risk Atlas is a public water-risk dataset operated by the World Resources Institute (WRI) (WRI, n.d.). It provides 13 modelled indicators covering water stress, drought risk and riverine/coastal flood risk at sub-catchment (watershed) granularity globally (WRI, n.d.-b). The source is accessed through a web map portal, direct download and an API, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the WMS/WFS endpoint (data.gv.at, n.d.-b) or download the shapefile/GeoPackage once and perform a local spatial join, assigning the returned zone value to each exposure. The result is parcel/address-level. The process is fully automatable.</t>
+          <t>The main limitation is coarse granularity relative to Austria's parcel-level sources. In particular, the source resolves only to sub-catchment (watershed) level, so exposures within the same watershed share an identical value, and it is a global tool not locally calibrated or validated for Austria specifically. Consequently, the source cannot differentiate exposures within a geographically concentrated Austrian portfolio, unless combined with finer national sources for the acute hazards it also covers.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>wlv_gefahrenzonenplan</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>The source is available as a High Value Dataset under Implementing Regulation (EU) 2023/138, free of charge with bulk download permitted via the WLV download service in ESRI shapefile format. The licence permits commercial use and systematic portfolio processing.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is providing dedicated, named indicators for chronic water-related hazards (water stress, drought) otherwise underrepresented among Austrian sources. It is particularly useful as a supplementary chronic-risk layer. However, its suitability is reduced by watershed-level granularity, coarser than the parcel-level Austrian sources for acute hazards. It is therefore best used as a supplementary source for water stress and drought, not as a primary classification layer.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>HORA (Natural Hazard Overview and Risk Assessment Austria) is a publicly accessible Austrian WebGIS application, operated by the Land-, Forst- und Wasserwirtschaftliche Rechenzentrum (LFRZ) on behalf of the responsible federal ministry (LFRZ, n.d.). It provides address- and cadastral-level initial information on natural hazards, currently covering flood, earthquake, storm, hail and snow, at parcel/address-level granularity across Austria (HORA, n.d.). The source is accessed through an interactive web interface via individual location queries, and is free to use. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then download the watershed-level dataset or query the API and perform a spatial join to the relevant watershed polygon, assigning the watershed's indicator value to each exposure. The result is sub-catchment (watershed) level. The process is fully automatable.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is the restricted use of the service for systematic portfolio-level analysis (LFRZ, n.d.). In particular, the source is designed primarily for individual location queries and does not provide unrestricted bulk download or a documented portfolio-level API, and the displayed information is intended as initial risk information rather than a legally binding assessment. Consequently, HORA cannot be used as the sole source for automated classification of an entire loan portfolio, unless a separate access agreement is obtained from the operator.</t>
+          <t>The source is described by the operator as free and openly accessible for any application, with attribution requested (WRI, n.d.). No formally stated open licence name was identified on the operator's own materials, and no commercial-use restriction was found.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, HORA is conditionally suitable. Its main advantage is Austrian address-level coverage combined with simple web-based access (HORA, n.d.). It is particularly useful for individual exposure checks and plausibility assessments. However, its suitability is reduced by the restricted portfolio-level access and the non-binding nature of the displayed information. It is therefore best used as a supplementary validation source rather than as the sole operational source for populating data point 0050.</t>
+          <t>This is a commercial dataset operated by Moody's ESG Solutions (Moody's, n.d.). It provides proprietary modelled physical climate risk scores covering floods, heat stress, hurricanes and typhoons, sea-level rise, water stress and wildfires at facility/object-level granularity globally (Moody's, n.d.-b). The source is accessed through a commercial analytics platform and an API, and is paid.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge for individual queries. A separate agreement with the operator (LFRZ) would be required for portfolio-level or bulk use.</t>
+          <t>The main limitation is that confirmed Austria-relevant coverage is narrower than the product's general marketing suggests (Moody's, n.d.-b). In particular, storm is modelled as tropical cyclones specifically, which does not affect Austria, and a distinct heat-wave product plus drought coverage could not be confirmed at all. Consequently, the source cannot be relied upon for storm, heat-wave or drought classification of Austrian exposures, unless the operator confirms specific coverage directly.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>To apply HORA to a portfolio, the institution would need to geocode the relevant exposure addresses and query the corresponding locations individually through the web interface (HORA, n.d.), then record and link the resulting hazard information to each exposure. Because unrestricted bulk access and a documented portfolio-level API are not available, the process is not fully automatable and is unsuitable for systematic portfolio processing under current access conditions.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is ready-made, high-granularity facility-level risk scores integrable via API with low processing effort (Moody's, n.d.). It is particularly useful for flood, heat stress, water stress and wildfire classification. However, its suitability is reduced by a commercial cost structure typically designed for larger institutions and by narrower-than-marketed Austria-relevant hazard coverage. It is therefore best used as a primary source only for the confirmed hazards, subject to cost negotiation appropriate to SNCI scale.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>pricing</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>The source is subject to specific terms of use that restrict bulk download and automated access (LFRZ, n.d.); the service is intended for individual location queries only. A separate agreement with the operator would be required for systematic portfolio-level use or regulatory reporting purposes.</t>
+          <t>Pricing is not publicly disclosed. Access is provided through a commercial analytics platform and API under a quote-based licence agreement (Moody's, n.d.). No product-specific price indication was identified; publicly available estimates for other Moody's products should therefore not be used as a proxy. The price information should be treated as not independently verified.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>The Aqueduct Water Risk Atlas is a public water-risk dataset operated by the World Resources Institute (WRI) (WRI, n.d.). It provides 13 modelled indicators covering water stress, drought risk and riverine/coastal flood risk at sub-catchment (watershed) granularity globally (WRI, n.d.-b). The source is accessed through a web map portal, direct download and an API, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source.</t>
+          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the API (Moody's, n.d.) and receive a facility-level risk score directly. No further spatial processing is required. The process is fully automatable for institutions with API access.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is coarse granularity relative to Austria's parcel-level sources. In particular, the source resolves only to sub-catchment (watershed) level, so exposures within the same watershed share an identical value, and it is a global tool not locally calibrated or validated for Austria specifically. Consequently, the source cannot differentiate exposures within a geographically concentrated Austrian portfolio, unless combined with finer national sources for the acute hazards it also covers.</t>
+          <t>The source is subject to a commercial licence agreement (Moody's, n.d.). Access terms, API scope and portfolio size limits depend on the specific subscription negotiated with Moody's. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is providing dedicated, named indicators for chronic water-related hazards (water stress, drought) otherwise underrepresented among Austrian sources. It is particularly useful as a supplementary chronic-risk layer. However, its suitability is reduced by watershed-level granularity, coarser than the parcel-level Austrian sources for acute hazards. It is therefore best used as a supplementary source for water stress and drought, not as a primary classification layer.</t>
+          <t>NATHAN Risk Suite is a commercial dataset operated by Munich Re (Munich Re, n.d.). It provides proprietary modelled natural hazard and climate scenario scores covering 15 hazards, including river flood, extratropical storm, wildfire and landslide, at facility/object-level granularity globally, with scenarios extending to 2100 (Munich Re, n.d.-b). The source is accessed through a commercial analytics platform and an API, and is paid.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available without registration (WRI, n.d.).</t>
+          <t>The main limitation is that heat, drought and water stress coverage could not be confirmed by name (Munich Re, n.d.-b). In particular, these hazards are only advertised via a separate, unnamed 'Climate Change Edition' covering '13 climate hazards' without individual naming in the materials reviewed. Consequently, the source cannot be relied upon for heat, drought or water stress classification with the same confidence as its 15 named Natural Hazards Edition hazards, unless the operator confirms specific coverage directly.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then download the watershed-level dataset or query the API and perform a spatial join to the relevant watershed polygon, assigning the watershed's indicator value to each exposure. The result is sub-catchment (watershed) level. The process is fully automatable.</t>
+          <t>For an SNCI, the source is suitable for its confirmed hazards. Its main advantage is very extensive scenario depth (to 2100) and ready-made facility-level scores for 15 explicitly named hazards, including landslide and extratropical storm. It is particularly useful for portfolio-scale exposure scoring via API. However, its suitability is reduced by pricing typically geared towards larger institutions and reinsurers, and by unconfirmed heat/drought/water-stress coverage. It is therefore best used as a primary source for the confirmed hazards, or via the accessible pay-per-location On-Demand option for smaller-scale use.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>pricing</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>The source is described by the operator as free and openly accessible for any application, with attribution requested (WRI, n.d.). No formally stated open licence name was identified on the operator's own materials, and no commercial-use restriction was found.</t>
+          <t>Pricing follows two distinct access models (Munich Re, n.d.-c). The On-Demand service uses pay-per-location pricing, with publicly displayed prices ranging from approximately EUR 100 to EUR 160 per location depending on package size. Portfolio-scale access through the Natural Hazards Edition or Climate Change Edition is subscription-based and quote-based, with API access available in the relevant business tiers. The publicly displayed On-Demand prices are not directly comparable with portfolio subscription costs.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>This is a commercial dataset operated by Moody's ESG Solutions (Moody's, n.d.). It provides proprietary modelled physical climate risk scores covering floods, heat stress, hurricanes and typhoons, sea-level rise, water stress and wildfires at facility/object-level granularity globally (Moody's, n.d.-b). The source is accessed through a commercial analytics platform and an API, and is paid. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the API (Munich Re, n.d.) and receive a facility-level risk score directly. No further spatial processing is required. The process is fully automatable for institutions with API/subscription access.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that confirmed Austria-relevant coverage is narrower than the product's general marketing suggests (Moody's, n.d.-b). In particular, storm is modelled as tropical cyclones specifically, which does not affect Austria, and a distinct heat-wave product plus drought coverage could not be confirmed at all. Consequently, the source cannot be relied upon for storm, heat-wave or drought classification of Austrian exposures, unless the operator confirms specific coverage directly.</t>
+          <t>The source is subject to a commercial licence agreement. The On-Demand service requires no subscription and is billed per location; portfolio-scale subscription tiers (Natural Hazards Edition, Climate Change Edition) determine API access and portfolio size limits. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is ready-made, high-granularity facility-level risk scores integrable via API with low processing effort (Moody's, n.d.). It is particularly useful for flood, heat stress, water stress and wildfire classification. However, its suitability is reduced by a commercial cost structure typically designed for larger institutions and by narrower-than-marketed Austria-relevant hazard coverage. It is therefore best used as a primary source only for the confirmed hazards, subject to cost negotiation appropriate to SNCI scale.</t>
+          <t>This is a public dataset collection operated by the World Bank Group in cooperation with GFDRR (World Bank/GFDRR, n.d.), comprising the Risk Data Library (downloadable hazard datasets) and the ThinkHazard! screening tool. It provides flood, landslide, wildfire, extreme-heat and water-scarcity hazard information at district (ADM2) to dataset-dependent granularity, with a development-country focus (GFDRR, n.d.). The source is accessed through a web portal, direct download and an API, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>Pricing is not publicly disclosed. Access is provided through a commercial analytics platform and API under a quote-based licence agreement (Moody's, n.d.). No product-specific price indication was identified; publicly available estimates for other Moody's products should therefore not be used as a proxy. The price information should be treated as not independently verified.</t>
+          <t>The main limitation is granularity that is not uniform across the source. In particular, ThinkHazard! resolves only to district (ADM2) level, while Risk Data Library datasets vary individually in resolution, and storm coverage via ThinkHazard!'s 'cyclone' hazard model is tropical-cyclone-oriented with unconfirmed applicability to Austria. Consequently, the source cannot differentiate exposures within a single Austrian district, unless combined with finer national sources.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the API (Moody's, n.d.) and receive a facility-level risk score directly. No further spatial processing is required. The process is fully automatable for institutions with API access.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is confirmed, commonly-available probabilistic coverage for flood, landslide, extreme heat, water scarcity and wildfire, accessible free via API (GFDRR, n.d.). It is particularly useful for plausibility checks and district-level screening. However, its suitability is reduced by district-level, not parcel-level, granularity. It is therefore best used as a supplementary or validation source rather than as the primary operational layer.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>moodys_physical_risk</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>The source is subject to a commercial licence agreement (Moody's, n.d.). Access terms, API scope and portfolio size limits depend on the specific subscription negotiated with Moody's. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then determine the ADM2 (district) administrative unit for each coordinate and query the ThinkHazard! API for the hazard level of that district, or download the relevant Risk Data Library dataset for gridded hazards and perform a spatial join, assigning the resulting value to each exposure. The result is district-level. The process is fully automatable, though district-level resolution limits differentiation.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>NATHAN Risk Suite is a commercial dataset operated by Munich Re (Munich Re, n.d.). It provides proprietary modelled natural hazard and climate scenario scores covering 15 hazards, including river flood, extratropical storm, wildfire and landslide, at facility/object-level granularity globally, with scenarios extending to 2100 (Munich Re, n.d.-b). The source is accessed through a commercial analytics platform and an API, and is paid. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>The source is available under the World Bank's open-data terms, free of charge and without registration (World Bank/GFDRR, n.d.). No restrictions on commercial or systematic use beyond standard attribution practice were identified.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that heat, drought and water stress coverage could not be confirmed by name (Munich Re, n.d.-b). In particular, these hazards are only advertised via a separate, unnamed 'Climate Change Edition' covering '13 climate hazards' without individual naming in the materials reviewed. Consequently, the source cannot be relied upon for heat, drought or water stress classification with the same confidence as its 15 named Natural Hazards Edition hazards, unless the operator confirms specific coverage directly.</t>
+          <t>KryoMon.AT is a publicly funded research consortium coordinated by the University of Graz, involving multiple Austrian universities, the Austrian and Bavarian Academies of Sciences, GeoSphere Austria and several associations (KryoMon.AT, n.d.; ORF Steiermark, 2026). It provides periodic reports on permafrost, glacier and snow trends covering permafrost hazard at station-based granularity across selected Austrian alpine sites (KryoMon.AT, n.d.). The source is accessed through a reports/publications website with PDF downloads, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable for its confirmed hazards. Its main advantage is very extensive scenario depth (to 2100) and ready-made facility-level scores for 15 explicitly named hazards, including landslide and extratropical storm. It is particularly useful for portfolio-scale exposure scoring via API. However, its suitability is reduced by pricing typically geared towards larger institutions and reinsurers, and by unconfirmed heat/drought/water-stress coverage. It is therefore best used as a primary source for the confirmed hazards, or via the accessible pay-per-location On-Demand option for smaller-scale use.</t>
+          <t>The main limitation is that the information exists only as narrative PDF reports, not as structured per-location data (KryoMon.AT, n.d.). In particular, coverage is station-/object-based rather than a nationwide spatial hazard layer. Consequently, the source cannot be overlaid with individual portfolio locations, unless the bank undertakes manual, qualitative interpretation per region.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>Pricing follows two distinct access models (Munich Re, n.d.-c). The On-Demand service uses pay-per-location pricing, with publicly displayed prices ranging from approximately EUR 100 to EUR 160 per location depending on package size. Portfolio-scale access through the Natural Hazards Edition or Climate Change Edition is subscription-based and quote-based, with API access available in the relevant business tiers. The publicly displayed On-Demand prices are not directly comparable with portfolio subscription costs.</t>
+          <t>For an SNCI, the source is not suitable for systematic classification. Its main advantage is being the best available current context on Austrian permafrost trends, produced by an authoritative multi-institutional research consortium (KryoMon.AT, n.d.; ORF Steiermark, 2026). It is particularly useful for background discussion and methodological context in the reporting narrative. However, its suitability is reduced by the complete absence of structured, location-specific data. It is therefore best used purely as a context source, not as an operational data source.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -10102,14 +9962,14 @@
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the API (Munich Re, n.d.) and receive a facility-level risk score directly. No further spatial processing is required. The process is fully automatable for institutions with API/subscription access.</t>
+          <t>Not applicable: the information exists only in narrative PDF reports (KryoMon.AT, n.d.), not as structured per-location data, so no automatable pipeline can be built against it. At best, a qualitative note per region could be manually derived.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>munich_re_nathan</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -10119,14 +9979,14 @@
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>The source is subject to a commercial licence agreement. The On-Demand service requires no subscription and is billed per location; portfolio-scale subscription tiers (Natural Hazards Edition, Climate Change Edition) determine API access and portfolio size limits. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
+          <t>The source is available under the reporting consortium's general open-access publication terms, free of charge, with attribution expected per standard academic practice (KryoMon.AT, n.d.). No commercial-use restriction was identified.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -10136,14 +9996,14 @@
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>This is a public dataset collection operated by the World Bank Group in cooperation with GFDRR (World Bank/GFDRR, n.d.), comprising the Risk Data Library (downloadable hazard datasets) and the ThinkHazard! screening tool. It provides flood, landslide, wildfire, extreme-heat and water-scarcity hazard information at district (ADM2) to dataset-dependent granularity, with a development-country focus (GFDRR, n.d.). The source is accessed through a web portal, direct download and an API, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a secondary source.</t>
+          <t>This is a public register operated by Statistik Austria (Statistik Austria, n.d.). It provides the official OeNACE 2025 (NACE Rev. 2.1) economic-activity code for each Austrian company, keyed to the Firmenbuch number, covering the full national company register at entity-level granularity. The source is accessed through direct bulk download in CSV format, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -10153,14 +10013,14 @@
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is granularity that is not uniform across the source. In particular, ThinkHazard! resolves only to district (ADM2) level, while Risk Data Library datasets vary individually in resolution, and storm coverage via ThinkHazard!'s 'cyclone' hazard model is tropical-cyclone-oriented with unconfirmed applicability to Austria. Consequently, the source cannot differentiate exposures within a single Austrian district, unless combined with finer national sources.</t>
+          <t>The main limitation is incomplete company coverage (Statistik Austria, n.d.). In particular, companies without an assigned OeNACE code remain unmatched, and unregistered sole traders are out of scope of the Firmenbuch-based register. Consequently, the source cannot classify every possible counterparty in an SNCI's loan portfolio, unless a complementary source is used for the unmatched residual.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -10170,738 +10030,738 @@
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is confirmed, commonly-available probabilistic coverage for flood, landslide, extreme heat, water scarcity and wildfire, accessible free via API (GFDRR, n.d.). It is particularly useful for plausibility checks and district-level screening. However, its suitability is reduced by district-level, not parcel-level, granularity. It is therefore best used as a supplementary or validation source rather than as the primary operational layer.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is being simultaneously official, freely accessible in bulk and directly joinable to a loan portfolio via the Firmenbuchnummer (Statistik Austria, n.d.). It is particularly useful as the primary operational source for populating the NACE subsector dimension. However, its suitability is reduced slightly by unmatched companies and out-of-scope sole traders. It is therefore best used as the primary transition-risk classification source, complemented by Wirtschafts-Compass where an existing licence is operationally simpler.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available without registration (World Bank/GFDRR, n.d.).</t>
+          <t>To apply the source to a portfolio, the institution can bulk-download the CSV file (Statistik Austria, n.d.) and join it directly to its internal exposure data using the Firmenbuchnummer, then transform the assigned OeNACE code to the required 4-digit reporting granularity. The result is entity-level. The process is fully automatable and does not require geocoding or spatial processing.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>hvd_fbnr_oenace</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then determine the ADM2 (district) administrative unit for each coordinate and query the ThinkHazard! API for the hazard level of that district, or download the relevant Risk Data Library dataset for gridded hazards and perform a spatial join, assigning the resulting value to each exposure. The result is district-level. The process is fully automatable, though district-level resolution limits differentiation.</t>
+          <t>The source is available under a CC BY 4.0 licence, published as a High Value Dataset under Implementing Regulation (EU) 2023/138. Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>The source is available under the World Bank's open-data terms, free of charge and without registration (World Bank/GFDRR, n.d.). No restrictions on commercial or systematic use beyond standard attribution practice were identified.</t>
+          <t>Wirtschafts-Compass is a commercial Austrian company-data service operated by Compass-Verlag GmbH (Compass-Verlag, n.d.). It provides an editorially enriched OeNACE classification per entity, covering the Austrian company landscape at entity-level granularity, delivered with daily currency. The source is accessed through an API and a web portal, and is paid.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>KryoMon.AT is a publicly funded research consortium coordinated by the University of Graz, involving multiple Austrian universities, the Austrian and Bavarian Academies of Sciences, GeoSphere Austria and several associations (KryoMon.AT, n.d.; ORF Steiermark, 2026). It provides periodic reports on permafrost, glacier and snow trends covering permafrost hazard at station-based granularity across selected Austrian alpine sites (KryoMon.AT, n.d.). The source is accessed through a reports/publications website with PDF downloads, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a context-only source.</t>
+          <t>The main limitation is that the classification is editorially enriched rather than the official statistical assignment (Compass-Verlag, n.d.). In particular, cost is institution-dependent, since some banks may already hold a sector licence while others would face a new subscription cost. Consequently, the source cannot be treated as an authoritative regulatory reference on the same footing as the official HVD dataset, unless used alongside HVD for cross-validation.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that the information exists only as narrative PDF reports, not as structured per-location data (KryoMon.AT, n.d.). In particular, coverage is station-/object-based rather than a nationwide spatial hazard layer. Consequently, the source cannot be overlaid with individual portfolio locations, unless the bank undertakes manual, qualitative interpretation per region.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is being directly usable, daily-updated and API-accessible, with existing institutional access reported in parts of the Austrian banking sector (Compass-Verlag, n.d.-b). It is particularly useful where an existing licence makes a single query operationally simpler than a bulk HVD join. However, its suitability is reduced by cost for institutions without an existing licence and by its non-official classification status. It is therefore best used as a primary operational source alongside the free HVD dataset.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>pricing</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is not suitable for systematic classification. Its main advantage is being the best available current context on Austrian permafrost trends, produced by an authoritative multi-institutional research consortium (KryoMon.AT, n.d.; ORF Steiermark, 2026). It is particularly useful for background discussion and methodological context in the reporting narrative. However, its suitability is reduced by the complete absence of structured, location-specific data. It is therefore best used purely as a context source, not as an operational data source.</t>
+          <t>Pricing is publicly disclosed for standard access: pay-per-query, from EUR 6 (excl. VAT) per quarter for up to 10 queries via the WKO-member service, or from EUR 24 per year for individual/basic access (Compass-Verlag, n.d.-c; Compass-Verlag, n.d.-d). Institutional/enterprise API pricing is not publicly listed and should be confirmed directly with the provider.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available without registration (KryoMon.AT, n.d.).</t>
+          <t>To apply the source to a portfolio, the institution would send the Firmenbuchnummer or company identifier to the API (Compass-Verlag, n.d.) and receive the OeNACE classification directly. No further processing is required. The process is fully automatable for institutions with API access.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Not applicable: the information exists only in narrative PDF reports (KryoMon.AT, n.d.), not as structured per-location data, so no automatable pipeline can be built against it. At best, a qualitative note per region could be manually derived.</t>
+          <t>The source is subject to a commercial licence agreement (Compass-Verlag, n.d.-c). Standard access is pay-per-query with published pricing; institutional API access terms depend on the specific subscription. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>The source is available under the reporting consortium's general open-access publication terms, free of charge, with attribution expected per standard academic practice (KryoMon.AT, n.d.). No commercial-use restriction was identified.</t>
+          <t>SPARTACUS-v3 is a public gridded climate dataset operated by GeoSphere Austria, the Austrian federal institute for geology, geophysics, climatology and meteorology (GeoSphere Austria, n.d.-a). It provides observed daily, monthly and quarterly temperature, precipitation and sunshine-duration fields, covering heat and precipitation hazards at 1km grid granularity across Austria since 1961 (GeoSphere Austria, n.d.-a). The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>This is a public register operated by Statistik Austria (Statistik Austria, n.d.). It provides the official OeNACE 2025 (NACE Rev. 2.1) economic-activity code for each Austrian company, keyed to the Firmenbuch number, covering the full national company register at entity-level granularity. The source is accessed through direct bulk download in CSV format, and is free of charge. In the context of Template D 01.01, it is relevant to the NACE subsector dimension as a primary source.</t>
+          <t>The main limitation is that the source provides raw climate variables, not a pre-classified hazard or risk score (GeoSphere Austria, n.d.-a). In particular, converting temperature or precipitation fields into a heat-wave or heavy-precipitation exposure indicator requires the institution's own threshold definition. Consequently, the source cannot be used directly for exposure classification, unless the bank first defines and validates its own index methodology.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is incomplete company coverage (Statistik Austria, n.d.). In particular, companies without an assigned OeNACE code remain unmatched, and unregistered sole traders are out of scope of the Firmenbuch-based register. Consequently, the source cannot classify every possible counterparty in an SNCI's loan portfolio, unless a complementary source is used for the unmatched residual.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is Austria's highest-resolution national gridded observation dataset, finer than Copernicus CDS, with a coordinate-based API enabling direct point queries (GeoSphere Austria, n.d.-a). It is particularly useful as the primary raw-data foundation for heat and heavy-precipitation indices tailored to Austrian conditions. However, its suitability is reduced by the own-methodology effort required to convert raw variables into a hazard indicator. It is therefore best used as a primary source for institutions willing to define their own threshold-based indices.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is being simultaneously official, freely accessible in bulk and directly joinable to a loan portfolio via the Firmenbuchnummer (Statistik Austria, n.d.). It is particularly useful as the primary operational source for populating the NACE subsector dimension. However, its suitability is reduced slightly by unmatched companies and out-of-scope sole traders. It is therefore best used as the primary transition-risk classification source, complemented by Wirtschafts-Compass where an existing licence is operationally simpler.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the GeoSphere Austria grid API with the coordinates for the relevant variable and apply a chosen threshold definition, assigning the resulting indicator to each exposure. The result is grid-level (1km). The process is fully automatable once the threshold methodology is defined.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available under a CC BY 4.0 licence, published as a High Value Dataset under Implementing Regulation (EU) 2023/138.</t>
+          <t>The source is available under the Creative Commons Public Domain Dedication (CC0 1.0), per GeoSphere Austria's own repository documentation, free for any use including commercial. No attribution is legally required, though it is good practice. The licence permits systematic portfolio processing.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution can bulk-download the CSV file (Statistik Austria, n.d.) and join it directly to its internal exposure data using the Firmenbuchnummer, then transform the assigned OeNACE code to the required 4-digit reporting granularity. The result is entity-level. The process is fully automatable and does not require geocoding or spatial processing.</t>
+          <t>WINFORE is a public gridded drought-index dataset operated by GeoSphere Austria (GeoSphere Austria, n.d.-b). It provides the Standardized Precipitation Evapotranspiration Index (SPEI) at 30-, 90- and 365-day aggregation, covering drought hazard at 1km grid granularity across Austria, derived from SPARTACUS temperature and precipitation fields. The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>hvd_fbnr_oenace</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>The source is available under a CC BY 4.0 licence, published as a High Value Dataset under Implementing Regulation (EU) 2023/138. Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
+          <t>The main limitation is that SPEI is a standardised statistical anomaly index, not an absolute water-deficit value (GeoSphere Austria, n.d.-b). In particular, it is derived via a normal-distribution transform over two climate reference periods, so its interpretation requires understanding this transform rather than reading a direct precipitation deficit. Consequently, the source cannot be interpreted at face value without methodological context, unless the reporting institution documents the SPEI transform in its own methodology notes.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>Wirtschafts-Compass is a commercial Austrian company-data service operated by Compass-Verlag GmbH (Compass-Verlag, n.d.). It provides an editorially enriched OeNACE classification per entity, covering the Austrian company landscape at entity-level granularity, delivered with daily currency. The source is accessed through an API and a web portal, and is paid. In the context of Template D 01.01, it is relevant to the NACE subsector dimension as a primary source.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is being a dedicated, purpose-built national drought index at fine (1km) resolution, filling a gap not covered by any other Austrian source in this matrix. It is particularly useful as the primary drought-classification source for data point 0050. However, its suitability is reduced somewhat by the need to correctly interpret the standardised anomaly value. It is therefore best used as the primary drought source, with a brief methodology note on SPEI interpretation.</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that the classification is editorially enriched rather than the official statistical assignment (Compass-Verlag, n.d.). In particular, cost is institution-dependent, since some banks may already hold a sector licence while others would face a new subscription cost. Consequently, the source cannot be treated as an authoritative regulatory reference on the same footing as the official HVD dataset, unless used alongside HVD for cross-validation.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the GeoSphere Austria grid API with the coordinates for the WINFORE SPEI variable at the desired aggregation window, assigning the returned value to each exposure. The result is grid-level (1km). The process is fully automatable.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is being directly usable, daily-updated and API-accessible, with existing institutional access reported in parts of the Austrian banking sector (Compass-Verlag, n.d.-b). It is particularly useful where an existing licence makes a single query operationally simpler than a bulk HVD join. However, its suitability is reduced by cost for institutions without an existing licence and by its non-official classification status. It is therefore best used as a primary operational source alongside the free HVD dataset.</t>
+          <t>The source is available under the Creative Commons Public Domain Dedication (CC0 1.0), per GeoSphere Austria's own repository documentation, free for any use including commercial. No attribution is legally required, though it is good practice.</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>Pricing is publicly disclosed for standard access: pay-per-query, from EUR 6 (excl. VAT) per quarter for up to 10 queries via the WKO-member service, or from EUR 24 per year for individual/basic access (Compass-Verlag, n.d.-c; Compass-Verlag, n.d.-d). Institutional/enterprise API pricing is not publicly listed and should be confirmed directly with the provider.</t>
+          <t>Spectra is a commercial physical climate risk platform operated by Climate X Ltd, a UK-based company founded in 2020 (Technology Tools, n.d.). It provides asset-level modelled physical hazard scores and financial loss projections across up to 16 hazards, including flooding, storms, heat stress, wildfires and landslides, at asset/facility-level granularity globally, with scenario projections to 2100 (Repath, n.d.). The source is accessed through a commercial SaaS platform and an API, and is paid.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution would send the Firmenbuchnummer or company identifier to the API (Compass-Verlag, n.d.) and receive the OeNACE classification directly. No further processing is required. The process is fully automatable for institutions with API access.</t>
+          <t>The main limitation is that pricing and the full hazard list are not published by the operator directly (Net Zero Compare, n.d.). In particular, only third-party estimates of cost are available, not operator-confirmed figures. Consequently, the source's exact scope and cost cannot be independently verified from public information, unless confirmed directly with Climate X.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>wirtschafts_compass</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>The source is subject to a commercial licence agreement (Compass-Verlag, n.d.-c). Standard access is pay-per-query with published pricing; institutional API access terms depend on the specific subscription. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is ready-made, high-granularity asset-level scores integrable via API for a broad set of confirmed hazards (Repath, n.d.; Net Zero Compare, n.d.). It is particularly useful for flood, storm, heat stress, wildfire and landslide classification. However, its suitability is reduced by unconfirmed pricing and enterprise-SaaS positioning that may exceed a typical SNCI's budget. It is therefore best used as a primary source subject to direct price confirmation appropriate to SNCI scale.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>pricing</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>SPARTACUS-v3 is a public gridded climate dataset operated by GeoSphere Austria, the Austrian federal institute for geology, geophysics, climatology and meteorology (GeoSphere Austria, n.d.-a). It provides observed daily, monthly and quarterly temperature, precipitation and sunshine-duration fields, covering heat and precipitation hazards at 1km grid granularity across Austria since 1961 (GeoSphere Austria, n.d.-a). The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>Pricing is not publicly disclosed by Climate X directly. Access is provided through a commercial SaaS platform and API under a quote-based licence agreement. Third-party industry comparison sources estimate EUR 20,000-60,000 per year for portfolios of 30-100 assets, described as 'mid-market' pricing (Repath, n.d.). The price information should be treated as indicative and not independently verified.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that the source provides raw climate variables, not a pre-classified hazard or risk score (GeoSphere Austria, n.d.-a). In particular, converting temperature or precipitation fields into a heat-wave or heavy-precipitation exposure indicator requires the institution's own threshold definition. Consequently, the source cannot be used directly for exposure classification, unless the bank first defines and validates its own index methodology.</t>
+          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the Spectra API (Climate X, n.d.) and receive an asset-level hazard/financial-loss score directly. No further spatial processing is required. The process is fully automatable for institutions with API access.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is Austria's highest-resolution national gridded observation dataset, finer than Copernicus CDS, with a coordinate-based API enabling direct point queries (GeoSphere Austria, n.d.-a). It is particularly useful as the primary raw-data foundation for heat and heavy-precipitation indices tailored to Austrian conditions. However, its suitability is reduced by the own-methodology effort required to convert raw variables into a hazard indicator. It is therefore best used as a primary source for institutions willing to define their own threshold-based indices.</t>
+          <t>The source is subject to a commercial licence agreement, quote-based, with no public price list (Net Zero Compare, n.d.). Access terms and portfolio size limits depend on the specific subscription negotiated. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available without registration (GeoSphere Austria/re3data, n.d.).</t>
+          <t>ClimateScore Global is a commercial physical climate risk platform operated by Jupiter Intelligence, Inc., a US company founded in 2017 (aigreentools.com, n.d.). It provides asset-level modelled physical hazard scores and finance-grade loss metrics across 9 physical perils, including flood, heat, drought, tropical cyclones and wildfire, at asset/facility-level granularity globally, based on peer-reviewed CMIP6/ERA5 science (aigreentools.com, n.d.). The source is accessed through a commercial SaaS platform and an API, and is paid.</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the GeoSphere Austria grid API with the coordinates for the relevant variable and apply a chosen threshold definition, assigning the resulting indicator to each exposure. The result is grid-level (1km). The process is fully automatable once the threshold methodology is defined.</t>
+          <t>The main limitation is enterprise-tier, quote-based pricing not publicly listed (Mitiga Solutions, n.d.). In particular, the platform's scientific and financial-metric depth is designed for enterprise-scale deployments across banks, insurers and asset managers. Consequently, the source cannot be assumed affordable for an SNCI without direct confirmation, unless a limited-scope engagement at the lower end of the stated price range is negotiated.</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>geosphere_spartacus</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>The source is available under the Creative Commons Public Domain Dedication (CC0 1.0), per GeoSphere Austria's own repository documentation, free for any use including commercial. No attribution is legally required, though it is good practice. The licence permits systematic portfolio processing.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is extensive, scientifically validated hazard and financial-metric coverage across 9 peer-reviewed perils (aigreentools.com, n.d.). It is particularly useful for institutions needing finance-grade physical risk metrics beyond simple hazard scores. However, its suitability is reduced by enterprise-tier pricing likely above a typical SNCI's budget for full portfolio deployment. It is therefore best used as a primary source for a limited scope, subject to direct price negotiation.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>pricing</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>WINFORE is a public gridded drought-index dataset operated by GeoSphere Austria (GeoSphere Austria, n.d.-b). It provides the Standardized Precipitation Evapotranspiration Index (SPEI) at 30-, 90- and 365-day aggregation, covering drought hazard at 1km grid granularity across Austria, derived from SPARTACUS temperature and precipitation fields. The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>Pricing is not publicly disclosed as a fixed list, but is quote-based. Jupiter's own CEO stated in a 2022 interview that 'subscription pricing ranges from $25,000 to multimillion-dollar contracts' depending on scope (Trellis/Clancy, 2022). Full portfolio deployments are typically six-figure annual commitments per third-party sources (Repath, n.d.). The price information should be treated as indicative, based on the operator's own public statement.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that SPEI is a standardised statistical anomaly index, not an absolute water-deficit value (GeoSphere Austria, n.d.-b). In particular, it is derived via a normal-distribution transform over two climate reference periods, so its interpretation requires understanding this transform rather than reading a direct precipitation deficit. Consequently, the source cannot be interpreted at face value without methodological context, unless the reporting institution documents the SPEI transform in its own methodology notes.</t>
+          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the ClimateScore Global API (Jupiter Intelligence, n.d.) and receive an asset-level hazard/financial-loss score directly. No further spatial processing is required. The process is fully automatable for institutions with API access.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>jupiter_intelligence</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is being a dedicated, purpose-built national drought index at fine (1km) resolution, filling a gap not covered by any other Austrian source in this matrix. It is particularly useful as the primary drought-classification source for data point 0050. However, its suitability is reduced somewhat by the need to correctly interpret the standardised anomaly value. It is therefore best used as the primary drought source, with a brief methodology note on SPEI interpretation.</t>
+          <t>The source is subject to a commercial licence agreement, quote-based and defined case-by-case with the client (Mitiga Solutions, n.d.). Access terms and portfolio size limits depend on the specific subscription negotiated. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>abstract</t>
         </is>
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge and available without registration (GeoSphere Austria/re3data, n.d.).</t>
+          <t>This is a set of standalone, ready-made physical hazard indicator products, published as individual datasets on the Copernicus Climate Data Store (CDS), distinct from the general-purpose raw climate variables covered by the separate copernicus_cds entry (ECMWF, n.d.). It provides ERA5-HEAT (UTCI/heat stress) and the SMHI hydrology dataset (flood, water stress/aridity, soil-moisture drought), covering these four hazards at grid granularity across Europe (Di Napoli et al., 2021; SMHI/C3S, n.d.). The source is accessed through direct download and a queryable API, and is free of charge.</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>limitations</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the GeoSphere Austria grid API with the coordinates for the WINFORE SPEI variable at the desired aggregation window, assigning the returned value to each exposure. The result is grid-level (1km). The process is fully automatable.</t>
+          <t>The main limitation is that meteorological (SPI-3) drought and the temperature/precipitation/wind-based ECDE indices (heat wave, heavy precipitation, storm) remain accessible only via raw copernicus_cds variables or the Climate-ADAPT-curated bundle, not as a standalone product under this entry. Consequently, a bank needing those specific indices cannot rely on this entry alone, unless it also consults copernicus_cds or eea_climate_adapt for them.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>geosphere_winfore_spei</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>suitability_snci</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>The source is available under the Creative Commons Public Domain Dedication (CC0 1.0), per GeoSphere Austria's own repository documentation, free for any use including commercial. No attribution is legally required, though it is good practice.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is that each product is a purpose-built, documented hazard indicator with no own index-definition effort required, unlike raw Copernicus CDS variables (Di Napoli et al., 2021; SMHI/C3S, n.d.). It is particularly useful for heat stress, flood, water stress and soil-moisture drought classification at low processing effort. However, its suitability is reduced by its narrower hazard breadth compared with the full CDS catalogue. It is therefore best used as a primary source for its four covered hazards, complemented by other sources for the remainder.</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>portfolio_pipeline</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>Spectra is a commercial physical climate risk platform operated by Climate X Ltd, a UK-based company founded in 2020 (Technology Tools, n.d.). It provides asset-level modelled physical hazard scores and financial loss projections across up to 16 hazards, including flooding, storms, heat stress, wildfires and landslides, at asset/facility-level granularity globally, with scenario projections to 2100 (Repath, n.d.). The source is accessed through a commercial SaaS platform and an API, and is paid. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query or download the relevant standalone product (ERA5-HEAT for heat stress, SMHI hydrology for flood/water stress/soil-moisture drought) for the coordinate, assigning the returned value to each exposure. The result is grid-level. The process is fully automatable.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>licensing</t>
         </is>
       </c>
       <c r="C184" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is that pricing and the full hazard list are not published by the operator directly (Net Zero Compare, n.d.). In particular, only third-party estimates of cost are available, not operator-confirmed figures. Consequently, the source's exact scope and cost cannot be independently verified from public information, unless confirmed directly with Climate X.</t>
+          <t>The source is available under CC-BY 4.0 since 2 July 2025, the same licence as copernicus_cds (ECMWF Forum, 2025), replacing the prior "Licence to Use Copernicus Products" (Version 1.2, Nov 2019). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>eba_esg_dashboard</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>technical_effort_rationale</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is ready-made, high-granularity asset-level scores integrable via API for a broad set of confirmed hazards (Repath, n.d.; Net Zero Compare, n.d.). It is particularly useful for flood, storm, heat stress, wildfire and landslide classification. However, its suitability is reduced by unconfirmed pricing and enterprise-SaaS positioning that may exceed a typical SNCI's budget. It is therefore best used as a primary source subject to direct price confirmation appropriate to SNCI scale.</t>
+          <t>Technical effort is rated Low because the source is accessed through a statistics dashboard with no download or API. The rating reflects only the effort to access and read the source's own aggregate output; it does not include the substantially higher, distinct effort of replicating a similar analysis using the institution's own portfolio data, since the EBA ESG Dashboard provides no per-exposure data at all.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>technical_effort_rationale</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Pricing is not publicly disclosed by Climate X directly. Access is provided through a commercial SaaS platform and API under a quote-based licence agreement. Third-party industry comparison sources estimate EUR 20,000-60,000 per year for portfolios of 30-100 assets, described as 'mid-market' pricing (Repath, n.d.). The price information should be treated as indicative and not independently verified.</t>
+          <t>Technical effort is rated High because the source provides no bulk download or API, only individual web-interface queries. Each portfolio location must be manually looked up and the resulting hazard information manually recorded and linked back to the exposure, since no structured, machine-readable output exists for systematic processing.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>technical_effort_rationale</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the Spectra API (Climate X, n.d.) and receive an asset-level hazard/financial-loss score directly. No further spatial processing is required. The process is fully automatable for institutions with API access.</t>
+          <t>Technical effort is rated Medium because the source provides pre-computed, named indicators (e.g. baseline water stress, riverine flood risk) directly via API or download, so no own index definition is needed. However, geocoding of exposure addresses and a spatial join to the relevant watershed (Pfafstetter basin) polygon are still required before a value can be assigned to an exposure.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>climate_x</t>
+          <t>world_bank_gfdrr</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>technical_effort_rationale</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>The source is subject to a commercial licence agreement, quote-based, with no public price list (Net Zero Compare, n.d.). Access terms and portfolio size limits depend on the specific subscription negotiated. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
+          <t>Technical effort is rated Medium because the ThinkHazard! component provides a pre-computed, categorical hazard level directly via API once the ADM2 (district) unit is determined, requiring geocoding but no own index definition. However, the Risk Data Library component provides gridded/vector datasets of varying formats that require their own spatial overlay, so overall effort is higher than for a single ready-made API product.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>technical_effort_rationale</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
         <is>
-          <t>ClimateScore Global is a commercial physical climate risk platform operated by Jupiter Intelligence, Inc., a US company founded in 2017 (aigreentools.com, n.d.). It provides asset-level modelled physical hazard scores and finance-grade loss metrics across 9 physical perils, including flood, heat, drought, tropical cyclones and wildfire, at asset/facility-level granularity globally, based on peer-reviewed CMIP6/ERA5 science (aigreentools.com, n.d.). The source is accessed through a commercial SaaS platform and an API, and is paid. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>Technical effort is rated High because the source exists only as narrative PDF reports, not as structured, machine-readable per-location data. There is no download format, API or spatial layer to query; any use requires manual reading and qualitative interpretation of the reports, with no possibility of an automated pipeline.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>geosphere_spartacus</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>technical_effort_rationale</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is enterprise-tier, quote-based pricing not publicly listed (Mitiga Solutions, n.d.). In particular, the platform's scientific and financial-metric depth is designed for enterprise-scale deployments across banks, insurers and asset managers. Consequently, the source cannot be assumed affordable for an SNCI without direct confirmation, unless a limited-scope engagement at the lower end of the stated price range is negotiated.</t>
+          <t>Technical effort is rated Medium because the source provides gridded 1km daily climate data (temperature, precipitation, sunshine) via a coordinate-based API. While the raw variables are directly queryable without geocoding difficulty, the institution must define its own hazard thresholds (for example, a heat-wave or heavy-precipitation definition) to convert the climate data into a regulatory-relevant indicator. This climatological processing step distinguishes it from sources with pre-defined hazard indices.</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>geosphere_winfore_spei</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>technical_effort_rationale</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is extensive, scientifically validated hazard and financial-metric coverage across 9 peer-reviewed perils (aigreentools.com, n.d.). It is particularly useful for institutions needing finance-grade physical risk metrics beyond simple hazard scores. However, its suitability is reduced by enterprise-tier pricing likely above a typical SNCI's budget for full portfolio deployment. It is therefore best used as a primary source for a limited scope, subject to direct price negotiation.</t>
+          <t>Technical effort is rated Medium because the source provides a gridded 1km drought index (SPEI) via a coordinate-based API, so unlike raw climate variables no own drought-index computation is needed. However, geocoding of exposure addresses and correct interpretation of the standardised SPEI anomaly value (rather than reading it as an absolute deficit) are still required before assigning a classification to an exposure.</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>climate_x</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>technical_effort_rationale</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>Pricing is not publicly disclosed as a fixed list, but is quote-based. Jupiter's own CEO stated in a 2022 interview that 'subscription pricing ranges from $25,000 to multimillion-dollar contracts' depending on scope (Trellis/Clancy, 2022). Full portfolio deployments are typically six-figure annual commitments per third-party sources (Repath, n.d.). The price information should be treated as indicative, based on the operator's own public statement.</t>
+          <t>Technical effort is rated Low because the source provides ready-made asset-level hazard and financial-loss scores, directly integrable via API. No own index definition, geocoding or spatial processing is required beyond sending exposure coordinates or addresses to the API, consistent with the Low rating for other commercial facility/asset-level providers (Moody's, Munich Re).</t>
         </is>
       </c>
     </row>
@@ -10913,216 +10773,216 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>technical_effort_rationale</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the ClimateScore Global API (Jupiter Intelligence, n.d.) and receive an asset-level hazard/financial-loss score directly. No further spatial processing is required. The process is fully automatable for institutions with API access.</t>
+          <t>Technical effort is rated Low because the source provides ready-made asset-level hazard and finance-grade loss scores, directly integrable via API. No own index definition, geocoding or spatial processing is required beyond sending exposure coordinates or addresses to the API, consistent with the Low rating for other commercial facility/asset-level providers.</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>jupiter_intelligence</t>
+          <t>eea_climate_adapt</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
         <is>
-          <t>The source is subject to a commercial licence agreement, quote-based and defined case-by-case with the client (Mitiga Solutions, n.d.). Access terms and portfolio size limits depend on the specific subscription negotiated. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
+          <t>The source is based on the ECDE indicator set, computed by the Climate Data Factory and B-Open under a C3S service contract from established EURO-CORDEX/ERA5 climate projections, with each index individually documented and traceable to named peer-reviewed methodology papers (e.g. Spinoni et al., 2018/2020; Jacob et al., 2013). Known issues: the EEA's own summary report table resolves only to European macro-regions, while the underlying indicator dataset itself is considerably finer; resolution varies by indicator from 5km to approximately 28km (EEA/C3S, n.d.).</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>copernicus_climate_indicators</t>
+          <t>jrc_risk_data_hub</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>abstract</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
         <is>
-          <t>This is a set of standalone, ready-made physical hazard indicator products, published as individual datasets on the Copernicus Climate Data Store (CDS), distinct from the general-purpose raw climate variables covered by the separate copernicus_cds entry (ECMWF, n.d.). It provides ERA5-HEAT (UTCI/heat stress) and the SMHI hydrology dataset (flood, water stress/aridity, soil-moisture drought), covering these four hazards at grid granularity across Europe (Di Napoli et al., 2021; SMHI/C3S, n.d.). The source is accessed through direct download and a queryable API, and is free of charge. In the context of Template D 01.01, it is relevant to data point 0050 as a primary source.</t>
+          <t>The source is based on modelled hazard, exposure and historical-loss data compiled by the Joint Research Centre from multiple national and EU inputs, documented in JRC technical reports (Antofie et al., 2023). Known issues: the Vulnerability and Risk Analysis modules are explicitly described by JRC itself as 'ongoing work'; only the Exposure Analysis and Historical Events modules are reliably documented and hazard-verified at present.</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>copernicus_climate_indicators</t>
+          <t>copernicus_cds</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>limitations</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
         <is>
-          <t>The main limitation is narrower hazard breadth than the full Copernicus CDS catalogue. In particular, only heat stress, flood, water stress and soil-moisture drought are covered as standalone products; meteorological (SPI-3) drought and the temperature/precipitation/wind-based ECDE indices (heat wave, heavy precipitation, storm) remain accessible only via raw copernicus_cds variables or the Climate-ADAPT-curated bundle, and wildfire is documented separately under effis_wildfire. Consequently, the source cannot serve as a comprehensive hazard reference on its own, unless complemented by copernicus_cds, Climate-ADAPT and effis_wildfire for the remaining hazards.</t>
+          <t>The source is based primarily on ERA5 reanalysis and EURO-CORDEX climate projections, produced by ECMWF and national contributing centres under C3S and documented through peer-reviewed literature and individual CDS catalogue entries (ECMWF, n.d.). Known issues: quality, vintage and resolution vary considerably across the more than 140 datasets hosted on the CDS, so no single quality statement applies uniformly - each dataset must be assessed on its own documentation.</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>copernicus_climate_indicators</t>
+          <t>eba_esg_dashboard</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>suitability_snci</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is that each product is a purpose-built, documented hazard indicator with no own index-definition effort required, unlike raw Copernicus CDS variables (Di Napoli et al., 2021; SMHI/C3S, n.d.). It is particularly useful for heat stress, flood, water stress and soil-moisture drought classification at low processing effort. However, its suitability is reduced by its narrower hazard breadth compared with the full CDS catalogue. It is therefore best used as a primary source for its four covered hazards, complemented by other sources for the remainder.</t>
+          <t>The source is based on aggregated supervisory data compiled by the European Banking Authority from EU/EEA banks' regulatory reporting, with the underlying methodology documented in the EBA's risk dashboard technical notes (EBA, n.d.-a). Known issues: aggregation to EU bank-level obscures any institution- or exposure-level variation entirely, since the dashboard was not designed for granular or per-exposure use.</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>copernicus_climate_indicators</t>
+          <t>ecb_physical_risk_indicators</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
-          <t>The source is free of charge (ECMWF, n.d.), though registration is required to download data via the CDS.</t>
+          <t>The source is based on ECB-compiled indicators combining AnaCredit/RIAD supervisory data with JRC/Copernicus hazard layers, with the methodology published and updated across successive numbered releases (ECB, n.d.). Known issues: heat stress inclusion is inconsistent across the ECB's own communications - named in some contexts but absent from the core 9-hazard indicator list - which is flagged here as a documentation inconsistency pending clarification.</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>copernicus_climate_indicators</t>
+          <t>hq_flood_extent</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>portfolio_pipeline</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query or download the relevant standalone product (ERA5-HEAT for heat stress, SMHI hydrology for flood/water stress/soil-moisture drought) for the coordinate, assigning the returned value to each exposure. The result is grid-level. The process is fully automatable.</t>
+          <t>The source is based on a composite of Abflussuntersuchungen (ABU), HORA and BWV/WLV hazard-zoning inputs, published via the INSPIRE Geoportal with BMLUK as data owner (INSPIRE Geoportal Oesterreich, n.d.-b). Known issues: the Datenstand is October 2020, roughly six years old as of this review, and the underlying component datasets may carry inconsistent vintages, since they are separately maintained and merged into a single layer.</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>copernicus_climate_indicators</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>licensing</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
         <is>
-          <t>The source is available under CC-BY 4.0 since 2 July 2025, the same licence as copernicus_cds (ECMWF Forum, 2025), replacing the prior "Licence to Use Copernicus Products" (Version 1.2, Nov 2019). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
+          <t>The source is based on a compilation of multiple underlying Austrian hazard datasets (flood, earthquake, storm, hail, snow), presented by the operator explicitly as initial screening information rather than a validated legal assessment (LFRZ, n.d.). Known issues: the operator itself states that the map content is not legally binding, and the vintage of the individual underlying hazard layers per query is not disclosed to the user.</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>eba_esg_dashboard</t>
+          <t>wri_aqueduct</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>technical_effort_rationale</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated Low because the source is accessed through a statistics dashboard with no download or API. The rating reflects only the effort to access and read the source's own aggregate output; it does not include the substantially higher, distinct effort of replicating a similar analysis using the institution's own portfolio data, since the EBA ESG Dashboard provides no per-exposure data at all.</t>
+          <t>The source is based on the Aqueduct 4.0 modelled water-risk framework, produced by the World Resources Institute using global hydrological models with a publicly documented methodology (WRI, n.d.-b). Known issues: as a global model, it is not locally calibrated or independently validated specifically for Austria, and watershed-level aggregation may obscure local variation within a single sub-catchment.</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>moodys_physical_risk</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>technical_effort_rationale</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated High because the source provides no bulk download or API, only individual web-interface queries. Each portfolio location must be manually looked up and the resulting hazard information manually recorded and linked back to the exposure, since no structured, machine-readable output exists for systematic processing.</t>
+          <t>The source is based on proprietary modelled physical risk scores, originally developed by Four Twenty Seven, Inc. and now operated by Moody's ESG Solutions following the 2019 acquisition (Moody's, n.d.-b). Known issues: the underlying methodology is not fully transparent or independently validated, as is typical for proprietary commercial risk models, and confirmed Austria-relevant hazard coverage is narrower than the product's general marketing suggests.</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>wri_aqueduct</t>
+          <t>munich_re_nathan</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>technical_effort_rationale</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated Medium because the source provides pre-computed, named indicators (e.g. baseline water stress, riverine flood risk) directly via API or download, so no own index definition is needed. However, geocoding of exposure addresses and a spatial join to the relevant watershed (Pfafstetter basin) polygon are still required before a value can be assigned to an exposure.</t>
+          <t>The source is based on proprietary modelled natural hazard and climate scenario scores, produced by Munich Re, a reinsurer with decades of natural-catastrophe modelling experience (Munich Re, n.d.-b). Known issues: the underlying methodology is not fully public and independent third-party validation is limited; only the 15 explicitly named Natural Hazards Edition hazards are confirmed, while heat, drought and water-stress coverage under the separate 'Climate Change Edition' could not be individually verified.</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>world_bank_gfdrr</t>
+          <t>kryomon_at</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>technical_effort_rationale</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated Medium because the ThinkHazard! component provides a pre-computed, categorical hazard level directly via API once the ADM2 (district) unit is determined, requiring geocoding but no own index definition. However, the Risk Data Library component provides gridded/vector datasets of varying formats that require their own spatial overlay, so overall effort is higher than for a single ready-made API product.</t>
+          <t>The source is based on periodic reports from a multi-institutional Austrian research consortium coordinated by the University of Graz, involving multiple universities and the Austrian and Bavarian Academies of Sciences (KryoMon.AT, n.d.). Known issues: reporting is narrative and qualitative rather than following a fixed statistical methodology, published irregularly with no disclosed fixed schedule, and no structured, machine-readable per-location data exists.</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>kryomon_at</t>
+          <t>wirtschafts_compass</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>technical_effort_rationale</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated High because the source exists only as narrative PDF reports, not as structured, machine-readable per-location data. There is no download format, API or spatial layer to query; any use requires manual reading and qualitative interpretation of the reports, with no possibility of an automated pipeline.</t>
+          <t>The source is based on editorially compiled and enriched company data, produced by Compass-Verlag GmbH, a long-established Austrian commercial business-information provider (Compass-Verlag, n.d.). Known issues: as an editorial rather than official classification, its methodology is not independently published or peer-reviewed, and individual entries may diverge from the official Statistik Austria HVD assignment - cross-validation against HVD is advisable where feasible.</t>
         </is>
       </c>
     </row>
@@ -11134,12 +10994,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>technical_effort_rationale</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated Medium because the source provides gridded 1km daily climate data (temperature, precipitation, sunshine) via a coordinate-based API. While the raw variables are directly queryable without geocoding difficulty, the institution must define its own hazard thresholds (for example, a heat-wave or heavy-precipitation definition) to convert the climate data into a regulatory-relevant indicator. This climatological processing step distinguishes it from sources with pre-defined hazard indices.</t>
+          <t>The source is based on gridded observational climate data produced by GeoSphere Austria from station measurements interpolated to a 1km grid, with the methodology documented in peer-reviewed literature and in operational use since 1961 (GeoSphere Austria, n.d.-a). Known issues: the interpolation process introduces some uncertainty in data-sparse high-alpine regions, and the most recent seven days of data are provisional pending final quality control.</t>
         </is>
       </c>
     </row>
@@ -11151,12 +11011,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>technical_effort_rationale</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated Medium because the source provides a gridded 1km drought index (SPEI) via a coordinate-based API, so unlike raw climate variables no own drought-index computation is needed. However, geocoding of exposure addresses and correct interpretation of the standardised SPEI anomaly value (rather than reading it as an absolute deficit) are still required before assigning a classification to an exposure.</t>
+          <t>The source is based on the SPEI drought index, derived from SPARTACUS temperature and precipitation fields using an established statistical methodology (a normal-distribution transform over defined climate reference periods), standard in the international drought-monitoring literature (GeoSphere Austria, n.d.-b). Known issues: as a standardised anomaly index, SPEI requires correct interpretation relative to its reference period rather than being read as an absolute water deficit.</t>
         </is>
       </c>
     </row>
@@ -11168,12 +11028,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>technical_effort_rationale</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated Low because the source provides ready-made asset-level hazard and financial-loss scores, directly integrable via API. No own index definition, geocoding or spatial processing is required beyond sending exposure coordinates or addresses to the API, consistent with the Low rating for other commercial facility/asset-level providers (Moody's, Munich Re).</t>
+          <t>The source is based on proprietary modelled asset-level physical risk scores, produced by Climate X Ltd, a UK-based climate-risk analytics company founded in 2020 (Technology Tools, n.d.). Known issues: neither the full methodology nor the complete hazard list is published by the operator directly, and no independent third-party validation was identified; pricing and hazard-list completeness rely on third-party industry sources rather than operator confirmation.</t>
         </is>
       </c>
     </row>
@@ -11185,19 +11045,19 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>technical_effort_rationale</t>
+          <t>data_quality</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t>Technical effort is rated Low because the source provides ready-made asset-level hazard and finance-grade loss scores, directly integrable via API. No own index definition, geocoding or spatial processing is required beyond sending exposure coordinates or addresses to the API, consistent with the Low rating for other commercial facility/asset-level providers.</t>
+          <t>The source is based on proprietary modelled asset-level physical risk and financial-loss metrics, produced by Jupiter Intelligence, Inc. from peer-reviewed CMIP6/ERA5 climate science (aigreentools.com, n.d.). Known issues: while the underlying climate science is peer-reviewed and publicly documented, the proprietary loss-translation methodology is not independently validated, and the only available pricing indication is a single CEO interview statement rather than a published price list.</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>eea_climate_adapt</t>
+          <t>copernicus_climate_indicators</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -11207,281 +11067,57 @@
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>The source is based on the ECDE indicator set, computed by the Climate Data Factory and B-Open under a C3S service contract from established EURO-CORDEX/ERA5 climate projections, with each index individually documented and traceable to named peer-reviewed methodology papers (e.g. Spinoni et al., 2018/2020; Jacob et al., 2013). Known issues: the EEA's own summary report table resolves only to European macro-regions, while the underlying indicator dataset itself is considerably finer; resolution varies by indicator from 5km to approximately 28km (EEA/C3S, n.d.).</t>
+          <t>The source comprises two named, quality-controlled products: ERA5-HEAT, peer-reviewed and produced by ECMWF (Di Napoli et al., 2021), and the SMHI hydrology dataset, produced and quality-assured by the Swedish Meteorological and Hydrological Institute for C3S (SMHI/C3S, n.d.). Known issues: the SMHI hydrology projections are static 30-year model outputs rather than continuously updated, so their currency should be checked against the stated reference period before use.</t>
         </is>
       </c>
     </row>
     <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>jrc_risk_data_hub</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C211" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on modelled hazard, exposure and historical-loss data compiled by the Joint Research Centre from multiple national and EU inputs, documented in JRC technical reports (Antofie et al., 2023). Known issues: the Vulnerability and Risk Analysis modules are explicitly described by JRC itself as 'ongoing work'; only the Exposure Analysis and Historical Events modules are reliably documented and hazard-verified at present.</t>
-        </is>
-      </c>
+      <c r="C211" s="4" t="n"/>
     </row>
     <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>copernicus_cds</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C212" s="4" t="inlineStr">
-        <is>
-          <t>The source is based primarily on ERA5 reanalysis and EURO-CORDEX climate projections, produced by ECMWF and national contributing centres under C3S and documented through peer-reviewed literature and individual CDS catalogue entries (ECMWF, n.d.). Known issues: quality, vintage and resolution vary considerably across the more than 140 datasets hosted on the CDS, so no single quality statement applies uniformly - each dataset must be assessed on its own documentation.</t>
-        </is>
-      </c>
+      <c r="C212" s="4" t="n"/>
     </row>
     <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>eba_esg_dashboard</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C213" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on aggregated supervisory data compiled by the European Banking Authority from EU/EEA banks' regulatory reporting, with the underlying methodology documented in the EBA's risk dashboard technical notes (EBA, n.d.-a). Known issues: aggregation to EU bank-level obscures any institution- or exposure-level variation entirely, since the dashboard was not designed for granular or per-exposure use.</t>
-        </is>
-      </c>
+      <c r="C213" s="4" t="n"/>
     </row>
     <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>ecb_physical_risk_indicators</t>
-        </is>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C214" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on ECB-compiled indicators combining AnaCredit/RIAD supervisory data with JRC/Copernicus hazard layers, with the methodology published and updated across successive numbered releases (ECB, n.d.). Known issues: heat stress inclusion is inconsistent across the ECB's own communications - named in some contexts but absent from the core 9-hazard indicator list - which is flagged here as a documentation inconsistency pending clarification.</t>
-        </is>
-      </c>
+      <c r="C214" s="4" t="n"/>
     </row>
     <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>hq_flood_extent</t>
-        </is>
-      </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C215" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on a composite of Abflussuntersuchungen (ABU), HORA and BWV/WLV hazard-zoning inputs, published via the INSPIRE Geoportal with BMLUK as data owner (INSPIRE Geoportal Oesterreich, n.d.-b). Known issues: the Datenstand is October 2020, roughly six years old as of this review, and the underlying component datasets may carry inconsistent vintages, since they are separately maintained and merged into a single layer.</t>
-        </is>
-      </c>
+      <c r="C215" s="4" t="n"/>
     </row>
     <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>hora</t>
-        </is>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C216" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on a compilation of multiple underlying Austrian hazard datasets (flood, earthquake, storm, hail, snow), presented by the operator explicitly as initial screening information rather than a validated legal assessment (LFRZ, n.d.). Known issues: the operator itself states that the map content is not legally binding, and the vintage of the individual underlying hazard layers per query is not disclosed to the user.</t>
-        </is>
-      </c>
+      <c r="C216" s="4" t="n"/>
     </row>
     <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>wri_aqueduct</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C217" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on the Aqueduct 4.0 modelled water-risk framework, produced by the World Resources Institute using global hydrological models with a publicly documented methodology (WRI, n.d.-b). Known issues: as a global model, it is not locally calibrated or independently validated specifically for Austria, and watershed-level aggregation may obscure local variation within a single sub-catchment.</t>
-        </is>
-      </c>
+      <c r="C217" s="4" t="n"/>
     </row>
     <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>moodys_physical_risk</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C218" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on proprietary modelled physical risk scores, originally developed by Four Twenty Seven, Inc. and now operated by Moody's ESG Solutions following the 2019 acquisition (Moody's, n.d.-b). Known issues: the underlying methodology is not fully transparent or independently validated, as is typical for proprietary commercial risk models, and confirmed Austria-relevant hazard coverage is narrower than the product's general marketing suggests.</t>
-        </is>
-      </c>
+      <c r="C218" s="4" t="n"/>
     </row>
     <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>munich_re_nathan</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C219" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on proprietary modelled natural hazard and climate scenario scores, produced by Munich Re, a reinsurer with decades of natural-catastrophe modelling experience (Munich Re, n.d.-b). Known issues: the underlying methodology is not fully public and independent third-party validation is limited; only the 15 explicitly named Natural Hazards Edition hazards are confirmed, while heat, drought and water-stress coverage under the separate 'Climate Change Edition' could not be individually verified.</t>
-        </is>
-      </c>
+      <c r="C219" s="4" t="n"/>
     </row>
     <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>kryomon_at</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C220" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on periodic reports from a multi-institutional Austrian research consortium coordinated by the University of Graz, involving multiple universities and the Austrian and Bavarian Academies of Sciences (KryoMon.AT, n.d.). Known issues: reporting is narrative and qualitative rather than following a fixed statistical methodology, published irregularly with no disclosed fixed schedule, and no structured, machine-readable per-location data exists.</t>
-        </is>
-      </c>
+      <c r="C220" s="4" t="n"/>
     </row>
     <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>wirtschafts_compass</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C221" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on editorially compiled and enriched company data, produced by Compass-Verlag GmbH, a long-established Austrian commercial business-information provider (Compass-Verlag, n.d.). Known issues: as an editorial rather than official classification, its methodology is not independently published or peer-reviewed, and individual entries may diverge from the official Statistik Austria HVD assignment - cross-validation against HVD is advisable where feasible.</t>
-        </is>
-      </c>
+      <c r="C221" s="4" t="n"/>
     </row>
     <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>geosphere_spartacus</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C222" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on gridded observational climate data produced by GeoSphere Austria from station measurements interpolated to a 1km grid, with the methodology documented in peer-reviewed literature and in operational use since 1961 (GeoSphere Austria, n.d.-a). Known issues: the interpolation process introduces some uncertainty in data-sparse high-alpine regions, and the most recent seven days of data are provisional pending final quality control.</t>
-        </is>
-      </c>
+      <c r="C222" s="4" t="n"/>
     </row>
     <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>geosphere_winfore_spei</t>
-        </is>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C223" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on the SPEI drought index, derived from SPARTACUS temperature and precipitation fields using an established statistical methodology (a normal-distribution transform over defined climate reference periods), standard in the international drought-monitoring literature (GeoSphere Austria, n.d.-b). Known issues: as a standardised anomaly index, SPEI requires correct interpretation relative to its reference period rather than being read as an absolute water deficit.</t>
-        </is>
-      </c>
+      <c r="C223" s="4" t="n"/>
     </row>
     <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>climate_x</t>
-        </is>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C224" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on proprietary modelled asset-level physical risk scores, produced by Climate X Ltd, a UK-based climate-risk analytics company founded in 2020 (Technology Tools, n.d.). Known issues: neither the full methodology nor the complete hazard list is published by the operator directly, and no independent third-party validation was identified; pricing and hazard-list completeness rely on third-party industry sources rather than operator confirmation.</t>
-        </is>
-      </c>
+      <c r="C224" s="4" t="n"/>
     </row>
     <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>jupiter_intelligence</t>
-        </is>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C225" s="4" t="inlineStr">
-        <is>
-          <t>The source is based on proprietary modelled asset-level physical risk and financial-loss metrics, produced by Jupiter Intelligence, Inc. from peer-reviewed CMIP6/ERA5 climate science (aigreentools.com, n.d.). Known issues: while the underlying climate science is peer-reviewed and publicly documented, the proprietary loss-translation methodology is not independently validated, and the only available pricing indication is a single CEO interview statement rather than a published price list.</t>
-        </is>
-      </c>
+      <c r="C225" s="4" t="n"/>
     </row>
     <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>copernicus_climate_indicators</t>
-        </is>
-      </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>data_quality</t>
-        </is>
-      </c>
-      <c r="C226" s="4" t="inlineStr">
-        <is>
-          <t>The source comprises two named, quality-controlled products: ERA5-HEAT, peer-reviewed and produced by ECMWF (Di Napoli et al., 2021), and the SMHI hydrology dataset, produced and quality-assured by the Swedish Meteorological and Hydrological Institute for C3S (SMHI/C3S, n.d.). Known issues: the SMHI hydrology projections are static 30-year model outputs rather than continuously updated, so their currency should be checked against the stated reference period before use.</t>
-        </is>
-      </c>
+      <c r="C226" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -12289,21 +11925,8 @@
       <c r="C33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>relevance</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Primary / Secondary - relevance of this specific source-datapoint combination.</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Distinct from relevance_level in sources.csv (one overall rating per source).</t>
-        </is>
-      </c>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Update ESG data source matrix
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ESG_Data_Source_Matrix_Structured.xlsx
+++ b/data/ESG_Data_Source_Matrix_Structured.xlsx
@@ -2366,7 +2366,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Partial because the only available index measures human thermal comfort rather than asset-level heat stress, and it is reanalysis-based with no climate projections available</t>
+          <t>Partial because the only available index measures human thermal comfort rather than asset-level heat stress, and it is reanalysis-based with no climate projections available (The Climate Data Factory and B-Open et al., 2024).</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Full because several dedicated heatwave indices with documented percentile thresholds are provided; the apparent-temperature variant comes from a different input dataset and is therefore not directly comparable with the others</t>
+          <t>Full because several dedicated heatwave indices with documented percentile thresholds are provided; the apparent-temperature variant comes from a different input dataset and is therefore not directly comparable with the others (The Climate Data Factory and B-Open et al., 2024).</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Full because dedicated fire-danger indices are provided; the resolution is finer than that of most other indices in this source, which come from a different input dataset</t>
+          <t>Full because dedicated fire-danger indices are provided; the resolution is finer than that of most other indices in this source, which come from a different input dataset (The Climate Data Factory and B-Open et al., 2024).</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Full because a dedicated wind-extremes index is provided; it is threshold-based and does not identify individual windstorm events</t>
+          <t>Full because a dedicated wind-extremes index is provided; it is threshold-based and does not identify individual windstorm events (The Climate Data Factory and B-Open et al., 2024).</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Partial because the only available index describes the climatic water balance and not water stress in the sense of demand relative to available supply</t>
+          <t>Partial because the only available index describes the climatic water balance and not water stress in the sense of demand relative to available supply (The Climate Data Factory and B-Open et al., 2024).</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Full because dedicated river-flooding indices from a hydrological model are provided; the resolution is finer than that of the atmospheric indices in this source, and coverage is limited to riverine flooding</t>
+          <t>Full because dedicated river-flooding indices from a hydrological model are provided; the resolution is finer than that of the atmospheric indices in this source, and coverage is limited to riverine flooding (The Climate Data Factory and B-Open et al., 2024).</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Full because three dedicated extreme-precipitation indices with documented percentile thresholds are provided</t>
+          <t>Full because three dedicated extreme-precipitation indices with documented percentile thresholds are provided (The Climate Data Factory and B-Open et al., 2024).</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Full because both meteorological and soil-moisture drought indices are provided; they come from different input datasets, so their resolutions differ and they are not directly comparable</t>
+          <t>Full because both meteorological and soil-moisture drought indices are provided; they come from different input datasets, so their resolutions differ and they are not directly comparable (The Climate Data Factory and B-Open et al., 2024).</t>
         </is>
       </c>
     </row>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Partial because the hazard appears only in the Loss Data module as historical event and damage records compiled from EM-DAT, media and other secondary sources; the Risk Analysis module provides no modelled forward-looking layer for it</t>
+          <t>Partial because the hazard appears only in the Loss Data module as historical event and damage records compiled from EM-DAT, media and other secondary sources; the Risk Analysis module provides no modelled forward-looking layer for it (Joint Research Centre / Disaster Risk Management Knowledge Centre, no date).</t>
         </is>
       </c>
     </row>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Full because a modelled hazard layer is provided in the Risk Analysis module and aggregated to administrative units</t>
+          <t>Full because a modelled hazard layer is provided in the Risk Analysis module and aggregated to administrative units (Joint Research Centre / Disaster Risk Management Knowledge Centre, no date).</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Partial because the hazard appears only in the Loss Data module as historical event and damage records compiled from EM-DAT, media and other secondary sources; the Risk Analysis module provides no modelled forward-looking layer for it</t>
+          <t>Partial because the hazard appears only in the Loss Data module as historical event and damage records compiled from EM-DAT, media and other secondary sources; the Risk Analysis module provides no modelled forward-looking layer for it (Joint Research Centre / Disaster Risk Management Knowledge Centre, no date).</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Full because a modelled hazard layer is provided in the Risk Analysis module and aggregated to administrative units; riverine and coastal flooding are covered, pluvial flooding is not</t>
+          <t>Full because a modelled hazard layer is provided in the Risk Analysis module and aggregated to administrative units; riverine and coastal flooding are covered, pluvial flooding is not (Joint Research Centre / Disaster Risk Management Knowledge Centre, no date).</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Partial because the hazard appears only in the Loss Data module as historical event and damage records compiled from EM-DAT, media and other secondary sources; the Risk Analysis module provides no modelled forward-looking layer for it</t>
+          <t>Partial because the hazard appears only in the Loss Data module as historical event and damage records compiled from EM-DAT, media and other secondary sources; the Risk Analysis module provides no modelled forward-looking layer for it (Joint Research Centre / Disaster Risk Management Knowledge Centre, no date).</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Partial because the hazard appears only in the Loss Data module as historical event and damage records compiled from EM-DAT, media and other secondary sources; the Risk Analysis module provides no modelled forward-looking layer for it</t>
+          <t>Partial because the hazard appears only in the Loss Data module as historical event and damage records compiled from EM-DAT, media and other secondary sources; the Risk Analysis module provides no modelled forward-looking layer for it (Joint Research Centre / Disaster Risk Management Knowledge Centre, no date).</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Full because a modelled susceptibility layer is provided; its resolution is finer than that of the other layers in this source, which are aggregated to administrative units</t>
+          <t>Full because a modelled susceptibility layer is provided; its resolution is finer than that of the other layers in this source, which are aggregated to administrative units (Joint Research Centre / Disaster Risk Management Knowledge Centre, no date).</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Full because dedicated fire-danger and burnt-area products are provided; the forecast grid is coarse relative to Austria, and the index is time-varying, so a static exposure attribute requires an own aggregation choice</t>
+          <t>Full because dedicated fire-danger and burnt-area products are provided; the forecast grid is coarse relative to Austria, and the index is time-varying, so a static exposure attribute requires an own aggregation choice (Copernicus Emergency Management Service / EFFIS, no date b; Rosadi et al., 2023).</t>
         </is>
       </c>
     </row>
@@ -3256,7 +3256,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Partial because no ready-made permafrost index exists in the catalogue; the raw variables are usable only as input to the institution’s own model</t>
+          <t>Partial because no ready-made permafrost index exists in the catalogue; the raw variables are usable only as input to the institution’s own model (Hersbach et al., 2023; ECMWF, 2026).</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3288,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Full because the temperature fields are the quantity that defines the hazard; the threshold and the index definition rest with the institution, and ready-made indices are reached through the separate ECDE dataset</t>
+          <t>Full because the temperature fields are the quantity that defines the hazard; the threshold and the index definition rest with the institution, and ready-made indices are reached through the separate ECDE dataset (ECMWF, 2026).</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Full because the wind-speed fields are the quantity that defines the hazard; the threshold definition rests with the institution, and the ready-made index is reached through the separate ECDE dataset</t>
+          <t>Full because the wind-speed fields are the quantity that defines the hazard; the threshold definition rests with the institution, and the ready-made index is reached through the separate ECDE dataset (ECMWF, 2026).</t>
         </is>
       </c>
     </row>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Full because the precipitation fields are the quantity that defines the hazard; the threshold and the index definition rest with the institution, and ready-made indices are reached through the separate ECDE dataset</t>
+          <t>Full because the precipitation fields are the quantity that defines the hazard; the threshold and the index definition rest with the institution, and ready-made indices are reached through the separate ECDE dataset (ECMWF, 2026).</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Partial because the meteorological component must be derived by the institution and the soil-moisture component belongs to a separate ready-made dataset</t>
+          <t>Partial because the meteorological component must be derived by the institution and the soil-moisture component belongs to a separate ready-made dataset (ECMWF, 2026).</t>
         </is>
       </c>
     </row>
@@ -3488,7 +3488,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Partial because no erosion index exists in the catalogue; using the source requires independent erosion modelling, for example of the RUSLE type</t>
+          <t>Partial because no erosion index exists in the catalogue; using the source requires independent erosion modelling, for example of the RUSLE type (ECMWF, 2026).</t>
         </is>
       </c>
     </row>
@@ -3523,24 +3523,10 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>partial</t>
-        </is>
-      </c>
-      <c r="D53" s="9" t="inlineStr">
-        <is>
-          <t>Institution/portfolio (bank-aggregate) level</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Physical-risk indicators aggregated from Pillar 3 ESG disclosures, published per institution and as EU aggregates</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Partial because the dashboard reports supervisory statistics on exposures flagged as subject to physical risk; it is not spatially resolved and cannot be attached to an individual exposure</t>
-        </is>
-      </c>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3645,24 +3631,10 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>partial</t>
-        </is>
-      </c>
-      <c r="D59" s="9" t="inlineStr">
-        <is>
-          <t>Institution/portfolio (bank-aggregate) level</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Physical-risk indicators aggregated from Pillar 3 ESG disclosures, published per institution and as EU aggregates</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Partial because the dashboard reports supervisory statistics on exposures flagged as subject to physical risk; it is not spatially resolved and cannot be attached to an individual exposure</t>
-        </is>
-      </c>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="n"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3890,7 +3862,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Full because the dataset is the official modelled inundation extent for the 30-, 100- and 300-year events, maintained under the implementation of the Floods Directive</t>
+          <t>Full because the dataset is the official modelled inundation extent for the 30-, 100- and 300-year events, maintained under the implementation of the Floods Directive (Umweltbundesamt, 2020).</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4092,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Partial because the plan covers torrent-related flood only, and is mapped only for municipalities with torrent, avalanche or erosion catchments and only within the spatially relevant area</t>
+          <t>Partial because the plan covers torrent-related flood only, and is mapped only for municipalities with torrent, avalanche or erosion catchments and only within the spatially relevant area (Forsttechnischer Dienst für Wildbach- und Lawinenverbauung, no date).</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4178,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Full because the hazard type is assessed in its own right. Mapped only for municipalities that contain torrent, avalanche or erosion catchments and only within the spatially relevant area, so an unmapped location is ambiguous</t>
+          <t>Full because the hazard type is assessed in its own right. Mapped only for municipalities that contain torrent, avalanche or erosion catchments and only within the spatially relevant area, so an unmapped location is ambiguous (Forsttechnischer Dienst für Wildbach- und Lawinenverbauung, no date).</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4210,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Full because the hazard type is assessed in its own right. Mapped only for municipalities that contain torrent, avalanche or erosion catchments and only within the spatially relevant area, so an unmapped location is ambiguous</t>
+          <t>Full because the hazard type is assessed in its own right. Mapped only for municipalities that contain torrent, avalanche or erosion catchments and only within the spatially relevant area, so an unmapped location is ambiguous (Forsttechnischer Dienst für Wildbach- und Lawinenverbauung, no date).</t>
         </is>
       </c>
     </row>
@@ -4342,7 +4314,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Full in the sense that Austria-wide wind information is available, but it describes current conditions rather than a long-term hazard zoning, and its grid is coarser than the parcel-level flood layer</t>
+          <t>Full in the sense that Austria-wide wind information is available, but it describes current conditions rather than a long-term hazard zoning, and its grid is coarser than the parcel-level flood layer (HORA, no date).</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4364,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Full because a dedicated Austria-wide flood hazard zoning is provided and can be queried for any address; it is published for first orientation and is not a legally binding hazard zone plan</t>
+          <t>Full because a dedicated Austria-wide flood hazard zoning is provided and can be queried for any address; it is published for first orientation and is not a legally binding hazard zone plan (Bundesministerium für Land- und Forstwirtschaft, Klima- und Umweltschutz, Regionen und Wasserwirtschaft, no date).</t>
         </is>
       </c>
     </row>
@@ -4496,7 +4468,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Partial because the layer is an indicative screening product, newer and less mature than the flood layer, and is provided on a grid rather than at parcel level</t>
+          <t>Partial because the layer is an indicative screening product, newer and less mature than the flood layer, and is provided on a grid rather than at parcel level (HORA, no date).</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4590,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Full because several dedicated water-stress indicators are provided, each as a raw value, a score on a scale from 0 to 5 and a category label; they are modelled with PCR-GLOBWB 2 and describe demand relative to available supply</t>
+          <t>Full because several dedicated water-stress indicators are provided, each as a raw value, a score on a scale from 0 to 5 and a category label; they are modelled with PCR-GLOBWB 2 and describe demand relative to available supply (World Resources Institute, no date a).</t>
         </is>
       </c>
     </row>
@@ -4650,7 +4622,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Full because dedicated flood indicators are provided in their own right rather than inferred from the water-stress indicators; they express expected annual affected population and assets, not inundation depth</t>
+          <t>Full because dedicated flood indicators are provided in their own right rather than inferred from the water-stress indicators; they express expected annual affected population and assets, not inundation depth (World Resources Institute, no date a).</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4672,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Full because a dedicated drought indicator is provided; it combines hazard, exposure and vulnerability into a risk score rather than describing the meteorological drought itself</t>
+          <t>Full because a dedicated drought indicator is provided; it combines hazard, exposure and vulnerability into a risk score rather than describing the meteorological drought itself (World Resources Institute, no date a).</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4758,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Full because heat stress is one of the named risk categories scored per facility</t>
+          <t>Full because heat stress is one of the named risk categories scored per facility (Moody's, no date a).</t>
         </is>
       </c>
     </row>
@@ -4821,10 +4793,24 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="D115" s="9" t="n"/>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t>Facility/object level</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>No separately named acute heat product; covered within the Heat Stress risk category; the underlying index and model are not publicly documented</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Partial because only a chronic heat-stress category is named among the six climate hazards; whether acute heatwave events are distinguished could not be established from the public documentation (Moody's, no date a).</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="30" customHeight="1" s="6">
       <c r="A116" t="inlineStr">
@@ -4854,7 +4840,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Full because wildfires are one of the named risk categories scored per facility</t>
+          <t>Full because wildfires are one of the named risk categories scored per facility (Moody's, no date a).</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4890,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Full because water stress is one of the named risk categories scored per facility</t>
+          <t>Full because water stress is one of the named risk categories scored per facility (Moody's, no date a).</t>
         </is>
       </c>
     </row>
@@ -4936,7 +4922,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Full because floods are one of the named risk categories scored per facility</t>
+          <t>Full because floods are one of the named risk categories scored per facility (Moody's, no date a).</t>
         </is>
       </c>
     </row>
@@ -5043,7 +5029,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>full</t>
         </is>
       </c>
       <c r="D125" s="9" t="inlineStr">
@@ -5053,12 +5039,12 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Not individually named; advertised within the Climate Change Edition; the underlying index and model are not publicly documented</t>
+          <t>Heat Stress Index of the Climate Change Edition</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Partial because the hazard is only advertised through the separate Climate Change Edition, which refers to 13 climate hazards without naming them individually in the material reviewed</t>
+          <t>Full because a dedicated heat-stress index is named among the eight climate hazard scores, provided per location for current conditions and for four projection years and scenarios (Munich Re, Risk Management Partners, no date c).</t>
         </is>
       </c>
     </row>
@@ -5103,12 +5089,12 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Not individually named; advertised within the Climate Change Edition; the underlying index and model are not publicly documented</t>
+          <t>No separately named acute heat product; covered within the Heat Stress Index</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Partial because the hazard is only advertised through the separate Climate Change Edition, which refers to 13 climate hazards without naming them individually in the material reviewed</t>
+          <t>Partial because only a chronic heat-stress index is named; whether acute heatwave events are distinguished is not stated in the product description (Munich Re, Risk Management Partners, no date c).</t>
         </is>
       </c>
     </row>
@@ -5135,12 +5121,12 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Wildfire peril of the Natural Hazards Edition; the underlying index and model are not publicly documented</t>
+          <t>Wildfire peril of the Natural Hazards Edition and the Fire Weather Stress Index of the Climate Change Edition</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Full because wildfire is named individually in the hazard list of the Natural Hazards Edition</t>
+          <t>Full because wildfire is scored in both editions, as a current hazard and as a forward-looking index (Munich Re, Risk Management Partners, no date c).</t>
         </is>
       </c>
     </row>
@@ -5167,12 +5153,12 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Extratropical storm peril of the Natural Hazards Edition; the underlying index and model are not publicly documented</t>
+          <t>Extratropical Storm and Tropical Cyclone perils of the Natural Hazards Edition</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Full because extratropical storm is named individually in the hazard list of the Natural Hazards Edition</t>
+          <t>Full because extratropical storm is scored as a named peril, which is the relevant process for Austria (Munich Re, Risk Management Partners, no date c).</t>
         </is>
       </c>
     </row>
@@ -5199,12 +5185,12 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Not individually named; advertised within the Climate Change Edition; the underlying index and model are not publicly documented</t>
+          <t>No dedicated index; covered indirectly through the Drought Stress Index</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Partial because the hazard is only advertised through the separate Climate Change Edition, which refers to 13 climate hazards without naming them individually in the material reviewed</t>
+          <t>Partial because water stress is not among the eight named climate hazard scores and is only approximated by the drought index (Munich Re, Risk Management Partners, no date c).</t>
         </is>
       </c>
     </row>
@@ -5231,12 +5217,12 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>River flood peril of the Natural Hazards Edition; the underlying index and model are not publicly documented</t>
+          <t>River Flood and Storm Surge perils of the Natural Hazards Edition, plus the River Flood climate hazard score</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Full because river flood is named individually in the hazard list of the Natural Hazards Edition</t>
+          <t>Full because river flood is scored as a named peril in both editions (Munich Re, Risk Management Partners, no date c).</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5239,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>full</t>
         </is>
       </c>
       <c r="D132" s="9" t="inlineStr">
@@ -5263,12 +5249,12 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Flash flood peril of the Natural Hazards Edition; the underlying index and model are not publicly documented</t>
+          <t>Precipitation Stress Index of the Climate Change Edition</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Partial because flash flood is covered but scored as a flood hazard rather than as a distinct heavy-precipitation indicator</t>
+          <t>Full because a dedicated precipitation index is named among the eight climate hazard scores; the Natural Hazards Edition additionally scores flash flood as a separate peril (Munich Re, Risk Management Partners, no date c).</t>
         </is>
       </c>
     </row>
@@ -5285,7 +5271,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>full</t>
         </is>
       </c>
       <c r="D133" s="9" t="inlineStr">
@@ -5295,12 +5281,12 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Not individually named; advertised within the Climate Change Edition; the underlying index and model are not publicly documented</t>
+          <t>Drought Stress Index of the Climate Change Edition</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Partial because the hazard is only advertised through the separate Climate Change Edition, which refers to 13 climate hazards without naming them individually in the material reviewed</t>
+          <t>Full because a dedicated drought index is named among the eight climate hazard scores (Munich Re, Risk Management Partners, no date c).</t>
         </is>
       </c>
     </row>
@@ -5363,12 +5349,12 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Landslide peril of the Natural Hazards Edition; the underlying index and model are not publicly documented</t>
+          <t>Landslide peril of the Natural Hazards Edition</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Full because landslide is named individually in the hazard list of the Natural Hazards Edition</t>
+          <t>Full because landslide is one of the fifteen named hazard scores of the Natural Hazards Edition (Munich Re, Risk Management Partners, no date c).</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5422,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Full because a dedicated hazard class based on probabilistic heat data is provided; the reported value is the highest class within the administrative unit</t>
+          <t>Full because a dedicated hazard class based on probabilistic heat data is provided; the reported value is the highest class within the administrative unit (GFDRR, no date a).</t>
         </is>
       </c>
     </row>
@@ -5468,7 +5454,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Full because a dedicated hazard class is provided; the reported value is the highest class within the administrative unit</t>
+          <t>Full because a dedicated hazard class is provided; the reported value is the highest class within the administrative unit (GFDRR, no date a).</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5486,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Partial because the hazard model and terminology are tropical-cyclone-oriented; applicability to European extratropical windstorms could not be confirmed from the documentation</t>
+          <t>Partial because the hazard model and terminology are tropical-cyclone-oriented; applicability to European extratropical windstorms could not be confirmed from the documentation (GFDRR, no date a).</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5518,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Full because a dedicated hazard class describing water availability relative to population is provided</t>
+          <t>Full because a dedicated hazard class describing water availability relative to population is provided (GFDRR, no date a).</t>
         </is>
       </c>
     </row>
@@ -5564,7 +5550,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Full because three dedicated flood hazard classes are provided; the reported value is the highest class within the administrative unit, not the hazard at a specific location</t>
+          <t>Full because three dedicated flood hazard classes are provided; the reported value is the highest class within the administrative unit, not the hazard at a specific location (GFDRR, no date a).</t>
         </is>
       </c>
     </row>
@@ -5614,7 +5600,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Partial because drought is not covered as a distinct event-based hazard, only through the chronic water scarcity class</t>
+          <t>Partial because drought is not covered as a distinct event-based hazard, only through the chronic water scarcity class (GFDRR, no date a).</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5668,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Full because a dedicated landslide dataset underlies the classification; the value is delivered as a district-level class rather than as the underlying grid</t>
+          <t>Full because a dedicated landslide dataset underlies the classification; the value is delivered as a district-level class rather than as the underlying grid (World Bank and Global Facility for Disaster Reduction and Recovery, 2021).</t>
         </is>
       </c>
     </row>
@@ -5804,7 +5790,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Full because the daily fields at 1 km resolution allow a heavy-precipitation index to be derived directly; the source supplies the variable, the threshold definition rests with the institution</t>
+          <t>Full because the daily fields at 1 km resolution allow a heavy-precipitation index to be derived directly; the source supplies the variable, the threshold definition rests with the institution (GeoSphere Austria, no date a).</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5822,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Full because the daily fields at 1 km resolution allow a heatwave index to be derived directly; the source supplies the variables, the threshold definition rests with the institution</t>
+          <t>Full because the daily fields at 1 km resolution allow a heatwave index to be derived directly; the source supplies the variables, the threshold definition rests with the institution (GeoSphere Austria, no date a).</t>
         </is>
       </c>
     </row>
@@ -5886,7 +5872,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Partial because the fields support only a basic dryness proxy; no drought index is part of this dataset, and the dedicated index is published separately as WINFORE</t>
+          <t>Partial because the fields support only a basic dryness proxy; no drought index is part of this dataset, and the dedicated index is published separately as WINFORE (GeoSphere Austria, no date a).</t>
         </is>
       </c>
     </row>
@@ -6116,7 +6102,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Full because a dedicated, purpose-built drought index is provided at national 1 km resolution</t>
+          <t>Full because a dedicated, purpose-built drought index is provided at national 1 km resolution (GeoSphere Austria, no date b).</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6134,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>Partial because the climatic water balance is oriented towards drought and dryness, not towards water stress in the sense of demand relative to available supply</t>
+          <t>Partial because the climatic water balance is oriented towards drought and dryness, not towards water stress in the sense of demand relative to available supply (GeoSphere Austria, no date b).</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6202,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Full because all three flood processes are named individually and modelled at street level</t>
+          <t>Full because all three flood processes are named individually and modelled at street level (Climate X Ltd, no date a).</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6234,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Full because landslide is named individually among the modelled perils</t>
+          <t>Full because landslide is named individually among the modelled perils (Climate X Ltd, no date a).</t>
         </is>
       </c>
     </row>
@@ -6316,7 +6302,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Full because a windstorm peril is named among the modelled perils</t>
+          <t>Full because a windstorm peril is named among the modelled perils (Climate X Ltd, no date a).</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6352,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Partial because only the chronic heat metric is named; whether acute heatwave events are distinguished could not be established from the public documentation</t>
+          <t>Partial because only the chronic heat metric is named; whether acute heatwave events are distinguished could not be established from the public documentation (Climate X Ltd, no date a).</t>
         </is>
       </c>
     </row>
@@ -6398,7 +6384,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Full because extreme heat is named individually among the modelled perils</t>
+          <t>Full because extreme heat is named individually among the modelled perils (Climate X Ltd, no date a).</t>
         </is>
       </c>
     </row>
@@ -6415,10 +6401,24 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="D181" s="9" t="n"/>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="D181" s="9" t="inlineStr">
+        <is>
+          <t>Asset/facility level</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Combined drought / water stress peril of Spectra</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Partial because drought is named among the eleven physical risks but is combined with water stress into a single peril, so the two are not reported separately (Climate X Ltd, no date b).</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="45" customHeight="1" s="6">
       <c r="A182" t="inlineStr">
@@ -6433,10 +6433,24 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="D182" s="9" t="n"/>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="D182" s="9" t="inlineStr">
+        <is>
+          <t>Asset/facility level</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Combined drought / water stress peril of Spectra</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Partial because water stress is named among the eleven physical risks but is combined with drought into a single peril, so the two are not reported separately (Climate X Ltd, no date b).</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -6466,7 +6480,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Full because wildfire is named among the modelled perils</t>
+          <t>Full because wildfire is named among the modelled perils (Climate X Ltd, no date a).</t>
         </is>
       </c>
     </row>
@@ -6516,7 +6530,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Full because flood is named individually among the modelled perils and resolved at asset level</t>
+          <t>Full because flood is named individually among the modelled perils and resolved at asset level (Jupiter Intelligence, Inc., no date a).</t>
         </is>
       </c>
     </row>
@@ -6602,7 +6616,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Full because wind is named individually among the modelled perils</t>
+          <t>Full because wind is named individually among the modelled perils (Jupiter Intelligence, Inc., no date a).</t>
         </is>
       </c>
     </row>
@@ -6619,10 +6633,24 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="D190" s="9" t="n"/>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="D190" s="9" t="inlineStr">
+        <is>
+          <t>Asset/facility level</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Extreme and chronic precipitation perils of ClimateScore Global</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Full because extreme and prolonged precipitation are named among the modelled perils (Jupiter Intelligence, Inc., no date b).</t>
+        </is>
+      </c>
     </row>
     <row r="191" ht="30" customHeight="1" s="6">
       <c r="A191" t="inlineStr">
@@ -6652,7 +6680,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Full because heat is named individually among the modelled perils</t>
+          <t>Full because heat is named individually among the modelled perils (Jupiter Intelligence, Inc., no date a).</t>
         </is>
       </c>
     </row>
@@ -6684,7 +6712,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Partial because only a general heat peril is named; whether it distinguishes chronic heat stress from acute heatwave events could not be established from the public documentation</t>
+          <t>Partial because only a general heat peril is named; whether it distinguishes chronic heat stress from acute heatwave events could not be established from the public documentation (Jupiter Intelligence, Inc., no date a).</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6744,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>Full because drought is named individually among the modelled perils</t>
+          <t>Full because drought is named individually among the modelled perils (Jupiter Intelligence, Inc., no date a).</t>
         </is>
       </c>
     </row>
@@ -6733,10 +6761,24 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="D194" s="9" t="n"/>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="D194" s="9" t="inlineStr">
+        <is>
+          <t>Asset/facility level</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Water stress peril of ClimateScore Global</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Full because water stress is named as a separate peril, added to the platform alongside extreme cold (Jupiter Intelligence, Inc., no date b).</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -6766,7 +6808,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Full because wildfire is named individually among the modelled perils</t>
+          <t>Full because wildfire is named individually among the modelled perils (Jupiter Intelligence, Inc., no date a).</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6858,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Full because the indices are published as a ready-made dataset that can be requested directly; coverage is limited to riverine flooding</t>
+          <t>Full because the indices are published as a ready-made dataset that can be requested directly; coverage is limited to riverine flooding (Copernicus Climate Change Service, Climate Data Store, 2021).</t>
         </is>
       </c>
     </row>
@@ -6956,7 +6998,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Full because a peer-reviewed thermal-stress dataset is published in its own right; it is reanalysis-based only, with no projections available</t>
+          <t>Full because a peer-reviewed thermal-stress dataset is published in its own right; it is reanalysis-based only, with no projections available (Di Napoli et al., 2021).</t>
         </is>
       </c>
     </row>
@@ -6988,7 +7030,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Full for the soil-moisture component, which is published as a ready-made indicator; the meteorological SPI-3 component is not part of this dataset and must be derived from raw variables</t>
+          <t>Full for the soil-moisture component, which is published as a ready-made indicator; the meteorological SPI-3 component is not part of this dataset and must be derived from raw variables (Copernicus Climate Change Service, Climate Data Store, 2021).</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7062,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Full in the sense that a ready-made indicator is published; as with Climate-ADAPT it describes the climatic water balance rather than demand relative to supply</t>
+          <t>Full in the sense that a ready-made indicator is published; as with Climate-ADAPT it describes the climatic water balance rather than demand relative to supply (Copernicus Climate Change Service, Climate Data Store, 2021).</t>
         </is>
       </c>
     </row>
@@ -7133,7 +7175,7 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Climate-ADAPT is a public knowledge portal operated by the European Environment Agency (EEA) (EEA, n.d.). It provides pre-computed, peer-reviewed climate hazard indices via the European Climate Data Explorer (ECDE), covering heat, precipitation, flood, drought, storm and wildfire hazards at EU-wide scope and grid-based granularity (0.1-0.25 degrees, 5km for hydrology-based indices) (EEA/C3S, n.d.). The source is accessed through a web portal, a queryable API and direct download, and is free of charge.</t>
+          <t>Climate-ADAPT is a public knowledge portal operated by the European Environment Agency (EEA) (no date). It provides pre-computed, peer-reviewed climate hazard indices via the European Climate Data Explorer (ECDE), covering heat, precipitation, flood, drought, storm and wildfire hazards at EU-wide scope and grid-based granularity (0.1-0.25 degrees, 5km for hydrology-based indices) (The Climate Data Factory and B-Open et al., 2024). The source is accessed through a web portal, a queryable API and direct download, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7150,7 +7192,7 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>The Risk Data Hub (RDH) is a public multi-hazard risk and loss data platform operated by the Joint Research Centre (JRC) in cooperation with the EU Disaster Risk Management Knowledge Centre (DRMKC) (JRC DRMKC, n.d.). It provides modelled hazard, exposure and historical-loss data covering flood, landslide, earthquake, wildfire and subsidence at NUTS 2/3 granularity across EU, EFTA and IPA countries (Antofie et al., 2023). The source is accessed through a web portal, direct download and an API, and is free of charge.</t>
+          <t>The Risk Data Hub (RDH) is a public multi-hazard risk and loss data platform operated by the Joint Research Centre (JRC) in cooperation with the EU Disaster Risk Management Knowledge Centre (DRMKC) (Joint Research Centre / Disaster Risk Management Knowledge Centre, no date). It provides modelled hazard, exposure and historical-loss data covering flood, landslide, earthquake, wildfire and subsidence at NUTS 2/3 granularity across EU, EFTA and IPA countries (Antofie et al., 2023). The source is accessed through a web portal, direct download and an API, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7167,7 +7209,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>EFFIS (European Forest Fire Information System) is a public wildfire information service operated jointly by the JRC and the Copernicus Emergency Management Service (JRC/Copernicus EMS, n.d.). It provides a daily fire danger forecast and a historical burnt-area database covering wildfire hazard across Europe, the Middle East and North Africa at grid resolutions ranging from approximately 8-16km (forecast) to 250m/20m (observed burnt area) (EFFIS, n.d.-a). The source is accessed through an OGC map service (WMS/WFS) and direct download, and is free of charge.</t>
+          <t>EFFIS (European Forest Fire Information System) is a public wildfire information service operated jointly by the JRC and the Copernicus Emergency Management Service (Joint Research Centre and Copernicus Emergency Management Service et al., no date). It provides a daily fire danger forecast and a historical burnt-area database covering wildfire hazard across Europe, the Middle East and North Africa at grid resolutions ranging from approximately 8-16km (forecast) to 250m/20m (observed burnt area) (Copernicus Emergency Management Service / EFFIS, no date b). The source is accessed through an OGC map service (WMS/WFS) and direct download, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7184,7 +7226,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>The Copernicus Climate Data Store (CDS) is a public climate data repository operated by ECMWF on behalf of the EU (ECMWF, n.d.), comprising datasets of raw and derived climate variables together with reanalysis and projection data. It provides raw climate variables (e.g. temperature, precipitation, wind fields) covering multiple physical hazards at grid resolutions of roughly 0.1-0.25 degrees globally, with an EU focus. The source is accessed through a web portal, direct download and an API, and is free of charge.</t>
+          <t>The Copernicus Climate Data Store (CDS) is a public climate data repository operated by ECMWF on behalf of the EU (no date), comprising datasets of raw and derived climate variables together with reanalysis and projection data. It provides raw climate variables from the ERA5 reanalysis (Hersbach et al., 2023), such as temperature, precipitation, wind fields and soil temperature at four soil levels between 0 and 289 cm depth (ECMWF, 2026), covering multiple physical hazards at grid resolutions of roughly 0.1-0.25 degrees globally, with an EU focus. The source is accessed through a web portal, direct download and an API, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7201,7 +7243,7 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>The EBA ESG Dashboard is a public statistics dashboard operated by the European Banking Authority (EBA) (EBA, n.d.). It provides aggregated ESG risk indicators at EU bank level, covering both physical and transition climate risk at institution/portfolio-level granularity across the EU/EEA (EBA, n.d.). The source is accessed through a statistics dashboard, and is free of charge.</t>
+          <t>The EBA ESG Dashboard is a public statistics dashboard operated by the European Banking Authority (EBA) (no date). It provides aggregated ESG risk indicators at EU bank level, covering both physical and transition climate risk at institution/portfolio-level granularity across the EU/EEA (European Banking Authority, no date). The source is accessed through a statistics dashboard, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7218,7 +7260,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>This is a national flood extent dataset, published via the INSPIRE Geoportal Oesterreich, with the Bundesministerium fuer Land- und Forstwirtschaft, Klima- und Umweltschutz, Regionen und Wasserwirtschaft (BMLUK) as data owner and Umweltbundesamt GmbH as technical operator (data.gv.at, n.d.-b). It provides harmonised flood extent layers for the 30-, 100- and 300-year return periods, covering flood hazard at parcel/address-level granularity across Austria. The source is accessed through OGC WMS/WFS services and direct GML/shapefile download, and is free of charge.</t>
+          <t>This is a national flood extent dataset, published via the INSPIRE Geoportal Österreich, with the Bundesministerium fuer Land- und Forstwirtschaft, Klima- und Umweltschutz, Regionen und Wasserwirtschaft (BMLUK) as data owner and Umweltbundesamt GmbH as technical operator (Umweltbundesamt, 2020). It provides harmonised flood extent layers for the 30-, 100- and 300-year return periods, covering flood hazard at parcel/address-level granularity across Austria. The source is accessed through OGC WMS/WFS services and direct GML/shapefile download, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7235,7 +7277,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>The Gefahrenzonenplan (GZP) is a public national hazard zoning dataset operated by the Forsttechnischer Dienst fuer Wildbach- und Lawinenverbauung (Federal Ministry BMLUK) (data.gv.at, n.d.-a). It is a statutory area-wide expert assessment under the Forstgesetz 1975, covering hazards from torrents, avalanches and erosion and additionally depicting rockfall and landslide processes. Hazard zones are delineated as polygons by technical criteria, independently of parcel boundaries, and can therefore be intersected with parcel or address locations. Plans are drawn up for those municipalities that contain torrent, avalanche or erosion catchments, and cover the spatially relevant area within them. The source is accessed through an OGC map service (WMS/WFS) and direct download, and is free of charge.</t>
+          <t>The Gefahrenzonenplan (GZP) is a public national hazard zoning dataset operated by the Forsttechnischer Dienst fuer Wildbach- und Lawinenverbauung (Federal Ministry BMLUK) (Forsttechnischer Dienst für Wildbach- und Lawinenverbauung, no date). It is a statutory area-wide expert assessment under the Forstgesetz 1975, covering hazards from torrents, avalanches and erosion and additionally depicting rockfall and landslide processes. Hazard zones are delineated as polygons by technical criteria, independently of parcel boundaries, and can therefore be intersected with parcel or address locations. Plans are drawn up for those municipalities that contain torrent, avalanche or erosion catchments, and cover the spatially relevant area within them. The source is accessed through an OGC map service (WMS/WFS) and direct download, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7252,7 +7294,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>HORA (Natural Hazard Overview and Risk Assessment Austria) is a publicly accessible Austrian WebGIS application, operated by the Land-, Forst- und Wasserwirtschaftliche Rechenzentrum (LFRZ) on behalf of the responsible federal ministry (LFRZ, n.d.). It provides address- and cadastral-level initial information on natural hazards, currently covering flood, avalanche, earthquake, landslide, storm, lightning, hail and snow (BMLUK, n.d.), at parcel/address-level granularity across Austria (HORA, n.d.). The source is accessed through an interactive web interface via individual location queries, and is free to use.</t>
+          <t>HORA (Natural Hazard Overview and Risk Assessment Austria) is a publicly accessible Austrian WebGIS application, operated by the Land-, Forst- und Wasserwirtschaftliche Rechenzentrum (LFRZ) on behalf of the responsible federal ministry (Land-, forst- und wasserwirtschaftliches Rechenzentrum, no date). It provides address- and cadastral-level initial information on natural hazards, currently covering flood, avalanche, earthquake, landslide, storm, lightning, hail and snow (Bundesministerium für Land- und Forstwirtschaft, Klima- und Umweltschutz, Regionen und Wasserwirtschaft, no date), at parcel/address-level granularity across Austria (HORA, no date). The source is accessed through an interactive web interface via individual location queries, and is free to use.</t>
         </is>
       </c>
     </row>
@@ -7269,7 +7311,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>The Aqueduct Water Risk Atlas is a public water-risk dataset operated by the World Resources Institute (WRI) (WRI, n.d.-a). It provides 13 modelled indicators covering water stress, drought risk and riverine/coastal flood risk at sub-catchment (watershed) granularity globally (WRI, n.d.-b). The source is accessed through a web map portal, direct download and an API, and is free of charge.</t>
+          <t>The Aqueduct Water Risk Atlas is a public water-risk dataset operated by the World Resources Institute (WRI) (no date b). It provides 13 modelled indicators covering water stress, drought risk and riverine/coastal flood risk at sub-catchment (watershed) granularity globally (World Resources Institute, no date a). The source is accessed through a web map portal, direct download and an API, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7286,7 +7328,7 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>This is a commercial dataset operated by Moody's ESG Solutions (Moody's, n.d.-a). It provides proprietary modelled physical climate risk scores covering floods, heat stress, hurricanes and typhoons, sea-level rise, water stress and wildfires at facility/object-level granularity globally (Moody's, n.d.-b). The source is accessed through a commercial analytics platform and an API, and is paid.</t>
+          <t>This is a commercial dataset operated by Moody's ESG Solutions (no date b). It provides proprietary modelled physical climate risk scores covering floods, heat stress, hurricanes and typhoons, sea-level rise, water stress and wildfires at facility/object-level granularity globally (Moody's, no date a). The source is accessed through a commercial analytics platform and an API, and is paid.</t>
         </is>
       </c>
     </row>
@@ -7303,7 +7345,7 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>NATHAN Risk Suite is a commercial dataset operated by Munich Re (Munich Re, n.d.-a). It provides proprietary modelled natural hazard and climate scenario scores covering 15 hazards, including river flood, extratropical storm, wildfire and landslide, at facility/object-level granularity globally, with scenarios extending to 2100 (Munich Re, n.d.-b). The source is accessed through a commercial analytics platform and an API, and is paid.</t>
+          <t>NATHAN Risk Suite is a commercial dataset operated by Munich Re (no date). It provides proprietary modelled natural hazard and climate scenario scores covering 15 hazards, including river flood, extratropical storm, wildfire and landslide, at facility/object-level granularity globally, with scenarios extending to 2100 (Munich Re, Risk Management Partners, no date b). The source is accessed through a commercial analytics platform and an API, and is paid.</t>
         </is>
       </c>
     </row>
@@ -7320,7 +7362,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>ThinkHazard! is a free, open-source hazard screening tool operated by the Global Facility for Disaster Reduction and Recovery (GFDRR) in cooperation with the World Bank (GFDRR, n.d.-a). It classifies eleven natural hazards into four levels, from very low to high, for any location worldwide, and returns the maximum hazard level within the containing administrative unit at country, province or district level. Hazard levels are derived from published hazard layers harvested from the GFDRR GeoNode (GFDRR, n.d.-b); where several datasets exist for a region and hazard, a documented decision tree selects the layer to use. The tool is accessed through a web interface and a public API, and is free of charge. The landslide classification draws on the Global Landslide Hazard Map produced by Arup for the World Bank and GFDRR (World Bank/GFDRR/Arup, n.d.).</t>
+          <t>ThinkHazard! is a free, open-source hazard screening tool operated by the Global Facility for Disaster Reduction and Recovery (GFDRR) in cooperation with the World Bank (no date a). It classifies eleven natural hazards into four levels, from very low to high, for any location worldwide, and returns the maximum hazard level within the containing administrative unit at country, province or district level. Hazard levels are derived from published hazard layers harvested from the GFDRR GeoNode (no date b); where several datasets exist for a region and hazard, a documented decision tree selects the layer to use. The tool is accessed through a web interface and a public API, and is free of charge. The landslide classification draws on the Global Landslide Hazard Map produced by Arup for the World Bank and GFDRR (World Bank and Global Facility for Disaster Reduction and Recovery, 2021).</t>
         </is>
       </c>
     </row>
@@ -7337,7 +7379,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>This is a public register operated by Statistik Austria (Statistik Austria, n.d.). It provides the official OeNACE 2025 (NACE Rev. 2.1) economic-activity code for each Austrian company, keyed to the Firmenbuch number, covering the full national company register at entity-level granularity. The source is accessed through direct bulk download in CSV format, and is free of charge.</t>
+          <t>This is a public register operated by Statistik Austria (no date). It provides the official OeNACE 2025 (NACE Rev. 2.1) economic-activity code for each Austrian company, keyed to the Firmenbuch number, covering the full national company register at entity-level granularity. The source is accessed through direct bulk download in CSV format, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7396,7 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Wirtschafts-Compass is a commercial Austrian company-data service operated by Compass-Verlag GmbH (Compass-Verlag, n.d.-a). It provides an editorially enriched OeNACE classification per entity, covering the Austrian company landscape at entity-level granularity, delivered with daily currency. The source is accessed through an API and a web portal, and is paid.</t>
+          <t>Wirtschafts-Compass is a commercial Austrian company-data service operated by Compass-Verlag GmbH (no date b). It provides an editorially enriched OeNACE classification per entity, covering the Austrian company landscape at entity-level granularity, delivered with daily currency. The source is accessed through an API and a web portal, and is paid.</t>
         </is>
       </c>
     </row>
@@ -7371,7 +7413,7 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>SPARTACUS-v3 is a public gridded climate dataset operated by GeoSphere Austria, the Austrian federal institute for geology, geophysics, climatology and meteorology (GeoSphere Austria, n.d.-a). It provides observed daily, monthly and quarterly temperature, precipitation and sunshine-duration fields, covering heat and precipitation hazards at 1km grid granularity across Austria since 1961 (GeoSphere Austria, n.d.-a). The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge.</t>
+          <t>SPARTACUS-v3 is a public gridded climate dataset operated by GeoSphere Austria, the Austrian federal institute for geology, geophysics, climatology and meteorology (GeoSphere Austria, no date a). It provides observed daily, monthly and quarterly temperature, precipitation and sunshine-duration fields, covering heat and precipitation hazards at 1km grid granularity across Austria since 1961 (GeoSphere Austria, no date a). The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7388,7 +7430,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>WINFORE is a public gridded drought-index dataset operated by GeoSphere Austria (GeoSphere Austria, n.d.-b). It provides the Standardized Precipitation Evapotranspiration Index (SPEI) at 30-, 90- and 365-day aggregation, covering drought hazard at 1km grid granularity across Austria, derived from SPARTACUS temperature and precipitation fields. The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge.</t>
+          <t>WINFORE is a public gridded drought-index dataset operated by GeoSphere Austria (no date b). It provides the Standardized Precipitation Evapotranspiration Index (SPEI) at 30-, 90- and 365-day aggregation, covering drought hazard at 1km grid granularity across Austria, derived from SPARTACUS temperature and precipitation fields. The source is accessed through a web interface, a coordinate-based REST API and HTTP bulk download, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7405,7 +7447,7 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Spectra is a commercial physical climate risk platform operated by Climate X Ltd, a UK-based company founded in 2020 (Technology Tools, n.d.). It provides asset-level modelled physical hazard scores and financial loss projections across up to 16 hazards, including flooding, storms, heat stress, wildfires and landslides, at asset/facility-level granularity globally, with scenario projections to 2100 (Repath, n.d.). The source is accessed through a commercial SaaS platform and an API, and is paid.</t>
+          <t>Spectra is a commercial physical climate risk platform operated by Climate X Ltd, a UK-based company founded in 2020 (Technology Tools, no date). It provides asset-level modelled physical hazard scores and financial loss projections across up to 16 hazards, including flooding, storms, heat stress, wildfires and landslides, at asset/facility-level granularity globally, with scenario projections to 2100 (Repath, no date). The source is accessed through a commercial SaaS platform and an API, and is paid.</t>
         </is>
       </c>
     </row>
@@ -7422,7 +7464,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>ClimateScore Global is a commercial physical climate risk platform operated by Jupiter Intelligence, Inc., a US company founded in 2017 (aigreentools.com, n.d.). It provides asset-level modelled physical hazard scores and finance-grade loss metrics across 9 physical perils, including flood, heat, drought, tropical cyclones and wildfire, at asset/facility-level granularity globally, based on peer-reviewed CMIP6/ERA5 science (aigreentools.com, n.d.). The source is accessed through a commercial SaaS platform and an API, and is paid.</t>
+          <t>ClimateScore Global is a commercial physical climate risk platform operated by Jupiter Intelligence, Inc., a US company founded in 2017 (aigreentools.com, no date). It provides asset-level modelled physical hazard scores and finance-grade loss metrics across 9 physical perils, including flood, heat, drought, tropical cyclones and wildfire, at asset/facility-level granularity globally, based on peer-reviewed CMIP6/ERA5 science (aigreentools.com, no date). The source is accessed through a commercial SaaS platform and an API, and is paid.</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7481,7 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>This is a set of standalone, ready-made physical hazard indicator products, published as individual datasets on the Copernicus Climate Data Store (CDS), distinct from the general-purpose raw climate variables covered by the separate copernicus_cds entry (ECMWF, n.d.). It provides ERA5-HEAT (UTCI/heat stress) and the SMHI hydrology dataset (flood, water stress/aridity, soil-moisture drought), covering these four hazards at grid granularity across Europe (Di Napoli et al., 2021; SMHI/C3S, n.d.). The source is accessed through direct download and a queryable API, and is free of charge.</t>
+          <t>This is a set of standalone, ready-made physical hazard indicator products, published as individual datasets on the Copernicus Climate Data Store (CDS), distinct from the general-purpose raw climate variables covered by the separate copernicus_cds entry (ECMWF, no date). It provides ERA5-HEAT (UTCI/heat stress) and the SMHI hydrology dataset (flood, water stress/aridity, soil-moisture drought), covering these four hazards at grid granularity across Europe (Di Napoli et al., 2021; Copernicus Climate Change Service, Climate Data Store, 2021). The source is accessed through direct download and a queryable API, and is free of charge.</t>
         </is>
       </c>
     </row>
@@ -7456,7 +7498,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>The source is based on a statutory hazard assessment under the Forstgesetz, produced by the Forsttechnischer Dienst fuer Wildbach- und Lawinenverbauung (data.gv.at, n.d.-a). Known issues: the design event is an approximately 150-year return period; zones represent process boundaries rather than inundation lines and include erosion and sediment-transport processes, so they are not directly comparable to flood inundation areas such as HQ30/HQ100/HQ300.</t>
+          <t>The source is based on a statutory hazard assessment under the Forstgesetz, produced by the Forsttechnischer Dienst fuer Wildbach- und Lawinenverbauung (Forsttechnischer Dienst für Wildbach- und Lawinenverbauung, no date). Known issues: the design event is an approximately 150-year return period; zones represent process boundaries rather than inundation lines and include erosion and sediment-transport processes, so they are not directly comparable to flood inundation areas such as HQ30/HQ100/HQ300.</t>
         </is>
       </c>
     </row>
@@ -7473,7 +7515,7 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>The source is based on the official OeNACE 2025 (NACE Rev. 2.1) assignment maintained by Statistik Austria under section 21 of the Bundesstatistikgesetz (Statistik Austria, n.d.). This was independently verified through structural analysis of the 682 distinct codes: division 45 is absent (abolished in Rev. 2.1), classes 47.41-47.43 are absent (merged into 47.40), and class 46.89 is present (newly created in Rev. 2.1), confirming alignment with the revision required by Template D 01.01. Known issues: companies without an assigned code remain unmatched, and unregistered sole traders are out of scope.</t>
+          <t>The source is based on the official OeNACE 2025 (NACE Rev. 2.1) assignment maintained by Statistik Austria under section 21 of the Bundesstatistikgesetz (no date). This was independently verified through structural analysis of the 682 distinct codes: division 45 is absent (abolished in Rev. 2.1), classes 47.41-47.43 are absent (merged into 47.40), and class 46.89 is present (newly created in Rev. 2.1), confirming alignment with the revision required by Template D 01.01. Known issues: companies without an assigned code remain unmatched, and unregistered sole traders are out of scope.</t>
         </is>
       </c>
     </row>
@@ -7490,7 +7532,7 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Hazard levels are not modelled by the tool itself but derived from third-party hazard layers, which are reviewed by GFDRR specialists and rated by age, methodology, assumptions and resolution before selection. Classification thresholds are documented in the published methodology report (GFDRR, n.d.-a), for example river flood is classified from the frequency at which at least one per cent of the administrative unit is flooded to a depth of 0.5 metres or more. The provenance of the selected layer is disclosed per hazard and country, so the origin of a given classification can be traced.</t>
+          <t>Hazard levels are not modelled by the tool itself but derived from third-party hazard layers, which are reviewed by GFDRR specialists and rated by age, methodology, assumptions and resolution before selection. Classification thresholds are documented in the published methodology report (GFDRR, no date a), for example river flood is classified from the frequency at which at least one per cent of the administrative unit is flooded to a depth of 0.5 metres or more. The provenance of the selected layer is disclosed per hazard and country, so the origin of a given classification can be traced.</t>
         </is>
       </c>
     </row>
@@ -7507,7 +7549,7 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>The source is based on two distinct production chains: the fire danger forecast is numerical-weather-model output (ECMWF/MeteoFrance), while the burnt-area database is satellite-derived (MODIS/Sentinel-2) and manually validated by the EFFIS network of national fire experts (JRC/Copernicus EMS, n.d.). Known issues: the burnt-area database has a minimum mapped fire size of 30 hectares, excluding smaller fires, and EFFIS is organisationally distinct from the CEMS Fire Danger historical dataset hosted separately on the CDS, which covers meteorological reconstruction only, not observed fire events.</t>
+          <t>The source is based on two distinct production chains: the fire danger forecast is numerical-weather-model output (ECMWF/MeteoFrance), while the burnt-area database is satellite-derived (MODIS/Sentinel-2) and manually validated by the EFFIS network of national fire experts (Joint Research Centre and Copernicus Emergency Management Service et al., no date). Known issues: the burnt-area database has a minimum mapped fire size of 30 hectares, excluding smaller fires, and EFFIS is organisationally distinct from the CEMS Fire Danger historical dataset hosted separately on the CDS, which covers meteorological reconstruction only, not observed fire events.</t>
         </is>
       </c>
     </row>
@@ -7524,7 +7566,7 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>The source is based on the ECDE indicator set, computed by the Climate Data Factory and B-Open under a C3S service contract from established EURO-CORDEX/ERA5 climate projections, with each index individually documented and traceable to the peer-reviewed methodology paper on which it is based (EEA/C3S, n.d.); the Climatological Heatwave Days index, for instance, follows the EURO-CORDEX definition of Jacob et al. (2013); historical fire-danger values come from the CEMS fire danger indices dataset (ECMWF/CEMS, n.d.). Known issues: the EEA's own summary report table resolves only to European macro-regions, while the underlying indicator dataset itself is considerably finer; resolution varies by indicator from 5km to approximately 28km (EEA/C3S, n.d.).</t>
+          <t>The source is based on the ECDE indicator set, computed by the Climate Data Factory and B-Open under a C3S service contract from established EURO-CORDEX/ERA5 climate projections, with each index individually documented and traceable to the peer-reviewed methodology paper on which it is based (The Climate Data Factory and B-Open et al., 2024); the Climatological Heatwave Days index, for instance, follows the EURO-CORDEX definition of Jacob et al. (2013); historical fire-danger values come from the CEMS fire danger indices dataset (Copernicus Climate Change Service, Climate Data Store, 2019). Known issues: the EEA's own summary report table resolves only to European macro-regions, while the underlying indicator dataset itself is considerably finer; resolution varies by indicator from 5km to approximately 28km (The Climate Data Factory and B-Open et al., 2024).</t>
         </is>
       </c>
     </row>
@@ -7558,7 +7600,7 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>The source is based primarily on ERA5 reanalysis and EURO-CORDEX climate projections, produced by ECMWF and national contributing centres under C3S and documented through peer-reviewed literature and individual CDS catalogue entries (ECMWF, n.d.). Known issues: quality, vintage and resolution vary considerably across the more than 140 datasets hosted on the CDS, so no single quality statement applies uniformly - each dataset must be assessed on its own documentation.</t>
+          <t>The source is based primarily on ERA5 reanalysis and EURO-CORDEX climate projections, produced by ECMWF and national contributing centres under C3S and documented through peer-reviewed literature and individual CDS catalogue entries (ECMWF, no date). Known issues: quality, vintage and resolution vary considerably across the more than 140 datasets hosted on the CDS, so no single quality statement applies uniformly - each dataset must be assessed on its own documentation.</t>
         </is>
       </c>
     </row>
@@ -7575,7 +7617,7 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>The source is based on aggregated supervisory data compiled by the European Banking Authority from EU/EEA banks' regulatory reporting, with the underlying methodology documented in the EBA's risk dashboard technical notes (EBA, n.d.). Known issues: aggregation to EU bank-level obscures any institution- or exposure-level variation entirely, since the dashboard was not designed for granular or per-exposure use.</t>
+          <t>The source is based on aggregated supervisory data compiled by the European Banking Authority from EU/EEA banks' regulatory reporting, with the underlying methodology documented in the EBA's risk dashboard technical notes (European Banking Authority, no date). Known issues: aggregation to EU bank-level obscures any institution- or exposure-level variation entirely, since the dashboard was not designed for granular or per-exposure use.</t>
         </is>
       </c>
     </row>
@@ -7592,7 +7634,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>The source is based on a composite of Abflussuntersuchungen (ABU), HORA and BWV/WLV hazard-zoning inputs, published via the INSPIRE Geoportal with BMLUK as data owner (data.gv.at, n.d.-b). Known issues: the Datenstand is October 2020, roughly six years old as of this review, and the underlying component datasets may carry inconsistent vintages, since they are separately maintained and merged into a single layer.</t>
+          <t>The source is based on a composite of Abflussuntersuchungen (ABU), HORA and BWV/WLV hazard-zoning inputs, published via the INSPIRE Geoportal with BMLUK as data owner (Umweltbundesamt, 2020). Known issues: the Datenstand is October 2020, roughly six years old as of this review, and the underlying component datasets may carry inconsistent vintages, since they are separately maintained and merged into a single layer.</t>
         </is>
       </c>
     </row>
@@ -7609,7 +7651,7 @@
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>The source is based on a compilation of multiple underlying Austrian hazard datasets (flood, earthquake, storm, hail, snow), presented by the operator explicitly as initial screening information rather than a validated legal assessment (LFRZ, n.d.). Known issues: the operator itself states that the map content is not legally binding, and the vintage of the individual underlying hazard layers per query is not disclosed to the user.</t>
+          <t>The source is based on a compilation of multiple underlying Austrian hazard datasets (flood, earthquake, storm, hail, snow), presented by the operator explicitly as initial screening information rather than a validated legal assessment (Land-, forst- und wasserwirtschaftliches Rechenzentrum, no date). Known issues: the operator itself states that the map content is not legally binding, and the vintage of the individual underlying hazard layers per query is not disclosed to the user.</t>
         </is>
       </c>
     </row>
@@ -7626,7 +7668,7 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>The source is based on the Aqueduct 4.0 modelled water-risk framework, produced by the World Resources Institute using global hydrological models with a publicly documented methodology (WRI, n.d.-b). Known issues: as a global model, it is not locally calibrated or independently validated specifically for Austria, and watershed-level aggregation may obscure local variation within a single sub-catchment.</t>
+          <t>The source is based on the Aqueduct 4.0 modelled water-risk framework, produced by the World Resources Institute using global hydrological models with a publicly documented methodology (World Resources Institute, no date a). Known issues: as a global model, it is not locally calibrated or independently validated specifically for Austria, and watershed-level aggregation may obscure local variation within a single sub-catchment.</t>
         </is>
       </c>
     </row>
@@ -7643,7 +7685,7 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>The source is based on proprietary modelled physical risk scores, originally developed by Four Twenty Seven, Inc. and now operated by Moody's ESG Solutions following the 2019 acquisition (Moody's, n.d.-b). Known issues: the underlying methodology is not fully transparent or independently validated, as is typical for proprietary commercial risk models, and confirmed Austria-relevant hazard coverage is narrower than the product's general marketing suggests.</t>
+          <t>The source is based on proprietary modelled physical risk scores, originally developed by Four Twenty Seven, Inc. and now operated by Moody's ESG Solutions following the 2019 acquisition (no date a). Known issues: the underlying methodology is not fully transparent or independently validated, as is typical for proprietary commercial risk models, and confirmed Austria-relevant hazard coverage is narrower than the product's general marketing suggests.</t>
         </is>
       </c>
     </row>
@@ -7660,7 +7702,7 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>The source is based on proprietary modelled natural hazard and climate scenario scores, produced by Munich Re, a reinsurer with decades of natural-catastrophe modelling experience (Munich Re, n.d.-b). Known issues: the underlying methodology is not fully public and independent third-party validation is limited; only the 15 explicitly named Natural Hazards Edition hazards are confirmed, while heat, drought and water-stress coverage under the separate 'Climate Change Edition' could not be individually verified.</t>
+          <t>The source is based on proprietary modelled natural hazard and climate scenario scores, produced by Munich Re, a reinsurer with decades of natural-catastrophe modelling experience (Munich Re, Risk Management Partners, no date b). Known issues: the underlying methodology is not fully public and independent third-party validation is limited; only the 15 explicitly named Natural Hazards Edition hazards are confirmed, while heat, drought and water-stress coverage under the separate 'Climate Change Edition' could not be individually verified.</t>
         </is>
       </c>
     </row>
@@ -7677,7 +7719,7 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>The source is based on editorially compiled and enriched company data, produced by Compass-Verlag GmbH, a long-established Austrian commercial business-information provider (Compass-Verlag, n.d.-a). Known issues: as an editorial rather than official classification, its methodology is not independently published or peer-reviewed, and individual entries may diverge from the official Statistik Austria HVD assignment - cross-validation against HVD is advisable where feasible.</t>
+          <t>The source is based on editorially compiled and enriched company data, produced by Compass-Verlag GmbH, a long-established Austrian commercial business-information provider (no date b). Known issues: as an editorial rather than official classification, its methodology is not independently published or peer-reviewed, and individual entries may diverge from the official Statistik Austria HVD assignment - cross-validation against HVD is advisable where feasible.</t>
         </is>
       </c>
     </row>
@@ -7694,7 +7736,7 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>The source is based on gridded observational climate data produced by GeoSphere Austria from station measurements interpolated to a 1km grid, with the methodology documented in peer-reviewed literature and in operational use since 1961 (GeoSphere Austria, n.d.-a). Known issues: the interpolation process introduces some uncertainty in data-sparse high-alpine regions, and the most recent seven days of data are provisional pending final quality control.</t>
+          <t>The source is based on gridded observational climate data produced by GeoSphere Austria from station measurements interpolated to a 1km grid, with the methodology documented in peer-reviewed literature and in operational use since 1961 (GeoSphere Austria, no date a). Known issues: the interpolation process introduces some uncertainty in data-sparse high-alpine regions, and the most recent seven days of data are provisional pending final quality control.</t>
         </is>
       </c>
     </row>
@@ -7711,7 +7753,7 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>The source is based on the SPEI drought index, derived from SPARTACUS temperature and precipitation fields using an established statistical methodology (a normal-distribution transform over defined climate reference periods), standard in the international drought-monitoring literature (GeoSphere Austria, n.d.-b). Known issues: as a standardised anomaly index, SPEI requires correct interpretation relative to its reference period rather than being read as an absolute water deficit.</t>
+          <t>The source is based on the SPEI drought index, derived from SPARTACUS temperature and precipitation fields using an established statistical methodology (a normal-distribution transform over defined climate reference periods), standard in the international drought-monitoring literature (GeoSphere Austria, no date b). Known issues: as a standardised anomaly index, SPEI requires correct interpretation relative to its reference period rather than being read as an absolute water deficit.</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7770,7 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>The source is based on proprietary modelled asset-level physical risk scores, produced by Climate X Ltd, a UK-based climate-risk analytics company founded in 2020 (Technology Tools, n.d.). Known issues: neither the full methodology nor the complete hazard list is published by the operator directly, and no independent third-party validation was identified; pricing and hazard-list completeness rely on third-party industry sources rather than operator confirmation.</t>
+          <t>The source is based on proprietary modelled asset-level physical risk scores, produced by Climate X Ltd, a UK-based climate-risk analytics company founded in 2020 (Technology Tools, no date). Known issues: neither the full methodology nor the complete hazard list is published by the operator directly, and no independent third-party validation was identified; pricing and hazard-list completeness rely on third-party industry sources rather than operator confirmation.</t>
         </is>
       </c>
     </row>
@@ -7745,7 +7787,7 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>The source is based on proprietary modelled asset-level physical risk and financial-loss metrics, produced by Jupiter Intelligence, Inc. from peer-reviewed CMIP6/ERA5 climate science (aigreentools.com, n.d.). Known issues: while the underlying climate science is peer-reviewed and publicly documented, the proprietary loss-translation methodology is not independently validated, and the only available pricing indication is a single CEO interview statement rather than a published price list.</t>
+          <t>The source is based on proprietary modelled asset-level physical risk and financial-loss metrics, produced by Jupiter Intelligence, Inc. from peer-reviewed CMIP6/ERA5 climate science (aigreentools.com, no date). Known issues: while the underlying climate science is peer-reviewed and publicly documented, the proprietary loss-translation methodology is not independently validated, and the only available pricing indication is a single CEO interview statement rather than a published price list.</t>
         </is>
       </c>
     </row>
@@ -7762,7 +7804,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>The source comprises two named, quality-controlled products: ERA5-HEAT, peer-reviewed and produced by ECMWF (Di Napoli et al., 2021), and the SMHI hydrology dataset, produced and quality-assured by the Swedish Meteorological and Hydrological Institute for C3S (SMHI/C3S, n.d.). Known issues: the SMHI hydrology projections are static 30-year model outputs rather than continuously updated, so their currency should be checked against the stated reference period before use.</t>
+          <t>The source comprises two named, quality-controlled products: ERA5-HEAT, peer-reviewed and produced by ECMWF (Di Napoli et al., 2021), and the SMHI hydrology dataset, produced and quality-assured by the Swedish Meteorological and Hydrological Institute for C3S (Copernicus Climate Change Service, Climate Data Store, 2021). Known issues: the SMHI hydrology projections are static 30-year model outputs rather than continuously updated, so their currency should be checked against the stated reference period before use.</t>
         </is>
       </c>
     </row>
@@ -8119,7 +8161,7 @@
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>download: Shapefile (vector, burnt-area perimeters), GeoTIFF (raster) - resolution differs by product: 250m (MODIS-based burnt area), 20m (Sentinel-2-based burnt area), ~8-16km (fire danger forecast, ECMWF/MeteoFrance model grid).</t>
+          <t>download: Shapefile (vector, burnt-area perimeters), GeoTIFF (raster) - resolution differs by product: 250m (MODIS-based burnt area), 20m (Sentinel-2-based burnt area), ~8-16km (fire danger forecast, ECMWF/MeteoFrance model grid) (Rosadi et al., 2023).</t>
         </is>
       </c>
     </row>
@@ -8306,7 +8348,7 @@
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>The source is available under the same CC-BY 4.0 licence that applies to the underlying Copernicus Climate Data Store since 2 July 2025 (ECMWF Forum, 2025). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
+          <t>The source is available under the same CC-BY 4.0 licence that applies to the underlying Copernicus Climate Data Store since 2 July 2025 (ECMWF Support, ECMWF Forum, 2025). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
         </is>
       </c>
     </row>
@@ -8323,7 +8365,7 @@
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>The source is available under an open EU data licence with attribution required, consistent with JRC's general data-sharing terms (JRC DRMKC, n.d.). The licence permits commercial use and systematic portfolio processing, provided that the source is appropriately credited.</t>
+          <t>The source is available under an open EU data licence with attribution required, consistent with JRC's general data-sharing terms (Joint Research Centre / Disaster Risk Management Knowledge Centre, no date). The licence permits commercial use and systematic portfolio processing, provided that the source is appropriately credited.</t>
         </is>
       </c>
     </row>
@@ -8340,7 +8382,7 @@
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>The source is available under a CC BY 4.0 licence, as confirmed on EFFIS's own dedicated data-licence page (EFFIS, n.d.-b). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
+          <t>The source is available under a CC BY 4.0 licence, as confirmed on EFFIS's own dedicated data-licence page (Copernicus Emergency Management Service / EFFIS, no date a). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
         </is>
       </c>
     </row>
@@ -8357,7 +8399,7 @@
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>The source is available under CC-BY 4.0 since 2 July 2025, replacing the previous bespoke "Licence to Use Copernicus Products" (Version 1.2, Nov 2019; ECMWF, 2019) that governed CDS access before that date (ECMWF Forum, 2025). Attribution is required when the data is reused. Individual sub-datasets may carry stricter third-party terms and should be verified per dataset before use.</t>
+          <t>The source is available under CC-BY 4.0 since 2 July 2025, replacing the previous bespoke "Licence to Use Copernicus Products" (Version 1.2, Nov 2019; European Union / ECMWF, 2019) that governed CDS access before that date (ECMWF Support, ECMWF Forum, 2025). Attribution is required when the data is reused. Individual sub-datasets may carry stricter third-party terms and should be verified per dataset before use.</t>
         </is>
       </c>
     </row>
@@ -8374,7 +8416,7 @@
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>The source is available under the EBA's standard open-data terms, free of charge and without registration (EBA, n.d.). No restrictions on commercial or systematic use beyond standard attribution practice were identified.</t>
+          <t>The source is available under the EBA's standard open-data terms, free of charge and without registration (European Banking Authority, no date). No restrictions on commercial or systematic use beyond standard attribution practice were identified.</t>
         </is>
       </c>
     </row>
@@ -8391,7 +8433,7 @@
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>The source is available under a CC BY 4.0 licence (data.gv.at, n.d.-b). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
+          <t>The source is available under a CC BY 4.0 licence (Umweltbundesamt, 2020). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
         </is>
       </c>
     </row>
@@ -8425,7 +8467,7 @@
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>The source is subject to specific terms of use that restrict bulk download and automated access (LFRZ, n.d.); the service is intended for individual location queries only. A separate agreement with the operator would be required for systematic portfolio-level use or regulatory reporting purposes.</t>
+          <t>The source is subject to specific terms of use that restrict bulk download and automated access (Land-, forst- und wasserwirtschaftliches Rechenzentrum, no date); the service is intended for individual location queries only. A separate agreement with the operator would be required for systematic portfolio-level use or regulatory reporting purposes.</t>
         </is>
       </c>
     </row>
@@ -8442,7 +8484,7 @@
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>The source is described by the operator as free and openly accessible for any application, with attribution requested (WRI, n.d.-a). No formally stated open licence name was identified on the operator's own materials, and no commercial-use restriction was found.</t>
+          <t>The source is described by the operator as free and openly accessible for any application, with attribution requested (World Resources Institute, no date b). No formally stated open licence name was identified on the operator's own materials, and no commercial-use restriction was found.</t>
         </is>
       </c>
     </row>
@@ -8459,7 +8501,7 @@
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>The source is subject to a commercial licence agreement (Moody's, n.d.-a). Access terms, API scope and portfolio size limits depend on the specific subscription negotiated with Moody's. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
+          <t>The source is subject to a commercial licence agreement (Moody's, no date b). Access terms, API scope and portfolio size limits depend on the specific subscription negotiated with Moody's. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
         </is>
       </c>
     </row>
@@ -8527,7 +8569,7 @@
       </c>
       <c r="C87" s="9" t="inlineStr">
         <is>
-          <t>The source is subject to a commercial licence agreement (Compass-Verlag, n.d.-c). Standard access is pay-per-query with published pricing; institutional API access terms depend on the specific subscription. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
+          <t>The source is subject to a commercial licence agreement (Compass-Verlag GmbH, via Wirtschaftskammer Österreich, no date). Standard access is pay-per-query with published pricing; institutional API access terms depend on the specific subscription. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
         </is>
       </c>
     </row>
@@ -8544,7 +8586,7 @@
       </c>
       <c r="C88" s="9" t="inlineStr">
         <is>
-          <t>The source is available under the Creative Commons Public Domain Dedication (CC0 1.0), per GeoSphere Austria's own repository documentation (GeoSphere Austria/re3data, n.d.), free for any use including commercial. No attribution is legally required, though it is good practice. The licence permits systematic portfolio processing.</t>
+          <t>The source is available under the Creative Commons Public Domain Dedication (CC0 1.0), per GeoSphere Austria's own repository documentation (re3data.org / GeoSphere Austria, no date), free for any use including commercial. No attribution is legally required, though it is good practice. The licence permits systematic portfolio processing.</t>
         </is>
       </c>
     </row>
@@ -8578,7 +8620,7 @@
       </c>
       <c r="C90" s="9" t="inlineStr">
         <is>
-          <t>The source is subject to a commercial licence agreement, quote-based, with no public price list (Net Zero Compare, n.d.). Access terms and portfolio size limits depend on the specific subscription negotiated. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
+          <t>The source is subject to a commercial licence agreement, quote-based, with no public price list (Net Zero Compare, 2025). Access terms and portfolio size limits depend on the specific subscription negotiated. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
         </is>
       </c>
     </row>
@@ -8595,7 +8637,7 @@
       </c>
       <c r="C91" s="9" t="inlineStr">
         <is>
-          <t>The source is subject to a commercial licence agreement, quote-based and defined case-by-case with the client (Mitiga Solutions, n.d.). Access terms and portfolio size limits depend on the specific subscription negotiated. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
+          <t>The source is subject to a commercial licence agreement, quote-based and defined case-by-case with the client (Mitiga Solutions, no date). Access terms and portfolio size limits depend on the specific subscription negotiated. The licence terms should be reviewed specifically for D 01.01 reporting use cases.</t>
         </is>
       </c>
     </row>
@@ -8612,7 +8654,7 @@
       </c>
       <c r="C92" s="9" t="inlineStr">
         <is>
-          <t>The source is available under CC-BY 4.0 since 2 July 2025, the same licence as copernicus_cds (ECMWF Forum, 2025), replacing the prior "Licence to Use Copernicus Products" (Version 1.2, Nov 2019; ECMWF, 2019). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
+          <t>The source is available under CC-BY 4.0 since 2 July 2025, the same licence as copernicus_cds (ECMWF Support, ECMWF Forum, 2025), replacing the prior "Licence to Use Copernicus Products" (Version 1.2, Nov 2019; European Union / ECMWF, 2019). Attribution is required when the data is reused. The licence permits commercial use and systematic portfolio processing.</t>
         </is>
       </c>
     </row>
@@ -8629,7 +8671,7 @@
       </c>
       <c r="C93" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is that heat stress and water stress are only covered via indirect proxies (UTCI; aridity), not dedicated indicators (EEA, 2021). In particular, these two proxies were not designed as hazard-specific indices and require careful interpretation before being treated as equivalent to the source's genuinely dedicated indices for heat wave, flood, drought, storm and wildfire. Consequently, the proxy-based hazards cannot be used with the same confidence as the dedicated ones, unless cross-checked against a hazard-specific source.</t>
+          <t>The main limitation is that heat stress and water stress are only covered via indirect proxies (UTCI; aridity), not dedicated indicators (European Environment Agency, 2021). In particular, these two proxies were not designed as hazard-specific indices and require careful interpretation before being treated as equivalent to the source's genuinely dedicated indices for heat wave, flood, drought, storm and wildfire. Consequently, the proxy-based hazards cannot be used with the same confidence as the dedicated ones, unless cross-checked against a hazard-specific source.</t>
         </is>
       </c>
     </row>
@@ -8697,7 +8739,7 @@
       </c>
       <c r="C97" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is that the source provides only aggregate EU bank-level statistics (EBA, n.d.). In particular, no download or API access exists and no per-exposure data is available whatsoever. Consequently, the source cannot be used to populate any individual exposure in D 01.01, unless it is used purely for peer-comparison or benchmarking purposes.</t>
+          <t>The main limitation is that the source provides only aggregate EU bank-level statistics (European Banking Authority, no date). In particular, no download or API access exists and no per-exposure data is available whatsoever. Consequently, the source cannot be used to populate any individual exposure in D 01.01, unless it is used purely for peer-comparison or benchmarking purposes.</t>
         </is>
       </c>
     </row>
@@ -8731,7 +8773,7 @@
       </c>
       <c r="C99" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is that hazards are mapped only within areas of spatial relevance (INSPIRE Geoportal Oesterreich, n.d.), meaning settled parts of a municipality with designated torrent or avalanche catchments (data.gv.at, n.d.-a). In particular, some zone plans remain available only in analogue form, and a portfolio location without a mapped result is ambiguous - it may indicate no hazard or simply no mapping. Consequently, the source cannot be used to conclusively rule out hazard for unmapped locations, unless cross-checked against the underlying zone-plan status.</t>
+          <t>The main limitation is that hazards are mapped only within areas of spatial relevance (INSPIRE Geoportal Österreich, no date), meaning settled parts of a municipality with designated torrent or avalanche catchments (Forsttechnischer Dienst für Wildbach- und Lawinenverbauung, no date). In particular, some zone plans remain available only in analogue form, and a portfolio location without a mapped result is ambiguous - it may indicate no hazard or simply no mapping. Consequently, the source cannot be used to conclusively rule out hazard for unmapped locations, unless cross-checked against the underlying zone-plan status.</t>
         </is>
       </c>
     </row>
@@ -8748,7 +8790,7 @@
       </c>
       <c r="C100" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is the restricted use of the service for systematic portfolio-level analysis (LFRZ, n.d.). In particular, the source is designed primarily for individual location queries and does not provide unrestricted bulk download or a documented portfolio-level API, and the displayed information is intended as initial risk information rather than a legally binding assessment. Consequently, HORA cannot be used as the sole source for automated classification of an entire loan portfolio, unless a separate access agreement is obtained from the operator. Pluvial flooding is not covered: heavy rain appears only as a current weather warning, not as an area-wide hazard layer, so surface-water flooding away from watercourses cannot be assessed with this source.</t>
+          <t>The main limitation is the restricted use of the service for systematic portfolio-level analysis (Land-, forst- und wasserwirtschaftliches Rechenzentrum, no date). In particular, the source is designed primarily for individual location queries and does not provide unrestricted bulk download or a documented portfolio-level API, and the displayed information is intended as initial risk information rather than a legally binding assessment. Consequently, HORA cannot be used as the sole source for automated classification of an entire loan portfolio, unless a separate access agreement is obtained from the operator. Pluvial flooding is not covered: heavy rain appears only as a current weather warning, not as an area-wide hazard layer, so surface-water flooding away from watercourses cannot be assessed with this source.</t>
         </is>
       </c>
     </row>
@@ -8782,7 +8824,7 @@
       </c>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is that confirmed Austria-relevant coverage is narrower than the product's general marketing suggests (Moody's, n.d.-b). In particular, storm is modelled as tropical cyclones specifically, which does not affect Austria, and a distinct heat-wave product plus drought coverage could not be confirmed at all. Consequently, the source cannot be relied upon for storm, heat-wave or drought classification of Austrian exposures, unless the operator confirms specific coverage directly.</t>
+          <t>The main limitation is that confirmed Austria-relevant coverage is narrower than the product's general marketing suggests (Moody's, no date a). In particular, the wind hazard is modelled as hurricanes and typhoons, that is tropical cyclones, while extratropical windstorms - the relevant wind process for Austria - are not among the six hazards, and sea level rise is irrelevant for a landlocked country, which does not affect Austria, and a distinct heat-wave product plus drought coverage could not be confirmed at all. Consequently, the source cannot be relied upon for storm, heat-wave or drought classification of Austrian exposures, unless the operator confirms specific coverage directly.</t>
         </is>
       </c>
     </row>
@@ -8799,7 +8841,7 @@
       </c>
       <c r="C103" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is that heat, drought and water stress coverage could not be confirmed by name (Munich Re, n.d.-b). In particular, these hazards are only advertised via a separate, unnamed 'Climate Change Edition' covering '13 climate hazards' without individual naming in the materials reviewed. Consequently, the source cannot be relied upon for heat, drought or water stress classification with the same confidence as its 15 named Natural Hazards Edition hazards, unless the operator confirms specific coverage directly.</t>
+          <t>The main limitation is that heat, drought and water stress coverage could not be confirmed by name (Munich Re, Risk Management Partners, no date b). In particular, these hazards are only advertised via a separate, unnamed 'Climate Change Edition' covering '13 climate hazards' without individual naming in the materials reviewed. Consequently, the source cannot be relied upon for heat, drought or water stress classification with the same confidence as its 15 named Natural Hazards Edition hazards, unless the operator confirms specific coverage directly.</t>
         </is>
       </c>
     </row>
@@ -8833,7 +8875,7 @@
       </c>
       <c r="C105" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is incomplete company coverage (Statistik Austria, n.d.). In particular, companies without an assigned OeNACE code remain unmatched, and unregistered sole traders are out of scope of the Firmenbuch-based register. Consequently, the source cannot classify every possible counterparty in an SNCI's loan portfolio, unless a complementary source is used for the unmatched residual.</t>
+          <t>The main limitation is incomplete company coverage (Statistik Austria, no date). In particular, companies without an assigned OeNACE code remain unmatched, and unregistered sole traders are out of scope of the Firmenbuch-based register. Consequently, the source cannot classify every possible counterparty in an SNCI's loan portfolio, unless a complementary source is used for the unmatched residual.</t>
         </is>
       </c>
     </row>
@@ -8850,7 +8892,7 @@
       </c>
       <c r="C106" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is that the classification is editorially enriched rather than the official statistical assignment (Compass-Verlag, n.d.-a). In particular, cost is institution-dependent, since some banks may already hold a sector licence while others would face a new subscription cost. Consequently, the source cannot be treated as an authoritative regulatory reference on the same footing as the official HVD dataset, unless used alongside HVD for cross-validation.</t>
+          <t>The main limitation is that the classification is editorially enriched rather than the official statistical assignment (Compass-Verlag GmbH, no date b). In particular, cost is institution-dependent, since some banks may already hold a sector licence while others would face a new subscription cost. Consequently, the source cannot be treated as an authoritative regulatory reference on the same footing as the official HVD dataset, unless used alongside HVD for cross-validation.</t>
         </is>
       </c>
     </row>
@@ -8867,7 +8909,7 @@
       </c>
       <c r="C107" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is that the source provides raw climate variables, not a pre-classified hazard or risk score (GeoSphere Austria, n.d.-a). In particular, converting temperature or precipitation fields into a heat-wave or heavy-precipitation exposure indicator requires the institution's own threshold definition. Consequently, the source cannot be used directly for exposure classification, unless the bank first defines and validates its own index methodology.</t>
+          <t>The main limitation is that the source provides raw climate variables, not a pre-classified hazard or risk score (GeoSphere Austria, no date a). In particular, converting temperature or precipitation fields into a heat-wave or heavy-precipitation exposure indicator requires the institution's own threshold definition. Consequently, the source cannot be used directly for exposure classification, unless the bank first defines and validates its own index methodology.</t>
         </is>
       </c>
     </row>
@@ -8884,7 +8926,7 @@
       </c>
       <c r="C108" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is that SPEI is a standardised statistical anomaly index, not an absolute water-deficit value (GeoSphere Austria, n.d.-b). In particular, it is derived via a normal-distribution transform over two climate reference periods, so its interpretation requires understanding this transform rather than reading a direct precipitation deficit. Consequently, the source cannot be interpreted at face value without methodological context, unless the reporting institution documents the SPEI transform in its own methodology notes.</t>
+          <t>The main limitation is that SPEI is a standardised statistical anomaly index, not an absolute water-deficit value (GeoSphere Austria, no date b). In particular, it is derived via a normal-distribution transform over two climate reference periods, so its interpretation requires understanding this transform rather than reading a direct precipitation deficit. Consequently, the source cannot be interpreted at face value without methodological context, unless the reporting institution documents the SPEI transform in its own methodology notes.</t>
         </is>
       </c>
     </row>
@@ -8901,7 +8943,7 @@
       </c>
       <c r="C109" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is that pricing and the full hazard list are not published by the operator directly (Net Zero Compare, n.d.). In particular, only third-party estimates of cost are available, not operator-confirmed figures. Consequently, the source's exact scope and cost cannot be independently verified from public information, unless confirmed directly with Climate X.</t>
+          <t>The main limitation is that pricing and the full hazard list are not published by the operator directly (Net Zero Compare, 2025). In particular, only third-party estimates of cost are available, not operator-confirmed figures. Consequently, the source's exact scope and cost cannot be independently verified from public information, unless confirmed directly with Climate X.</t>
         </is>
       </c>
     </row>
@@ -8918,7 +8960,7 @@
       </c>
       <c r="C110" s="9" t="inlineStr">
         <is>
-          <t>The main limitation is enterprise-tier, quote-based pricing not publicly listed (Mitiga Solutions, n.d.). In particular, the platform's scientific and financial-metric depth is designed for enterprise-scale deployments across banks, insurers and asset managers. Consequently, the source cannot be assumed affordable for an SNCI without direct confirmation, unless a limited-scope engagement at the lower end of the stated price range is negotiated.</t>
+          <t>The main limitation is enterprise-tier, quote-based pricing not publicly listed (Mitiga Solutions, no date). In particular, the platform's scientific and financial-metric depth is designed for enterprise-scale deployments across banks, insurers and asset managers. Consequently, the source cannot be assumed affordable for an SNCI without direct confirmation, unless a limited-scope engagement at the lower end of the stated price range is negotiated.</t>
         </is>
       </c>
     </row>
@@ -9020,7 +9062,7 @@
       </c>
       <c r="C116" s="9" t="inlineStr">
         <is>
-          <t>Not applicable: the source provides only aggregate EU bank-level statistics with no per-exposure data (EBA, n.d.), so no portfolio-level pipeline can be built against it. Integration step: no machine access; values must be looked up manually; technical effort therefore low.</t>
+          <t>Not applicable: the source provides only aggregate EU bank-level statistics with no per-exposure data (European Banking Authority, no date), so no portfolio-level pipeline can be built against it. Integration step: no machine access; values must be looked up manually; technical effort therefore low.</t>
         </is>
       </c>
     </row>
@@ -9054,7 +9096,7 @@
       </c>
       <c r="C118" s="9" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the WMS/WFS endpoint (data.gv.at, n.d.-a) or download the shapefile/GeoPackage once and perform a local spatial join, assigning the returned zone value to each exposure. The result is parcel/address-level. The process is fully automatable. Integration step: a download followed by a spatial or entity join; technical effort therefore low.</t>
+          <t>To apply the source to a portfolio, the institution must first geocode the relevant exposure addresses to coordinates. It must then query the WMS/WFS endpoint (Forsttechnischer Dienst für Wildbach- und Lawinenverbauung, no date) or download the shapefile/GeoPackage once and perform a local spatial join, assigning the returned zone value to each exposure. The result is parcel/address-level. The process is fully automatable. Integration step: a download followed by a spatial or entity join; technical effort therefore low.</t>
         </is>
       </c>
     </row>
@@ -9071,7 +9113,7 @@
       </c>
       <c r="C119" s="9" t="inlineStr">
         <is>
-          <t>To apply HORA to a portfolio, the institution would need to geocode the relevant exposure addresses and query the corresponding locations individually through the web interface (HORA, n.d.), then record and link the resulting hazard information to each exposure. Because unrestricted bulk access and a documented portfolio-level API are not available, the process is not fully automatable and is unsuitable for systematic portfolio processing under current access conditions. Integration step: no machine access; values must be looked up manually; technical effort therefore high.</t>
+          <t>To apply HORA to a portfolio, the institution would need to geocode the relevant exposure addresses and query the corresponding locations individually through the web interface (HORA, no date), then record and link the resulting hazard information to each exposure. Because unrestricted bulk access and a documented portfolio-level API are not available, the process is not fully automatable and is unsuitable for systematic portfolio processing under current access conditions. Integration step: no machine access; values must be looked up manually; technical effort therefore high.</t>
         </is>
       </c>
     </row>
@@ -9105,7 +9147,7 @@
       </c>
       <c r="C121" s="9" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the API (Moody's, n.d.-a) and receive a facility-level risk score directly. No further spatial processing is required. The process is fully automatable for institutions with API access. Integration step: a point query against the provider; technical effort therefore low.</t>
+          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the API (Moody's, no date b) and receive a facility-level risk score directly. No further spatial processing is required. The process is fully automatable for institutions with API access. Integration step: a point query against the provider; technical effort therefore low.</t>
         </is>
       </c>
     </row>
@@ -9122,7 +9164,7 @@
       </c>
       <c r="C122" s="9" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the API (Munich Re, n.d.-a) and receive a facility-level risk score directly. No further spatial processing is required. The process is fully automatable for institutions with API/subscription access. Integration step: a point query against the provider; technical effort therefore low.</t>
+          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the API (Munich Re, no date) and receive a facility-level risk score directly. No further spatial processing is required. The process is fully automatable for institutions with API/subscription access. Integration step: a point query against the provider; technical effort therefore low.</t>
         </is>
       </c>
     </row>
@@ -9156,7 +9198,7 @@
       </c>
       <c r="C124" s="9" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution can bulk-download the CSV file (Statistik Austria, n.d.) and join it directly to its internal exposure data using the Firmenbuchnummer, then transform the assigned OeNACE code to the required 4-digit reporting granularity. The result is entity-level. The process is fully automatable and does not require geocoding or spatial processing. Integration step: a download followed by a spatial or entity join; technical effort therefore low.</t>
+          <t>To apply the source to a portfolio, the institution can bulk-download the CSV file (Statistik Austria, no date) and join it directly to its internal exposure data using the Firmenbuchnummer, then transform the assigned OeNACE code to the required 4-digit reporting granularity. The result is entity-level. The process is fully automatable and does not require geocoding or spatial processing. Integration step: a download followed by a spatial or entity join; technical effort therefore low.</t>
         </is>
       </c>
     </row>
@@ -9173,7 +9215,7 @@
       </c>
       <c r="C125" s="9" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution would send the Firmenbuchnummer or company identifier to the API (Compass-Verlag, n.d.-a) and receive the OeNACE classification directly. No further processing is required. The process is fully automatable for institutions with API access. Integration step: a point query against the provider; technical effort therefore low.</t>
+          <t>To apply the source to a portfolio, the institution would send the Firmenbuchnummer or company identifier to the API (Compass-Verlag GmbH, no date b) and receive the OeNACE classification directly. No further processing is required. The process is fully automatable for institutions with API access. Integration step: a point query against the provider; technical effort therefore low.</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9266,7 @@
       </c>
       <c r="C128" s="9" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the Spectra API (Climate X, n.d.) and receive an asset-level hazard/financial-loss score directly. No further spatial processing is required. The process is fully automatable for institutions with API access. Integration step: a point query against the provider; technical effort therefore low.</t>
+          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the Spectra API (Climate X Ltd, no date a) and receive an asset-level hazard/financial-loss score directly. No further spatial processing is required. The process is fully automatable for institutions with API access. Integration step: a point query against the provider; technical effort therefore low.</t>
         </is>
       </c>
     </row>
@@ -9241,7 +9283,7 @@
       </c>
       <c r="C129" s="9" t="inlineStr">
         <is>
-          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the ClimateScore Global API (Jupiter Intelligence, n.d.) and receive an asset-level hazard/financial-loss score directly. No further spatial processing is required. The process is fully automatable for institutions with API access. Integration step: a point query against the provider; technical effort therefore low.</t>
+          <t>To apply the source to a portfolio, the institution would send exposure coordinates or addresses to the ClimateScore Global API (Jupiter Intelligence, Inc., no date a) and receive an asset-level hazard/financial-loss score directly. No further spatial processing is required. The process is fully automatable for institutions with API access. Integration step: a point query against the provider; technical effort therefore low.</t>
         </is>
       </c>
     </row>
@@ -9275,7 +9317,7 @@
       </c>
       <c r="C131" s="9" t="inlineStr">
         <is>
-          <t>Pricing is not publicly disclosed. Access is provided through a commercial analytics platform and API under a quote-based licence agreement (Moody's, n.d.-a). No product-specific price indication was identified; publicly available estimates for other Moody's products should therefore not be used as a proxy. The price information should be treated as not independently verified.</t>
+          <t>Pricing is not publicly disclosed. Access is provided through a commercial analytics platform and API under a quote-based licence agreement (Moody's, no date b). No product-specific price indication was identified; publicly available estimates for other Moody's products should therefore not be used as a proxy. The price information should be treated as not independently verified.</t>
         </is>
       </c>
     </row>
@@ -9292,7 +9334,7 @@
       </c>
       <c r="C132" s="9" t="inlineStr">
         <is>
-          <t>Pricing follows two distinct access models (Munich Re, n.d.-c). The On-Demand service uses pay-per-location pricing, with publicly displayed prices ranging from approximately EUR 100 to EUR 160 per location depending on package size. Portfolio-scale access through the Natural Hazards Edition or Climate Change Edition is subscription-based and quote-based, with API access available in the relevant business tiers. The publicly displayed On-Demand prices are not directly comparable with portfolio subscription costs.</t>
+          <t>Pricing follows two distinct access models (Munich Re, Risk Management Partners, no date a). The On-Demand service uses pay-per-location pricing, with publicly displayed prices ranging from approximately EUR 100 to EUR 160 per location depending on package size. Portfolio-scale access through the Natural Hazards Edition or Climate Change Edition is subscription-based and quote-based, with API access available in the relevant business tiers. The publicly displayed On-Demand prices are not directly comparable with portfolio subscription costs.</t>
         </is>
       </c>
     </row>
@@ -9309,7 +9351,7 @@
       </c>
       <c r="C133" s="9" t="inlineStr">
         <is>
-          <t>Pricing is publicly disclosed for standard access: pay-per-query, from EUR 6 (excl. VAT) per quarter for up to 10 queries via the WKO-member service, or from EUR 24 per year for individual/basic access (Compass-Verlag, n.d.-c; Compass-Verlag, n.d.-d). Institutional/enterprise API pricing is not publicly listed and should be confirmed directly with the provider.</t>
+          <t>Pricing is publicly disclosed for standard access: pay-per-query, from EUR 6 (excl. VAT) per quarter for up to 10 queries via the WKO-member service, or from EUR 24 per year for individual/basic access (Compass-Verlag GmbH, via Wirtschaftskammer Österreich, no date; Compass-Verlag GmbH, no date c). Institutional/enterprise API pricing is not publicly listed and should be confirmed directly with the provider.</t>
         </is>
       </c>
     </row>
@@ -9326,7 +9368,7 @@
       </c>
       <c r="C134" s="9" t="inlineStr">
         <is>
-          <t>Pricing is not publicly disclosed by Climate X directly. Access is provided through a commercial SaaS platform and API under a quote-based licence agreement. Third-party industry comparison sources estimate EUR 20,000-60,000 per year for portfolios of 30-100 assets, described as 'mid-market' pricing (Repath, n.d.). The price information should be treated as indicative and not independently verified.</t>
+          <t>Pricing is not publicly disclosed by Climate X directly. Access is provided through a commercial SaaS platform and API under a quote-based licence agreement. Third-party industry comparison sources estimate EUR 20,000-60,000 per year for portfolios of 30-100 assets, described as 'mid-market' pricing (Repath, no date). The price information should be treated as indicative and not independently verified.</t>
         </is>
       </c>
     </row>
@@ -9343,7 +9385,7 @@
       </c>
       <c r="C135" s="9" t="inlineStr">
         <is>
-          <t>Pricing is not publicly disclosed as a fixed list, but is quote-based. Jupiter's own CEO stated in a 2022 interview that 'subscription pricing ranges from $25,000 to multimillion-dollar contracts' depending on scope (Trellis/Clancy, 2022). Full portfolio deployments are typically six-figure annual commitments per third-party sources (Repath, n.d.). The price information should be treated as indicative, based on the operator's own public statement.</t>
+          <t>Pricing is not publicly disclosed as a fixed list, but is quote-based. Jupiter's own CEO stated in a 2022 interview that 'subscription pricing ranges from $25,000 to multimillion-dollar contracts' depending on scope (Clancy, 2022). Full portfolio deployments are typically six-figure annual commitments per third-party sources (Repath, no date). The price information should be treated as indicative, based on the operator's own public statement.</t>
         </is>
       </c>
     </row>
@@ -9360,7 +9402,7 @@
       </c>
       <c r="C136" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is providing ready-made, peer-reviewed hazard indices with documented methodology (EEA/C3S, n.d.) for six hazards (heat wave, heavy precipitation, flood, drought, storm, wildfire), saving the index-definition effort that raw climate variables would require. It is particularly useful as a primary source for these six hazards at moderate processing effort. However, its suitability is reduced by grid resolution coarser than Austria's parcel-level sources, and by the proxy-only nature of its heat-stress and water-stress coverage. It is therefore best used as a primary source for its six directly covered hazards, complemented by dedicated Austrian layers where finer resolution is needed.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is providing ready-made, peer-reviewed hazard indices with documented methodology (The Climate Data Factory and B-Open et al., 2024) for six hazards (heat wave, heavy precipitation, flood, drought, storm, wildfire), saving the index-definition effort that raw climate variables would require. It is particularly useful as a primary source for these six hazards at moderate processing effort. However, its suitability is reduced by grid resolution coarser than Austria's parcel-level sources, and by the proxy-only nature of its heat-stress and water-stress coverage. It is therefore best used as a primary source for its six directly covered hazards, complemented by dedicated Austrian layers where finer resolution is needed.</t>
         </is>
       </c>
     </row>
@@ -9394,7 +9436,7 @@
       </c>
       <c r="C138" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is being the only dedicated European wildfire dataset covering both forecast fire danger and observed fire history (JRC/Copernicus EMS, n.d.). It is particularly useful for national-level wildfire screening and historical plausibility checks. However, its suitability is reduced by the coarse forecast-grid resolution for a country the size of Austria and by the raw, unprocessed nature of both layers. It is therefore best used as a supplementary source for wildfire, complemented by own aggregation of the raw data.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is being the only dedicated European wildfire dataset covering both forecast fire danger and observed fire history (Joint Research Centre and Copernicus Emergency Management Service et al., no date). It is particularly useful for national-level wildfire screening and historical plausibility checks. However, its suitability is reduced by the coarse forecast-grid resolution for a country the size of Austria and by the raw, unprocessed nature of both layers. It is therefore best used as a supplementary source for wildfire, complemented by own aggregation of the raw data.</t>
         </is>
       </c>
     </row>
@@ -9411,7 +9453,7 @@
       </c>
       <c r="C139" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is being authoritative, EU-wide consistent and covering the broadest range of underlying climate variables of any source in the matrix (ECMWF, n.d.). It is particularly useful as the raw-data foundation when no ready-made indicator exists elsewhere. However, its suitability is reduced by the substantial climatological and GIS processing effort required before any variable becomes an exposure classification. It is therefore best used as a fallback source for hazards not covered by ready-made products, rather than as an operational primary source.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is being authoritative, EU-wide consistent and covering the broadest range of underlying climate variables of any source in the matrix (ECMWF, no date). It is particularly useful as the raw-data foundation when no ready-made indicator exists elsewhere. However, its suitability is reduced by the substantial climatological and GIS processing effort required before any variable becomes an exposure classification. It is therefore best used as a fallback source for hazards not covered by ready-made products, rather than as an operational primary source.</t>
         </is>
       </c>
     </row>
@@ -9428,7 +9470,7 @@
       </c>
       <c r="C140" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is not suitable for populating individual exposures. Its main advantage is providing an authoritative EU/EEA peer-comparison benchmark (EBA, n.d.). It is particularly useful for contextualising an institution's own physical and transition risk exposure against sector averages. However, its suitability is reduced by the complete absence of per-exposure or downloadable data. It is therefore best used purely as a context/benchmarking source, not as an operational data source.</t>
+          <t>For an SNCI, the source is not suitable for populating individual exposures. Its main advantage is providing an authoritative EU/EEA peer-comparison benchmark (European Banking Authority, no date). It is particularly useful for contextualising an institution's own physical and transition risk exposure against sector averages. However, its suitability is reduced by the complete absence of per-exposure or downloadable data. It is therefore best used purely as a context/benchmarking source, not as an operational data source.</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9487,7 @@
       </c>
       <c r="C141" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is combining several underlying Austrian flood sources into a single, harmonised layer with a standard OGC interface and no access restriction, unlike HORA (data.gv.at, n.d.-b). It is particularly useful as the primary operational flood layer for populating data point 0050. However, its suitability is reduced somewhat by the dataset's data currency. It is therefore best used as the primary flood-hazard source, complemented by periodic currency checks.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is combining several underlying Austrian flood sources into a single, harmonised layer with a standard OGC interface and no access restriction, unlike HORA (Umweltbundesamt, 2020). It is particularly useful as the primary operational flood layer for populating data point 0050. However, its suitability is reduced somewhat by the dataset's data currency. It is therefore best used as the primary flood-hazard source, complemented by periodic currency checks.</t>
         </is>
       </c>
     </row>
@@ -9462,7 +9504,7 @@
       </c>
       <c r="C142" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is being the strongest national source for mass-movement and torrent hazards, based on a statutory hazard assessment under the Forstgesetz (data.gv.at, n.d.-a). It is particularly useful for classifying torrent, avalanche and related mass-movement exposure at data point 0050. However, its suitability is reduced by incomplete settlement-area-only mapping and residual analogue-only zone plans. It is therefore best used as the primary source for these hazards, with unmapped locations flagged for manual review.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is being the strongest national source for mass-movement and torrent hazards, based on a statutory hazard assessment under the Forstgesetz (Forsttechnischer Dienst für Wildbach- und Lawinenverbauung, no date). It is particularly useful for classifying torrent, avalanche and related mass-movement exposure at data point 0050. However, its suitability is reduced by incomplete settlement-area-only mapping and residual analogue-only zone plans. It is therefore best used as the primary source for these hazards, with unmapped locations flagged for manual review.</t>
         </is>
       </c>
     </row>
@@ -9479,7 +9521,7 @@
       </c>
       <c r="C143" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, HORA is conditionally suitable. Its main advantage is Austrian address-level coverage combined with simple web-based access (HORA, n.d.). It is particularly useful for individual exposure checks and plausibility assessments. However, its suitability is reduced by the restricted portfolio-level access and the non-binding nature of the displayed information. It is therefore best used as a supplementary validation source rather than as the sole operational source for populating data point 0050.</t>
+          <t>For an SNCI, HORA is conditionally suitable. Its main advantage is Austrian address-level coverage combined with simple web-based access (HORA, no date). It is particularly useful for individual exposure checks and plausibility assessments. However, its suitability is reduced by the restricted portfolio-level access and the non-binding nature of the displayed information. It is therefore best used as a supplementary validation source rather than as the sole operational source for populating data point 0050.</t>
         </is>
       </c>
     </row>
@@ -9513,7 +9555,7 @@
       </c>
       <c r="C145" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is ready-made, high-granularity facility-level risk scores integrable via API with low processing effort (Moody's, n.d.-a). It is particularly useful for flood, heat stress, water stress and wildfire classification. However, its suitability is reduced by a commercial cost structure typically designed for larger institutions and by narrower-than-marketed Austria-relevant hazard coverage. It is therefore best used as a primary source only for the confirmed hazards, subject to cost negotiation appropriate to SNCI scale.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is ready-made, high-granularity facility-level risk scores integrable via API with low processing effort (Moody's, no date b). It is particularly useful for flood, heat stress, water stress and wildfire classification. However, its suitability is reduced by a commercial cost structure typically designed for larger institutions and by narrower-than-marketed Austria-relevant hazard coverage. It is therefore best used as a primary source only for the confirmed hazards, subject to cost negotiation appropriate to SNCI scale. The scores are populated for Europe at sub-national level; Moody's reports that 21 per cent of European NUTS 3 areas are highly exposed to heat stress (Moody's ESG Solutions, 2021).</t>
         </is>
       </c>
     </row>
@@ -9564,7 +9606,7 @@
       </c>
       <c r="C148" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is being simultaneously official, freely accessible in bulk and directly joinable to a loan portfolio via the Firmenbuchnummer (Statistik Austria, n.d.). It is particularly useful as the primary operational source for populating the NACE subsector dimension. However, its suitability is reduced slightly by unmatched companies and out-of-scope sole traders. It is therefore best used as the primary transition-risk classification source, complemented by Wirtschafts-Compass where an existing licence is operationally simpler.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is being simultaneously official, freely accessible in bulk and directly joinable to a loan portfolio via the Firmenbuchnummer (Statistik Austria, no date). It is particularly useful as the primary operational source for populating the NACE subsector dimension. However, its suitability is reduced slightly by unmatched companies and out-of-scope sole traders. It is therefore best used as the primary transition-risk classification source, complemented by Wirtschafts-Compass where an existing licence is operationally simpler.</t>
         </is>
       </c>
     </row>
@@ -9581,7 +9623,7 @@
       </c>
       <c r="C149" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is being directly usable, daily-updated and API-accessible, with existing institutional access reported in parts of the Austrian banking sector (Compass-Verlag, n.d.-b). It is particularly useful where an existing licence makes a single query operationally simpler than a bulk HVD join. However, its suitability is reduced by cost for institutions without an existing licence and by its non-official classification status. It is therefore best used as a primary operational source alongside the free HVD dataset.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is being directly usable, daily-updated and API-accessible, with existing institutional access reported in parts of the Austrian banking sector (Compass-Verlag GmbH, no date a). It is particularly useful where an existing licence makes a single query operationally simpler than a bulk HVD join. However, its suitability is reduced by cost for institutions without an existing licence and by its non-official classification status. It is therefore best used as a primary operational source alongside the free HVD dataset.</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9640,7 @@
       </c>
       <c r="C150" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is Austria's highest-resolution national gridded observation dataset, finer than Copernicus CDS, with a coordinate-based API enabling direct point queries (GeoSphere Austria, n.d.-a). It is particularly useful as the primary raw-data foundation for heat and heavy-precipitation indices tailored to Austrian conditions. However, its suitability is reduced by the own-methodology effort required to convert raw variables into a hazard indicator. It is therefore best used as a primary source for institutions willing to define their own threshold-based indices.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is Austria's highest-resolution national gridded observation dataset, finer than Copernicus CDS, with a coordinate-based API enabling direct point queries (GeoSphere Austria, no date a). It is particularly useful as the primary raw-data foundation for heat and heavy-precipitation indices tailored to Austrian conditions. However, its suitability is reduced by the own-methodology effort required to convert raw variables into a hazard indicator. It is therefore best used as a primary source for institutions willing to define their own threshold-based indices.</t>
         </is>
       </c>
     </row>
@@ -9632,7 +9674,7 @@
       </c>
       <c r="C152" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is ready-made, high-granularity asset-level scores integrable via API for a broad set of confirmed hazards (Repath, n.d.; Net Zero Compare, n.d.). It is particularly useful for flood, storm, heat stress, wildfire and landslide classification. However, its suitability is reduced by unconfirmed pricing and enterprise-SaaS positioning that may exceed a typical SNCI's budget. It is therefore best used as a primary source subject to direct price confirmation appropriate to SNCI scale.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is ready-made, high-granularity asset-level scores integrable via API for a broad set of confirmed hazards (Repath, no date; Net Zero Compare, 2025). It is particularly useful for flood, storm, heat stress, wildfire and landslide classification. However, its suitability is reduced by unconfirmed pricing and enterprise-SaaS positioning that may exceed a typical SNCI's budget. It is therefore best used as a primary source subject to direct price confirmation appropriate to SNCI scale.</t>
         </is>
       </c>
     </row>
@@ -9649,7 +9691,7 @@
       </c>
       <c r="C153" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is conditionally suitable. Its main advantage is extensive, scientifically validated hazard and financial-metric coverage across 9 peer-reviewed perils (aigreentools.com, n.d.). It is particularly useful for institutions needing finance-grade physical risk metrics beyond simple hazard scores. However, its suitability is reduced by enterprise-tier pricing likely above a typical SNCI's budget for full portfolio deployment. It is therefore best used as a primary source for a limited scope, subject to direct price negotiation.</t>
+          <t>For an SNCI, the source is conditionally suitable. Its main advantage is extensive, scientifically validated hazard and financial-metric coverage across 9 peer-reviewed perils (aigreentools.com, no date). It is particularly useful for institutions needing finance-grade physical risk metrics beyond simple hazard scores. However, its suitability is reduced by enterprise-tier pricing likely above a typical SNCI's budget for full portfolio deployment. It is therefore best used as a primary source for a limited scope, subject to direct price negotiation.</t>
         </is>
       </c>
     </row>
@@ -9666,7 +9708,7 @@
       </c>
       <c r="C154" s="9" t="inlineStr">
         <is>
-          <t>For an SNCI, the source is suitable. Its main advantage is that each product is a purpose-built, documented hazard indicator with no own index-definition effort required, unlike raw Copernicus CDS variables (Di Napoli et al., 2021; SMHI/C3S, n.d.). It is particularly useful for heat stress, flood, water stress and soil-moisture drought classification at low processing effort. However, its suitability is reduced by its narrower hazard breadth compared with the full CDS catalogue. It is therefore best used as a primary source for its four covered hazards, complemented by other sources for the remainder.</t>
+          <t>For an SNCI, the source is suitable. Its main advantage is that each product is a purpose-built, documented hazard indicator with no own index-definition effort required, unlike raw Copernicus CDS variables (Di Napoli et al., 2021; Copernicus Climate Change Service, Climate Data Store, 2021). It is particularly useful for heat stress, flood, water stress and soil-moisture drought classification at low processing effort. However, its suitability is reduced by its narrower hazard breadth compared with the full CDS catalogue. It is therefore best used as a primary source for its four covered hazards, complemented by other sources for the remainder.</t>
         </is>
       </c>
     </row>
@@ -10166,11 +10208,6 @@
           <t>data_point</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Relevance</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>